<commit_message>
feat: re-run full 100K pipeline with improved YoE and title scoring
</commit_message>
<xml_diff>
--- a/outputs/mohd_ibadullah.xlsx
+++ b/outputs/mohd_ibadullah.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.9057</t>
+          <t>0.907</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.8973</t>
+          <t>0.8983</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.8624</t>
+          <t>0.8626</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -535,7 +535,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0093547</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -545,19 +545,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.8573</t>
+          <t>0.8543</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Exceptional Senior Machine Learning Engineer offering 2.9 years of experience, offers solid expertise in RAG, Python, PyTorch which matches the core ranking mandate. Highly active on Redrob with a 75% recruiter response rate.</t>
+          <t>Highly relevant Senior AI Engineer with 5.9 years of background, offers solid expertise in FAISS, TensorFlow, NLP which matches the core ranking mandate. Excellent platform engagement with 80% response rate.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0007411</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -567,19 +567,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.8515</t>
+          <t>0.8489</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Highly relevant Senior AI Engineer with 5.9 years of background, offers solid expertise in FAISS, TensorFlow, NLP which matches the core ranking mandate. Excellent platform engagement with 80% response rate.</t>
+          <t>Top-tier candidate currently working as Senior Machine Learning Engineer (8.0 YoE), offers solid expertise in Vector Search, PyTorch, Information Retrieval which matches the core ranking mandate. Excellent platform engagement with 12% response rate.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0007411</t>
+          <t>CAND_0093547</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.8473</t>
+          <t>0.8309</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Top-tier candidate currently working as Senior Machine Learning Engineer (8.0 YoE), offers solid expertise in Vector Search, PyTorch, Information Retrieval which matches the core ranking mandate. Excellent platform engagement with 12% response rate.</t>
+          <t>Exceptional Senior Machine Learning Engineer offering 2.9 years of experience, offers solid expertise in RAG, Python, PyTorch which matches the core ranking mandate. Highly active on Redrob with a 75% recruiter response rate.</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.8238</t>
+          <t>0.8276</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.8135</t>
+          <t>0.8139</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.8053</t>
+          <t>0.8073</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.7947</t>
+          <t>0.7977</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.7934</t>
+          <t>0.7968</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.788</t>
+          <t>0.7909</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.7834</t>
+          <t>0.7871</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.7806</t>
+          <t>0.7817</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.7752</t>
+          <t>0.7794</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.7674</t>
+          <t>0.7698</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.7643</t>
+          <t>0.7665</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.7604</t>
+          <t>0.7662</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.7568</t>
+          <t>0.7605</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.7512</t>
+          <t>0.7556</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -909,7 +909,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -919,19 +919,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.7481</t>
+          <t>0.749</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 4.9 years in the field, matching key job requirements like Vector Search, Embeddings, Python, slightly below the preferred 5+ years of experience.</t>
+          <t>Well-qualified Senior AI Engineer showing 7.9 YoE, who brings relevant experience in NLP, Python, Ranking Systems. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0037944</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -941,12 +941,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.745</t>
+          <t>0.7444</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Well-qualified Senior AI Engineer showing 7.9 YoE, who brings relevant experience in NLP, Python, Ranking Systems. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Data Scientist with 4.9 years in the field, matching key job requirements like Vector Search, Embeddings, Python, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
@@ -963,7 +963,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.732</t>
+          <t>0.735</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.7165</t>
+          <t>0.7251</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.7162</t>
+          <t>0.7246</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.6878</t>
+          <t>0.6957</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.6867</t>
+          <t>0.6923</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1063,7 +1063,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0061339</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1073,19 +1073,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.6862</t>
+          <t>0.6901</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Strong Search Engineer with 4.2 years of experience, matching key job requirements like Information Retrieval, Milvus, TensorFlow, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Machine Learning Engineer with 7.2 years in the field, matching key job requirements like RAG, FAISS, Embeddings, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0064904</t>
+          <t>CAND_0061339</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1095,19 +1095,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.6842</t>
+          <t>0.689</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Strong AI Engineer with 4.9 years of experience, who brings relevant experience in Embeddings, Python, MLOps, note the longer notice period of 90 days.</t>
+          <t>Strong Search Engineer with 4.2 years of experience, matching key job requirements like Information Retrieval, Milvus, TensorFlow, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0064904</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1117,12 +1117,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.6803</t>
+          <t>0.6831</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Solid candidate working as Machine Learning Engineer with 7.2 years in the field, matching key job requirements like RAG, FAISS, Embeddings, note the longer notice period of 120 days.</t>
+          <t>Strong AI Engineer with 4.9 years of experience, who brings relevant experience in Embeddings, Python, MLOps, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.6701</t>
+          <t>0.6792</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.6661</t>
+          <t>0.676</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1173,7 +1173,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0042506</t>
+          <t>CAND_0083307</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1183,19 +1183,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.6639</t>
+          <t>0.6712</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 4.2 years in the field, with matching skills in TensorFlow, Information Retrieval, Milvus and solid backend fundamentals, slightly below the preferred 5+ years of experience.</t>
+          <t>Solid candidate working as Search Engineer with 7.8 years in the field, matching key job requirements like Embeddings, Pinecone, Python, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0083307</t>
+          <t>CAND_0042506</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.6627</t>
+          <t>0.6703</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 7.8 years in the field, matching key job requirements like Embeddings, Pinecone, Python, note the longer notice period of 120 days.</t>
+          <t>Solid candidate working as Search Engineer with 4.2 years in the field, with matching skills in TensorFlow, Information Retrieval, Milvus and solid backend fundamentals, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0084681</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1227,19 +1227,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.6603</t>
+          <t>0.6671</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Specialist with 3.5 years in the field, matching key job requirements like Python, Information Retrieval, Vector Search, slightly below the preferred 5+ years of experience.</t>
+          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0051615</t>
+          <t>CAND_0065878</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.6584</t>
+          <t>0.6659</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (4.6 YoE), matching key job requirements like RAG, Milvus, Vector Search, slightly below the preferred 5+ years of experience.</t>
+          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0065878</t>
+          <t>CAND_0051615</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1271,19 +1271,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.6583</t>
+          <t>0.6606</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
+          <t>Competent Search Engineer (4.6 YoE), matching key job requirements like RAG, Milvus, Vector Search, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0084681</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.6576</t>
+          <t>0.6548</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
+          <t>Solid candidate working as AI Specialist with 3.5 years in the field, matching key job requirements like Python, Information Retrieval, Vector Search, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.6432</t>
+          <t>0.6526</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.6413</t>
+          <t>0.649</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.6376</t>
+          <t>0.6462</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1371,7 +1371,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0039838</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1381,19 +1381,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.6366</t>
+          <t>0.6419</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Strong Recommendation Systems Engineer with 4.9 years of experience, with matching skills in MLOps, Embeddings, RAG and solid backend fundamentals, note the longer notice period of 90 days.</t>
+          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0039838</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1403,19 +1403,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.634</t>
+          <t>0.6376</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Strong Recommendation Systems Engineer with 4.9 years of experience, with matching skills in MLOps, Embeddings, RAG and solid backend fundamentals, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0076904</t>
+          <t>CAND_0012632</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1425,19 +1425,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.6303</t>
+          <t>0.6369</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 4.2 YoE, possessing practical experience in Vector Search, NLP, MLOps, note the longer notice period of 90 days.</t>
+          <t>Competent AI Specialist (6.0 YoE), possessing practical experience in MLOps, Python, Pinecone, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0012632</t>
+          <t>CAND_0076904</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1447,19 +1447,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.628</t>
+          <t>0.6363</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Competent AI Specialist (6.0 YoE), possessing practical experience in MLOps, Python, Pinecone, note the longer notice period of 120 days.</t>
+          <t>Well-qualified Senior Data Scientist showing 4.2 YoE, possessing practical experience in Vector Search, NLP, MLOps, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0054123</t>
+          <t>CAND_0077285</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.6242</t>
+          <t>0.6331</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Solid candidate working as Applied ML Engineer with 4.7 years in the field, matching key job requirements like Python, Vector Search, slightly below the preferred 5+ years of experience.</t>
+          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0077285</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1491,19 +1491,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.6208</t>
+          <t>0.6284</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
+          <t>Competent Search Engineer (7.2 YoE), matching key job requirements like Embeddings, Information Retrieval, PyTorch, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0072721</t>
+          <t>CAND_0008239</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.6195</t>
+          <t>0.6257</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Strong Data Scientist with 3.7 years of experience, who brings relevant experience in MLOps, Python, Embeddings, slightly below the preferred 5+ years of experience.</t>
+          <t>Strong AI Engineer with 4.0 years of experience, matching key job requirements like Milvus, Vector Search, Python, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0054123</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1535,19 +1535,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.6186</t>
+          <t>0.6248</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (7.2 YoE), matching key job requirements like Embeddings, Information Retrieval, PyTorch, note the longer notice period of 120 days.</t>
+          <t>Solid candidate working as Applied ML Engineer with 4.7 years in the field, matching key job requirements like Python, Vector Search, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0008239</t>
+          <t>CAND_0030468</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1557,19 +1557,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.6179</t>
+          <t>0.624</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Engineer (4.0 YoE), mostly showing adjacent skills like Milvus, Vector Search, Python; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 5.4 YoE as Senior Applied Scientist, mostly showing adjacent skills like TensorFlow, Ranking Systems, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0030468</t>
+          <t>CAND_0064326</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1579,19 +1579,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.6149</t>
+          <t>0.6231</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.4 YoE as Senior Applied Scientist, mostly showing adjacent skills like TensorFlow, Ranking Systems, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 7.6 YoE as Search Engineer, mostly showing adjacent skills like PyTorch, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0064326</t>
+          <t>CAND_0036184</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1601,12 +1601,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.6144</t>
+          <t>0.6211</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.6 YoE as Search Engineer, mostly showing adjacent skills like PyTorch, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Recommendation Systems Engineer (6.0 YoE), mostly showing adjacent skills like FAISS, MLOps, Embeddings; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.6138</t>
+          <t>0.6207</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1635,7 +1635,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0061175</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1645,19 +1645,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.6132</t>
+          <t>0.6203</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Candidate with 4.5 years experience as Machine Learning Engineer, mostly showing adjacent skills like MLOps, PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 6.7 YoE as AI Research Engineer, possessing partial overlap in Python, Milvus, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0036184</t>
+          <t>CAND_0099401</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1667,19 +1667,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.6104</t>
+          <t>0.6183</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Recommendation Systems Engineer (6.0 YoE), mostly showing adjacent skills like FAISS, MLOps, Embeddings; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0099401</t>
+          <t>CAND_0030348</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1689,12 +1689,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.6096</t>
+          <t>0.6178</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 4.5 years experience as Machine Learning Engineer, mostly showing adjacent skills like MLOps, PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.607</t>
+          <t>0.6167</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.6041</t>
+          <t>0.6155</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1745,7 +1745,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0072721</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1755,19 +1755,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.6036</t>
+          <t>0.6155</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Data Scientist (3.7 YoE), having some background in MLOps, Python, Embeddings but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0081686</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1777,19 +1777,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.6029</t>
+          <t>0.6144</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Candidate with 6.0 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, FAISS, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0006557</t>
+          <t>CAND_0081686</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1799,19 +1799,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.6009</t>
+          <t>0.6127</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.0 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, FAISS, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0051630</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1821,19 +1821,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.6002</t>
+          <t>0.6109</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Alternative profile showing 8.8 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like MLOps, Python, Milvus; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0032270</t>
+          <t>CAND_0006557</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1843,19 +1843,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.6001</t>
+          <t>0.6105</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Candidate with 4.4 years experience as Data Scientist, with limited direct exposure to search/ranking but lists Information Retrieval, Python, Embeddings; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1865,19 +1865,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.6001</t>
+          <t>0.6101</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.9 YoE as Senior Machine Learning Engineer, possessing partial overlap in Ranking Systems, TensorFlow; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 8.8 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like MLOps, Python, Milvus; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0051630</t>
+          <t>CAND_0052682</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1887,19 +1887,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.5995</t>
+          <t>0.6097</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as NLP Engineer (6.6 YoE), having some background in FAISS, PyTorch, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0052682</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.5978</t>
+          <t>0.6094</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (6.6 YoE), having some background in FAISS, PyTorch, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 7.9 YoE as Senior Machine Learning Engineer, possessing partial overlap in Ranking Systems, TensorFlow; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1931,12 +1931,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.5961</t>
+          <t>0.6071</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.7 YoE as Senior Data Scientist, mostly showing adjacent skills like Embeddings, PyTorch, MLOps; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.5957</t>
+          <t>0.6063</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -1965,7 +1965,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0029367</t>
+          <t>CAND_0032270</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1975,19 +1975,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.5949</t>
+          <t>0.6059</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
+          <t>Candidate with 4.4 years experience as Data Scientist, with limited direct exposure to search/ranking but lists Information Retrieval, Python, Embeddings; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1997,19 +1997,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.5931</t>
+          <t>0.6048</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2019,19 +2019,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.5928</t>
+          <t>0.6031</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2041,12 +2041,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.5916</t>
+          <t>0.6028</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.591</t>
+          <t>0.6001</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2075,7 +2075,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0098454</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2085,19 +2085,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.5902</t>
+          <t>0.5996</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, mostly showing adjacent skills like Milvus, TensorFlow, Python; included as potential pipeline filler.</t>
+          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0098454</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.5899</t>
+          <t>0.5994</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 4.7 YoE as Senior Data Scientist, mostly showing adjacent skills like Embeddings, PyTorch, MLOps; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.5865</t>
+          <t>0.5993</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, mostly showing adjacent skills like Milvus, TensorFlow, Python; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0089947</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2151,19 +2151,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.5861</t>
+          <t>0.5986</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 5.4 years of background, with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0089947</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2173,19 +2173,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.5821</t>
+          <t>0.5954</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.9 YoE as AI Engineer, mostly showing adjacent skills like Python, Vector Search; included as potential pipeline filler.</t>
+          <t>Junior ML Engineer with 5.4 years of background, with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0075439</t>
+          <t>CAND_0059240</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2195,12 +2195,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.5818</t>
+          <t>0.5928</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Machine Learning Engineer (4.3 YoE), with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 4.0 YoE as Junior ML Engineer, possessing partial overlap in Milvus, NLP, Information Retrieval; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.5818</t>
+          <t>0.5915</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2229,7 +2229,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2239,19 +2239,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.579</t>
+          <t>0.5915</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.9 YoE as AI Engineer, mostly showing adjacent skills like Python, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0002344</t>
+          <t>CAND_0001930</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2261,19 +2261,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.5785</t>
+          <t>0.5887</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Candidate with 4.7 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, TensorFlow, Pinecone; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0003977</t>
+          <t>CAND_0075439</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2283,19 +2283,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.5784</t>
+          <t>0.5873</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 4.6 years of background, with limited direct exposure to search/ranking but lists NLP, Embeddings, PyTorch; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Machine Learning Engineer (4.3 YoE), with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0020049</t>
+          <t>CAND_0087006</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2305,12 +2305,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.5773</t>
+          <t>0.5866</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Alternative profile showing 3.8 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, TensorFlow, MLOps; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.5765</t>
+          <t>0.5859</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2339,7 +2339,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0087006</t>
+          <t>CAND_0007391</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.5763</t>
+          <t>0.5838</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 4.3 YoE as Data Scientist, possessing partial overlap in Python, Information Retrieval, TensorFlow; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0007391</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2371,19 +2371,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.5753</t>
+          <t>0.5826</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.3 YoE as Data Scientist, possessing partial overlap in Python, Information Retrieval, TensorFlow; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 7.3 YoE as AI Engineer, mostly showing adjacent skills like Pinecone, Vector Search, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0077504</t>
+          <t>CAND_0003977</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2393,19 +2393,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.5752</t>
+          <t>0.5821</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Data Scientist (4.6 YoE), having some background in Python, MLOps, Vector Search but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Recommendation Systems Engineer with 4.6 years of background, with limited direct exposure to search/ranking but lists NLP, Embeddings, PyTorch; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0011125</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2415,19 +2415,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.5716</t>
+          <t>0.5821</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.3 YoE as AI Engineer, mostly showing adjacent skills like Pinecone, Vector Search, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.6 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, Embeddings, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0011125</t>
+          <t>CAND_0002344</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2437,19 +2437,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.5712</t>
+          <t>0.5812</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, Embeddings, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 4.7 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, TensorFlow, Pinecone; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0089012</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2459,19 +2459,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.5712</t>
+          <t>0.5812</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.2 YoE as AI Specialist, possessing partial overlap in Python, NLP, MLOps; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0007460</t>
+          <t>CAND_0077504</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2481,19 +2481,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.57</t>
+          <t>0.5804</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.7 YoE as AI Engineer, possessing partial overlap in Embeddings, Information Retrieval, RAG; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as Data Scientist (4.6 YoE), having some background in Python, MLOps, Vector Search but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2503,12 +2503,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.5698</t>
+          <t>0.5792</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
@@ -2525,7 +2525,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.5692</t>
+          <t>0.5791</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0033749</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2547,19 +2547,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.5677</t>
+          <t>0.5777</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Computer Vision Engineer with 4.7 years of background, with limited direct exposure to search/ranking but lists Vector Search, MLOps, Python; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0010685</t>
+          <t>CAND_0089012</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.5673</t>
+          <t>0.5775</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.7 YoE as NLP Engineer, possessing partial overlap in PyTorch, Information Retrieval, RAG; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 4.2 YoE as AI Specialist, possessing partial overlap in Python, NLP, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0010685</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2591,12 +2591,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.5669</t>
+          <t>0.5774</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.7 YoE as NLP Engineer, possessing partial overlap in PyTorch, Information Retrieval, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
@@ -2613,7 +2613,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.566</t>
+          <t>0.5768</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.5653</t>
+          <t>0.5755</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">

</xml_diff>

<commit_message>
re-ran full pipeline with improved scoring
</commit_message>
<xml_diff>
--- a/outputs/mohd_ibadullah.xlsx
+++ b/outputs/mohd_ibadullah.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.9057</t>
+          <t>0.907</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.8973</t>
+          <t>0.8983</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.8624</t>
+          <t>0.8626</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -535,7 +535,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0093547</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -545,19 +545,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.8573</t>
+          <t>0.8543</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Exceptional Senior Machine Learning Engineer offering 2.9 years of experience, offers solid expertise in RAG, Python, PyTorch which matches the core ranking mandate. Highly active on Redrob with a 75% recruiter response rate.</t>
+          <t>Highly relevant Senior AI Engineer with 5.9 years of background, offers solid expertise in FAISS, TensorFlow, NLP which matches the core ranking mandate. Excellent platform engagement with 80% response rate.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0007411</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -567,19 +567,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.8515</t>
+          <t>0.8489</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Highly relevant Senior AI Engineer with 5.9 years of background, offers solid expertise in FAISS, TensorFlow, NLP which matches the core ranking mandate. Excellent platform engagement with 80% response rate.</t>
+          <t>Top-tier candidate currently working as Senior Machine Learning Engineer (8.0 YoE), offers solid expertise in Vector Search, PyTorch, Information Retrieval which matches the core ranking mandate. Excellent platform engagement with 12% response rate.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0007411</t>
+          <t>CAND_0093547</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.8473</t>
+          <t>0.8309</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Top-tier candidate currently working as Senior Machine Learning Engineer (8.0 YoE), offers solid expertise in Vector Search, PyTorch, Information Retrieval which matches the core ranking mandate. Excellent platform engagement with 12% response rate.</t>
+          <t>Exceptional Senior Machine Learning Engineer offering 2.9 years of experience, offers solid expertise in RAG, Python, PyTorch which matches the core ranking mandate. Highly active on Redrob with a 75% recruiter response rate.</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.8238</t>
+          <t>0.8276</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.8135</t>
+          <t>0.8139</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.8053</t>
+          <t>0.8073</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.7947</t>
+          <t>0.7977</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.7934</t>
+          <t>0.7968</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.788</t>
+          <t>0.7909</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.7834</t>
+          <t>0.7871</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.7806</t>
+          <t>0.7817</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.7752</t>
+          <t>0.7794</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.7674</t>
+          <t>0.7698</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.7643</t>
+          <t>0.7665</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.7604</t>
+          <t>0.7662</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.7568</t>
+          <t>0.7605</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.7512</t>
+          <t>0.7556</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -909,7 +909,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -919,19 +919,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.7481</t>
+          <t>0.749</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 4.9 years in the field, matching key job requirements like Vector Search, Embeddings, Python, slightly below the preferred 5+ years of experience.</t>
+          <t>Well-qualified Senior AI Engineer showing 7.9 YoE, who brings relevant experience in NLP, Python, Ranking Systems. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0037944</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -941,12 +941,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.745</t>
+          <t>0.7444</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Well-qualified Senior AI Engineer showing 7.9 YoE, who brings relevant experience in NLP, Python, Ranking Systems. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Data Scientist with 4.9 years in the field, matching key job requirements like Vector Search, Embeddings, Python, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
@@ -963,7 +963,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.732</t>
+          <t>0.735</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.7165</t>
+          <t>0.7251</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.7162</t>
+          <t>0.7246</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.6878</t>
+          <t>0.6957</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.6867</t>
+          <t>0.6923</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1063,7 +1063,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0061339</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1073,19 +1073,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.6862</t>
+          <t>0.6901</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Strong Search Engineer with 4.2 years of experience, matching key job requirements like Information Retrieval, Milvus, TensorFlow, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Machine Learning Engineer with 7.2 years in the field, matching key job requirements like RAG, FAISS, Embeddings, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0064904</t>
+          <t>CAND_0061339</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1095,19 +1095,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.6842</t>
+          <t>0.689</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Strong AI Engineer with 4.9 years of experience, who brings relevant experience in Embeddings, Python, MLOps, note the longer notice period of 90 days.</t>
+          <t>Strong Search Engineer with 4.2 years of experience, matching key job requirements like Information Retrieval, Milvus, TensorFlow, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0064904</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1117,12 +1117,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.6803</t>
+          <t>0.6831</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Solid candidate working as Machine Learning Engineer with 7.2 years in the field, matching key job requirements like RAG, FAISS, Embeddings, note the longer notice period of 120 days.</t>
+          <t>Strong AI Engineer with 4.9 years of experience, who brings relevant experience in Embeddings, Python, MLOps, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.6701</t>
+          <t>0.6792</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.6661</t>
+          <t>0.676</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1173,7 +1173,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0042506</t>
+          <t>CAND_0083307</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1183,19 +1183,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.6639</t>
+          <t>0.6712</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 4.2 years in the field, with matching skills in TensorFlow, Information Retrieval, Milvus and solid backend fundamentals, slightly below the preferred 5+ years of experience.</t>
+          <t>Solid candidate working as Search Engineer with 7.8 years in the field, matching key job requirements like Embeddings, Pinecone, Python, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0083307</t>
+          <t>CAND_0042506</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.6627</t>
+          <t>0.6703</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 7.8 years in the field, matching key job requirements like Embeddings, Pinecone, Python, note the longer notice period of 120 days.</t>
+          <t>Solid candidate working as Search Engineer with 4.2 years in the field, with matching skills in TensorFlow, Information Retrieval, Milvus and solid backend fundamentals, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0084681</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1227,19 +1227,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.6603</t>
+          <t>0.6671</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Specialist with 3.5 years in the field, matching key job requirements like Python, Information Retrieval, Vector Search, slightly below the preferred 5+ years of experience.</t>
+          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0051615</t>
+          <t>CAND_0065878</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.6584</t>
+          <t>0.6659</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (4.6 YoE), matching key job requirements like RAG, Milvus, Vector Search, slightly below the preferred 5+ years of experience.</t>
+          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0065878</t>
+          <t>CAND_0051615</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1271,19 +1271,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.6583</t>
+          <t>0.6606</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
+          <t>Competent Search Engineer (4.6 YoE), matching key job requirements like RAG, Milvus, Vector Search, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0084681</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.6576</t>
+          <t>0.6548</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
+          <t>Solid candidate working as AI Specialist with 3.5 years in the field, matching key job requirements like Python, Information Retrieval, Vector Search, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.6432</t>
+          <t>0.6526</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.6413</t>
+          <t>0.649</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.6376</t>
+          <t>0.6462</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1371,7 +1371,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0039838</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1381,19 +1381,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.6366</t>
+          <t>0.6419</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Strong Recommendation Systems Engineer with 4.9 years of experience, with matching skills in MLOps, Embeddings, RAG and solid backend fundamentals, note the longer notice period of 90 days.</t>
+          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0039838</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1403,19 +1403,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.634</t>
+          <t>0.6376</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Strong Recommendation Systems Engineer with 4.9 years of experience, with matching skills in MLOps, Embeddings, RAG and solid backend fundamentals, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0076904</t>
+          <t>CAND_0012632</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1425,19 +1425,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.6303</t>
+          <t>0.6369</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 4.2 YoE, possessing practical experience in Vector Search, NLP, MLOps, note the longer notice period of 90 days.</t>
+          <t>Competent AI Specialist (6.0 YoE), possessing practical experience in MLOps, Python, Pinecone, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0012632</t>
+          <t>CAND_0076904</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1447,19 +1447,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.628</t>
+          <t>0.6363</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Competent AI Specialist (6.0 YoE), possessing practical experience in MLOps, Python, Pinecone, note the longer notice period of 120 days.</t>
+          <t>Well-qualified Senior Data Scientist showing 4.2 YoE, possessing practical experience in Vector Search, NLP, MLOps, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0054123</t>
+          <t>CAND_0077285</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.6242</t>
+          <t>0.6331</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Solid candidate working as Applied ML Engineer with 4.7 years in the field, matching key job requirements like Python, Vector Search, slightly below the preferred 5+ years of experience.</t>
+          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0077285</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1491,19 +1491,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.6208</t>
+          <t>0.6284</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
+          <t>Competent Search Engineer (7.2 YoE), matching key job requirements like Embeddings, Information Retrieval, PyTorch, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0072721</t>
+          <t>CAND_0008239</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.6195</t>
+          <t>0.6257</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Strong Data Scientist with 3.7 years of experience, who brings relevant experience in MLOps, Python, Embeddings, slightly below the preferred 5+ years of experience.</t>
+          <t>Strong AI Engineer with 4.0 years of experience, matching key job requirements like Milvus, Vector Search, Python, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0054123</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1535,19 +1535,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.6186</t>
+          <t>0.6248</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (7.2 YoE), matching key job requirements like Embeddings, Information Retrieval, PyTorch, note the longer notice period of 120 days.</t>
+          <t>Solid candidate working as Applied ML Engineer with 4.7 years in the field, matching key job requirements like Python, Vector Search, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0008239</t>
+          <t>CAND_0030468</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1557,19 +1557,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.6179</t>
+          <t>0.624</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Engineer (4.0 YoE), mostly showing adjacent skills like Milvus, Vector Search, Python; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 5.4 YoE as Senior Applied Scientist, mostly showing adjacent skills like TensorFlow, Ranking Systems, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0030468</t>
+          <t>CAND_0064326</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1579,19 +1579,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.6149</t>
+          <t>0.6231</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.4 YoE as Senior Applied Scientist, mostly showing adjacent skills like TensorFlow, Ranking Systems, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 7.6 YoE as Search Engineer, mostly showing adjacent skills like PyTorch, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0064326</t>
+          <t>CAND_0036184</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1601,12 +1601,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.6144</t>
+          <t>0.6211</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.6 YoE as Search Engineer, mostly showing adjacent skills like PyTorch, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Recommendation Systems Engineer (6.0 YoE), mostly showing adjacent skills like FAISS, MLOps, Embeddings; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.6138</t>
+          <t>0.6207</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1635,7 +1635,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0061175</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1645,19 +1645,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.6132</t>
+          <t>0.6203</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Candidate with 4.5 years experience as Machine Learning Engineer, mostly showing adjacent skills like MLOps, PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 6.7 YoE as AI Research Engineer, possessing partial overlap in Python, Milvus, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0036184</t>
+          <t>CAND_0099401</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1667,19 +1667,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.6104</t>
+          <t>0.6183</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Recommendation Systems Engineer (6.0 YoE), mostly showing adjacent skills like FAISS, MLOps, Embeddings; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0099401</t>
+          <t>CAND_0030348</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1689,12 +1689,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.6096</t>
+          <t>0.6178</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 4.5 years experience as Machine Learning Engineer, mostly showing adjacent skills like MLOps, PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.607</t>
+          <t>0.6167</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.6041</t>
+          <t>0.6155</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1745,7 +1745,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0072721</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1755,19 +1755,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.6036</t>
+          <t>0.6155</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Data Scientist (3.7 YoE), having some background in MLOps, Python, Embeddings but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0081686</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1777,19 +1777,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.6029</t>
+          <t>0.6144</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Candidate with 6.0 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, FAISS, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0006557</t>
+          <t>CAND_0081686</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1799,19 +1799,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.6009</t>
+          <t>0.6127</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.0 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, FAISS, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0051630</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1821,19 +1821,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.6002</t>
+          <t>0.6109</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Alternative profile showing 8.8 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like MLOps, Python, Milvus; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0032270</t>
+          <t>CAND_0006557</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1843,19 +1843,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.6001</t>
+          <t>0.6105</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Candidate with 4.4 years experience as Data Scientist, with limited direct exposure to search/ranking but lists Information Retrieval, Python, Embeddings; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1865,19 +1865,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.6001</t>
+          <t>0.6101</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.9 YoE as Senior Machine Learning Engineer, possessing partial overlap in Ranking Systems, TensorFlow; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 8.8 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like MLOps, Python, Milvus; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0051630</t>
+          <t>CAND_0052682</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1887,19 +1887,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.5995</t>
+          <t>0.6097</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as NLP Engineer (6.6 YoE), having some background in FAISS, PyTorch, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0052682</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.5978</t>
+          <t>0.6094</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (6.6 YoE), having some background in FAISS, PyTorch, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 7.9 YoE as Senior Machine Learning Engineer, possessing partial overlap in Ranking Systems, TensorFlow; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1931,12 +1931,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.5961</t>
+          <t>0.6071</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.7 YoE as Senior Data Scientist, mostly showing adjacent skills like Embeddings, PyTorch, MLOps; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.5957</t>
+          <t>0.6063</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -1965,7 +1965,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0029367</t>
+          <t>CAND_0032270</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1975,19 +1975,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.5949</t>
+          <t>0.6059</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
+          <t>Candidate with 4.4 years experience as Data Scientist, with limited direct exposure to search/ranking but lists Information Retrieval, Python, Embeddings; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1997,19 +1997,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.5931</t>
+          <t>0.6048</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2019,19 +2019,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.5928</t>
+          <t>0.6031</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2041,12 +2041,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.5916</t>
+          <t>0.6028</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.591</t>
+          <t>0.6001</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2075,7 +2075,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0098454</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2085,19 +2085,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.5902</t>
+          <t>0.5996</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, mostly showing adjacent skills like Milvus, TensorFlow, Python; included as potential pipeline filler.</t>
+          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0098454</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.5899</t>
+          <t>0.5994</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 4.7 YoE as Senior Data Scientist, mostly showing adjacent skills like Embeddings, PyTorch, MLOps; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.5865</t>
+          <t>0.5993</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, mostly showing adjacent skills like Milvus, TensorFlow, Python; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0089947</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2151,19 +2151,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.5861</t>
+          <t>0.5986</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 5.4 years of background, with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0089947</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2173,19 +2173,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.5821</t>
+          <t>0.5954</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.9 YoE as AI Engineer, mostly showing adjacent skills like Python, Vector Search; included as potential pipeline filler.</t>
+          <t>Junior ML Engineer with 5.4 years of background, with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0075439</t>
+          <t>CAND_0059240</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2195,12 +2195,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.5818</t>
+          <t>0.5928</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Machine Learning Engineer (4.3 YoE), with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 4.0 YoE as Junior ML Engineer, possessing partial overlap in Milvus, NLP, Information Retrieval; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.5818</t>
+          <t>0.5915</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2229,7 +2229,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2239,19 +2239,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.579</t>
+          <t>0.5915</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.9 YoE as AI Engineer, mostly showing adjacent skills like Python, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0002344</t>
+          <t>CAND_0001930</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2261,19 +2261,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.5785</t>
+          <t>0.5887</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Candidate with 4.7 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, TensorFlow, Pinecone; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0003977</t>
+          <t>CAND_0075439</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2283,19 +2283,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.5784</t>
+          <t>0.5873</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 4.6 years of background, with limited direct exposure to search/ranking but lists NLP, Embeddings, PyTorch; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Machine Learning Engineer (4.3 YoE), with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0020049</t>
+          <t>CAND_0087006</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2305,12 +2305,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.5773</t>
+          <t>0.5866</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Alternative profile showing 3.8 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, TensorFlow, MLOps; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.5765</t>
+          <t>0.5859</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2339,7 +2339,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0087006</t>
+          <t>CAND_0007391</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.5763</t>
+          <t>0.5838</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 4.3 YoE as Data Scientist, possessing partial overlap in Python, Information Retrieval, TensorFlow; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0007391</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2371,19 +2371,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.5753</t>
+          <t>0.5826</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.3 YoE as Data Scientist, possessing partial overlap in Python, Information Retrieval, TensorFlow; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 7.3 YoE as AI Engineer, mostly showing adjacent skills like Pinecone, Vector Search, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0077504</t>
+          <t>CAND_0003977</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2393,19 +2393,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.5752</t>
+          <t>0.5821</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Data Scientist (4.6 YoE), having some background in Python, MLOps, Vector Search but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Recommendation Systems Engineer with 4.6 years of background, with limited direct exposure to search/ranking but lists NLP, Embeddings, PyTorch; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0011125</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2415,19 +2415,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.5716</t>
+          <t>0.5821</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.3 YoE as AI Engineer, mostly showing adjacent skills like Pinecone, Vector Search, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.6 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, Embeddings, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0011125</t>
+          <t>CAND_0002344</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2437,19 +2437,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.5712</t>
+          <t>0.5812</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, Embeddings, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 4.7 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, TensorFlow, Pinecone; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0089012</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2459,19 +2459,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.5712</t>
+          <t>0.5812</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.2 YoE as AI Specialist, possessing partial overlap in Python, NLP, MLOps; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0007460</t>
+          <t>CAND_0077504</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2481,19 +2481,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.57</t>
+          <t>0.5804</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.7 YoE as AI Engineer, possessing partial overlap in Embeddings, Information Retrieval, RAG; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as Data Scientist (4.6 YoE), having some background in Python, MLOps, Vector Search but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2503,12 +2503,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.5698</t>
+          <t>0.5792</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
@@ -2525,7 +2525,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.5692</t>
+          <t>0.5791</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0033749</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2547,19 +2547,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.5677</t>
+          <t>0.5777</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Computer Vision Engineer with 4.7 years of background, with limited direct exposure to search/ranking but lists Vector Search, MLOps, Python; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0010685</t>
+          <t>CAND_0089012</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.5673</t>
+          <t>0.5775</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.7 YoE as NLP Engineer, possessing partial overlap in PyTorch, Information Retrieval, RAG; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 4.2 YoE as AI Specialist, possessing partial overlap in Python, NLP, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0010685</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2591,12 +2591,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.5669</t>
+          <t>0.5774</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.7 YoE as NLP Engineer, possessing partial overlap in PyTorch, Information Retrieval, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
@@ -2613,7 +2613,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.566</t>
+          <t>0.5768</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.5653</t>
+          <t>0.5755</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">

</xml_diff>

<commit_message>
fix: enforce strict YoE penalty to down-rank candidates below 5 YoE, add openpyxl to requirements.txt, update contact info
</commit_message>
<xml_diff>
--- a/outputs/mohd_ibadullah.xlsx
+++ b/outputs/mohd_ibadullah.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.907</t>
+          <t>0.9074</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.8983</t>
+          <t>0.8985</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.8626</t>
+          <t>0.8627</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -545,7 +545,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.8543</t>
+          <t>0.855</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.8489</t>
+          <t>0.8493</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -579,7 +579,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0093547</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -589,19 +589,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.8309</t>
+          <t>0.8286</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Exceptional Senior Machine Learning Engineer offering 2.9 years of experience, offers solid expertise in RAG, Python, PyTorch which matches the core ranking mandate. Highly active on Redrob with a 75% recruiter response rate.</t>
+          <t>Highly relevant Lead AI Engineer with 6.7 years of background, demonstrates strong proficiency in Information Retrieval, PyTorch, Vector Search and alignment with the JD. Highly active on Redrob with a 73% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0092278</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.8276</t>
+          <t>0.814</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Highly relevant Lead AI Engineer with 6.7 years of background, demonstrates strong proficiency in Information Retrieval, PyTorch, Vector Search and alignment with the JD. Highly active on Redrob with a 73% recruiter response rate.</t>
+          <t>Exceptional Senior NLP Engineer offering 6.8 years of experience, offers solid expertise in TensorFlow, NLP, Vector Search which matches the core ranking mandate. Highly active on Redrob with a 7% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0092278</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -633,19 +633,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.8139</t>
+          <t>0.8079</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 6.8 years of experience, offers solid expertise in TensorFlow, NLP, Vector Search which matches the core ranking mandate. Highly active on Redrob with a 7% recruiter response rate.</t>
+          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in TensorFlow, FAISS, Embeddings and search infrastructure. Available quickly with a short notice period of 15 days.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0011687</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -655,19 +655,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.8073</t>
+          <t>0.7985</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in TensorFlow, FAISS, Embeddings and search infrastructure. Available quickly with a short notice period of 15 days.</t>
+          <t>Exceptional Senior AI Engineer offering 7.8 years of experience, offers solid expertise in Pinecone, Information Retrieval, Embeddings which matches the core ranking mandate. Highly active on Redrob with a 76% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -677,19 +677,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.7977</t>
+          <t>0.7978</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Exceptional Senior AI Engineer offering 7.8 years of experience, offers solid expertise in Pinecone, Information Retrieval, Embeddings which matches the core ranking mandate. Highly active on Redrob with a 76% recruiter response rate.</t>
+          <t>Exceptional Staff Machine Learning Engineer offering 8.6 years of experience, shows deep technical expertise in Pinecone, RAG, TensorFlow and search infrastructure. Highly active on Redrob with a 83% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -699,19 +699,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.7968</t>
+          <t>0.7917</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Exceptional Staff Machine Learning Engineer offering 8.6 years of experience, shows deep technical expertise in Pinecone, RAG, TensorFlow and search infrastructure. Highly active on Redrob with a 83% recruiter response rate.</t>
+          <t>Highly relevant Lead AI Engineer with 8.6 years of background, demonstrates strong proficiency in Vector Search, NLP, MLOps and alignment with the JD. Highly active on Redrob with a 11% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -721,19 +721,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.7909</t>
+          <t>0.7881</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Highly relevant Lead AI Engineer with 8.6 years of background, demonstrates strong proficiency in Vector Search, NLP, MLOps and alignment with the JD. Highly active on Redrob with a 11% recruiter response rate.</t>
+          <t>Exceptional Senior Machine Learning Engineer offering 7.2 years of experience, has successfully deployed systems involving Pinecone, Information Retrieval, Milvus at scale. Highly active on Redrob with a 61% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -743,19 +743,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.7871</t>
+          <t>0.782</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Exceptional Senior Machine Learning Engineer offering 7.2 years of experience, has successfully deployed systems involving Pinecone, Information Retrieval, Milvus at scale. Highly active on Redrob with a 61% recruiter response rate.</t>
+          <t>Highly relevant Senior NLP Engineer with 8.9 years of background, has successfully deployed systems involving Python, Pinecone at scale. Highly active on Redrob with a 78% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0046064</t>
+          <t>CAND_0039754</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -765,19 +765,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.7817</t>
+          <t>0.7805</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Highly relevant Senior NLP Engineer with 8.9 years of background, has successfully deployed systems involving Python, Pinecone at scale. Highly active on Redrob with a 78% recruiter response rate.</t>
+          <t>Exceptional Senior Applied Scientist offering 16.2 years of experience, offers solid expertise in NLP, Python, TensorFlow which matches the core ranking mandate. Highly active on Redrob with a 81% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0039754</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -787,19 +787,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.7794</t>
+          <t>0.7705</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Strong Senior Applied Scientist with 16.2 years of experience, possessing practical experience in NLP, Python, TensorFlow. Good overall behavioral signals.</t>
+          <t>Strong Senior Machine Learning Engineer with 6.1 years of experience, matching key job requirements like Information Retrieval, TensorFlow, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0095528</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -809,12 +809,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.7698</t>
+          <t>0.7678</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Strong Senior Machine Learning Engineer with 6.1 years of experience, matching key job requirements like Information Retrieval, TensorFlow, NLP. Good overall behavioral signals.</t>
+          <t>Competent Senior Data Scientist (5.3 YoE), matching key job requirements like PyTorch, Vector Search, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.7665</t>
+          <t>0.7671</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -843,7 +843,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0095528</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -853,19 +853,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.7662</t>
+          <t>0.7614</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Competent Senior Data Scientist (5.3 YoE), matching key job requirements like PyTorch, Vector Search, Python. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Staff Machine Learning Engineer with 7.0 years in the field, matching key job requirements like Pinecone, Information Retrieval, RAG. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0060072</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -875,19 +875,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.7605</t>
+          <t>0.7568</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Solid candidate working as Staff Machine Learning Engineer with 7.0 years in the field, matching key job requirements like Pinecone, Information Retrieval, RAG. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Staff Machine Learning Engineer with 5.7 years in the field, matching key job requirements like PyTorch, Milvus, Embeddings, though platform response rate is lower (10%).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0060072</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -897,19 +897,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.7556</t>
+          <t>0.7501</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Solid candidate working as Staff Machine Learning Engineer with 5.7 years in the field, matching key job requirements like PyTorch, Milvus, Embeddings, though platform response rate is lower (10%).</t>
+          <t>Well-qualified Senior AI Engineer showing 7.9 YoE, who brings relevant experience in NLP, Python, Ranking Systems. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0037944</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -919,19 +919,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.749</t>
+          <t>0.7362</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Well-qualified Senior AI Engineer showing 7.9 YoE, who brings relevant experience in NLP, Python, Ranking Systems. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Data Scientist with 4.9 years in the field, matching key job requirements like Vector Search, Embeddings, Python, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0041611</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -941,19 +941,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.7444</t>
+          <t>0.7358</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 4.9 years in the field, matching key job requirements like Vector Search, Embeddings, Python, slightly below the preferred 5+ years of experience.</t>
+          <t>Competent Staff Machine Learning Engineer (6.4 YoE), possessing practical experience in PyTorch, NLP, MLOps, though platform response rate is lower (7%).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0041611</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -963,19 +963,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.735</t>
+          <t>0.7274</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Competent Staff Machine Learning Engineer (6.4 YoE), possessing practical experience in PyTorch, NLP, MLOps, though platform response rate is lower (7%).</t>
+          <t>Competent AI Engineer (5.7 YoE), who brings relevant experience in Information Retrieval, PyTorch, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -985,19 +985,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.7251</t>
+          <t>0.7269</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (5.7 YoE), who brings relevant experience in Information Retrieval, PyTorch, Python. Good overall behavioral signals.</t>
+          <t>Competent Applied ML Engineer (14.1 YoE), matching key job requirements like PyTorch, NLP, Embeddings, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1007,19 +1007,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.7246</t>
+          <t>0.6978</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Competent Applied ML Engineer (14.1 YoE), matching key job requirements like PyTorch, NLP, Embeddings, note the longer notice period of 90 days.</t>
+          <t>Strong Lead AI Engineer with 6.4 years of experience, who brings relevant experience in Python, Ranking Systems, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1029,19 +1029,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.6957</t>
+          <t>0.6938</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Strong Lead AI Engineer with 6.4 years of experience, who brings relevant experience in Python, Ranking Systems, NLP. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior AI Engineer with 5.9 years in the field, matching key job requirements like Python, PyTorch, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1051,19 +1051,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.6923</t>
+          <t>0.6928</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior AI Engineer with 5.9 years in the field, matching key job requirements like Python, PyTorch, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Machine Learning Engineer with 7.2 years in the field, matching key job requirements like RAG, FAISS, Embeddings, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0049896</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1073,19 +1073,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.6901</t>
+          <t>0.6817</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Solid candidate working as Machine Learning Engineer with 7.2 years in the field, matching key job requirements like RAG, FAISS, Embeddings, note the longer notice period of 120 days.</t>
+          <t>Competent Search Engineer (7.3 YoE), with matching skills in PyTorch, Information Retrieval, NLP and solid backend fundamentals, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0061339</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1095,12 +1095,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.689</t>
+          <t>0.6787</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Strong Search Engineer with 4.2 years of experience, matching key job requirements like Information Retrieval, Milvus, TensorFlow, note the longer notice period of 90 days.</t>
+          <t>Competent AI Engineer (16.9 YoE), with matching skills in Information Retrieval, FAISS, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.6831</t>
+          <t>0.6757</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1129,7 +1129,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0049896</t>
+          <t>CAND_0083307</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1139,19 +1139,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.6792</t>
+          <t>0.6735</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (7.3 YoE), with matching skills in PyTorch, Information Retrieval, NLP and solid backend fundamentals, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Search Engineer with 7.8 years in the field, matching key job requirements like Embeddings, Pinecone, Python, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1161,19 +1161,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.676</t>
+          <t>0.6696</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (16.9 YoE), with matching skills in Information Retrieval, FAISS, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0083307</t>
+          <t>CAND_0065878</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1183,19 +1183,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.6712</t>
+          <t>0.6679</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 7.8 years in the field, matching key job requirements like Embeddings, Pinecone, Python, note the longer notice period of 120 days.</t>
+          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0042506</t>
+          <t>CAND_0032515</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.6703</t>
+          <t>0.6552</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 4.2 years in the field, with matching skills in TensorFlow, Information Retrieval, Milvus and solid backend fundamentals, slightly below the preferred 5+ years of experience.</t>
+          <t>Strong Machine Learning Engineer with 5.1 years of experience, who brings relevant experience in Milvus, Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0093912</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1227,19 +1227,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.6671</t>
+          <t>0.6485</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
+          <t>Well-qualified Senior Data Scientist showing 5.3 YoE, who brings relevant experience in Milvus, Embeddings, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0065878</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.6659</t>
+          <t>0.644</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0051615</t>
+          <t>CAND_0012632</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1271,19 +1271,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.6606</t>
+          <t>0.6394</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (4.6 YoE), matching key job requirements like RAG, Milvus, Vector Search, slightly below the preferred 5+ years of experience.</t>
+          <t>Competent AI Specialist (6.0 YoE), possessing practical experience in MLOps, Python, Pinecone, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0084681</t>
+          <t>CAND_0077285</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1293,19 +1293,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.6548</t>
+          <t>0.6364</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Specialist with 3.5 years in the field, matching key job requirements like Python, Information Retrieval, Vector Search, slightly below the preferred 5+ years of experience.</t>
+          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0032515</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1315,19 +1315,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.6526</t>
+          <t>0.6311</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Strong Machine Learning Engineer with 5.1 years of experience, who brings relevant experience in Milvus, Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Competent Search Engineer (7.2 YoE), matching key job requirements like Embeddings, Information Retrieval, PyTorch, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0092245</t>
+          <t>CAND_0039838</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1337,19 +1337,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.649</t>
+          <t>0.6307</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Strong Senior Data Scientist with 4.1 years of experience, matching key job requirements like Embeddings, RAG, FAISS, slightly below the preferred 5+ years of experience.</t>
+          <t>Strong Recommendation Systems Engineer with 4.9 years of experience, with matching skills in MLOps, Embeddings, RAG and solid backend fundamentals, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0093912</t>
+          <t>CAND_0030468</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1359,19 +1359,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.6462</t>
+          <t>0.6265</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 5.3 YoE, who brings relevant experience in Milvus, Embeddings, Vector Search. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Applied Scientist with 5.4 years in the field, matching key job requirements like TensorFlow, Ranking Systems, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0024620</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1381,19 +1381,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.6419</t>
+          <t>0.6264</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (5.9 YoE), possessing practical experience in Information Retrieval, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0039838</t>
+          <t>CAND_0064326</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1403,19 +1403,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.6376</t>
+          <t>0.6254</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Strong Recommendation Systems Engineer with 4.9 years of experience, with matching skills in MLOps, Embeddings, RAG and solid backend fundamentals, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Search Engineer with 7.6 years in the field, matching key job requirements like PyTorch, Milvus, RAG. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0012632</t>
+          <t>CAND_0051615</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1425,19 +1425,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.6369</t>
+          <t>0.6246</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Competent AI Specialist (6.0 YoE), possessing practical experience in MLOps, Python, Pinecone, note the longer notice period of 120 days.</t>
+          <t>Competent Search Engineer (4.6 YoE), matching key job requirements like RAG, Milvus, Vector Search, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0076904</t>
+          <t>CAND_0036184</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1447,19 +1447,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.6363</t>
+          <t>0.624</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 4.2 YoE, possessing practical experience in Vector Search, NLP, MLOps, note the longer notice period of 90 days.</t>
+          <t>Strong Recommendation Systems Engineer with 6.0 years of experience, matching key job requirements like FAISS, MLOps, Embeddings. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0077285</t>
+          <t>CAND_0061175</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.6331</t>
+          <t>0.6225</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
+          <t>Solid candidate working as AI Research Engineer with 6.7 years in the field, with matching skills in Python, Milvus, Vector Search and solid backend fundamentals, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0099401</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1491,19 +1491,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.6284</t>
+          <t>0.6206</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (7.2 YoE), matching key job requirements like Embeddings, Information Retrieval, PyTorch, note the longer notice period of 120 days.</t>
+          <t>Strong NLP Engineer with 7.7 years of experience, who brings relevant experience in Embeddings, Information Retrieval, Python, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0008239</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.6257</t>
+          <t>0.6193</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Strong AI Engineer with 4.0 years of experience, matching key job requirements like Milvus, Vector Search, Python, slightly below the preferred 5+ years of experience.</t>
+          <t>Solid candidate working as AI Engineer with 6.7 years in the field, with matching skills in Embeddings, TensorFlow, Information Retrieval and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0054123</t>
+          <t>CAND_0070202</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1535,19 +1535,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.6248</t>
+          <t>0.6185</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Solid candidate working as Applied ML Engineer with 4.7 years in the field, matching key job requirements like Python, Vector Search, slightly below the preferred 5+ years of experience.</t>
+          <t>Competent Machine Learning Engineer (5.1 YoE), matching key job requirements like Embeddings, PyTorch, RAG, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0030468</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1557,19 +1557,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.624</t>
+          <t>0.6173</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.4 YoE as Senior Applied Scientist, mostly showing adjacent skills like TensorFlow, Ranking Systems, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0064326</t>
+          <t>CAND_0081686</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1579,19 +1579,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.6231</t>
+          <t>0.6153</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.6 YoE as Search Engineer, mostly showing adjacent skills like PyTorch, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 6.0 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, FAISS, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0036184</t>
+          <t>CAND_0061339</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1601,19 +1601,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.6211</t>
+          <t>0.614</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Recommendation Systems Engineer (6.0 YoE), mostly showing adjacent skills like FAISS, MLOps, Embeddings; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Search Engineer (4.2 YoE), mostly showing adjacent skills like Information Retrieval, Milvus, TensorFlow; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0051003</t>
+          <t>CAND_0051630</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1623,19 +1623,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.6207</t>
+          <t>0.6139</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.0 YoE as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists Embeddings, MLOps, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0061175</t>
+          <t>CAND_0006557</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1645,19 +1645,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.6203</t>
+          <t>0.613</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.7 YoE as AI Research Engineer, possessing partial overlap in Python, Milvus, Vector Search; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0099401</t>
+          <t>CAND_0052682</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1667,19 +1667,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.6183</t>
+          <t>0.6129</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as NLP Engineer (6.6 YoE), having some background in FAISS, PyTorch, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.6178</t>
+          <t>0.6128</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Candidate with 4.5 years experience as Machine Learning Engineer, mostly showing adjacent skills like MLOps, PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 8.8 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like MLOps, Python, Milvus; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1711,19 +1711,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.6167</t>
+          <t>0.6119</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.7 YoE as AI Engineer, possessing partial overlap in Embeddings, TensorFlow, Information Retrieval; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 7.9 YoE as Senior Machine Learning Engineer, possessing partial overlap in Ranking Systems, TensorFlow; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0070202</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1733,19 +1733,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.6155</t>
+          <t>0.6103</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Candidate with 5.1 years experience as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, PyTorch, RAG; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0072721</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1755,19 +1755,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.6155</t>
+          <t>0.6092</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Data Scientist (3.7 YoE), having some background in MLOps, Python, Embeddings but less specialized; included as potential pipeline filler.</t>
+          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1777,19 +1777,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.6144</t>
+          <t>0.6081</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0081686</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1799,19 +1799,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.6127</t>
+          <t>0.6062</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Candidate with 6.0 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, FAISS, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0051630</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1821,19 +1821,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.6109</t>
+          <t>0.6054</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
+          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0006557</t>
+          <t>CAND_0096172</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1843,19 +1843,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.6105</t>
+          <t>0.6036</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 5.2 YoE as NLP Engineer, possessing partial overlap in Python, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0058412</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1865,19 +1865,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.6101</t>
+          <t>0.6026</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Alternative profile showing 8.8 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like MLOps, Python, Milvus; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.6 YoE as Senior Software Engineer (ML), possessing partial overlap in Embeddings, Milvus, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0052682</t>
+          <t>CAND_0098454</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1887,19 +1887,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.6097</t>
+          <t>0.6022</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (6.6 YoE), having some background in FAISS, PyTorch, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.6094</t>
+          <t>0.6018</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.9 YoE as Senior Machine Learning Engineer, possessing partial overlap in Ranking Systems, TensorFlow; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, mostly showing adjacent skills like Milvus, TensorFlow, Python; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0029367</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1931,19 +1931,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.6071</t>
+          <t>0.6018</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0025971</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1953,19 +1953,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.6063</t>
+          <t>0.5987</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Junior ML Engineer with 5.4 years of background, having some background in FAISS, Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0032270</t>
+          <t>CAND_0054123</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1975,19 +1975,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.6059</t>
+          <t>0.5981</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Candidate with 4.4 years experience as Data Scientist, with limited direct exposure to search/ranking but lists Information Retrieval, Python, Embeddings; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 4.7 YoE as Applied ML Engineer, mostly showing adjacent skills like Python, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0089947</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1997,19 +1997,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.6048</t>
+          <t>0.5979</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Junior ML Engineer with 5.4 years of background, with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0042506</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2019,19 +2019,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.6031</t>
+          <t>0.5962</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 4.2 YoE as Search Engineer, possessing partial overlap in TensorFlow, Information Retrieval, Milvus; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2041,19 +2041,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.6028</t>
+          <t>0.5942</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
+          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0058412</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2063,19 +2063,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.6001</t>
+          <t>0.594</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Senior Software Engineer (ML), possessing partial overlap in Embeddings, Milvus, RAG; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.9 YoE as AI Engineer, mostly showing adjacent skills like Python, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0098454</t>
+          <t>CAND_0001930</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2085,19 +2085,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.5996</t>
+          <t>0.5913</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0087006</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.5994</t>
+          <t>0.5893</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.7 YoE as Senior Data Scientist, mostly showing adjacent skills like Embeddings, PyTorch, MLOps; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0077067</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.5993</t>
+          <t>0.5883</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, mostly showing adjacent skills like Milvus, TensorFlow, Python; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 5.4 YoE as AI Specialist, mostly showing adjacent skills like Python, Pinecone, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2151,19 +2151,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.5986</t>
+          <t>0.5855</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 7.3 YoE as AI Engineer, mostly showing adjacent skills like Pinecone, Vector Search, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0089947</t>
+          <t>CAND_0011125</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2173,19 +2173,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.5954</t>
+          <t>0.5851</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 5.4 years of background, with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 6.6 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, Embeddings, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0059240</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2195,19 +2195,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.5928</t>
+          <t>0.5843</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.0 YoE as Junior ML Engineer, possessing partial overlap in Milvus, NLP, Information Retrieval; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2217,19 +2217,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.5915</t>
+          <t>0.5818</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0081852</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2239,19 +2239,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.5915</t>
+          <t>0.5818</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.9 YoE as AI Engineer, mostly showing adjacent skills like Python, Vector Search; included as potential pipeline filler.</t>
+          <t>Senior Data Scientist with 5.9 years of background, having some background in Milvus, Vector Search, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2261,19 +2261,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.5887</t>
+          <t>0.5806</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0075439</t>
+          <t>CAND_0010685</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2283,19 +2283,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.5873</t>
+          <t>0.5802</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Machine Learning Engineer (4.3 YoE), with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.7 YoE as NLP Engineer, possessing partial overlap in PyTorch, Information Retrieval, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0087006</t>
+          <t>CAND_0061265</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2305,19 +2305,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.5866</t>
+          <t>0.5797</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0076831</t>
+          <t>CAND_0089498</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2327,19 +2327,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.5859</t>
+          <t>0.5791</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.0 YoE as Search Engineer, possessing partial overlap in MLOps, Milvus, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 5.8 YoE as AI Specialist, mostly showing adjacent skills like RAG, PyTorch, Python; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0007391</t>
+          <t>CAND_0064256</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.5838</t>
+          <t>0.5783</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.3 YoE as Data Scientist, possessing partial overlap in Python, Information Retrieval, TensorFlow; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0041568</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2371,19 +2371,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.5826</t>
+          <t>0.578</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.3 YoE as AI Engineer, mostly showing adjacent skills like Pinecone, Vector Search, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Search Engineer with 5.2 years of background, having some background in Vector Search, TensorFlow, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0003977</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2393,19 +2393,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.5821</t>
+          <t>0.5775</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 4.6 years of background, with limited direct exposure to search/ranking but lists NLP, Embeddings, PyTorch; included as potential pipeline filler.</t>
+          <t>Candidate with 6.8 years experience as AI Engineer, mostly showing adjacent skills like PyTorch, FAISS, NLP; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0011125</t>
+          <t>CAND_0051486</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2415,19 +2415,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.5821</t>
+          <t>0.5756</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, Embeddings, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>AI Specialist with 5.9 years of background, having some background in Pinecone, Vector Search, TensorFlow but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0002344</t>
+          <t>CAND_0091899</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2437,19 +2437,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.5812</t>
+          <t>0.5739</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Candidate with 4.7 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, TensorFlow, Pinecone; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 5.8 years experience as Senior Software Engineer (ML), possessing partial overlap in FAISS, NLP, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2459,19 +2459,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.5812</t>
+          <t>0.5736</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 4.7 YoE as Senior Data Scientist, mostly showing adjacent skills like Embeddings, PyTorch, MLOps; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0077504</t>
+          <t>CAND_0030348</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2481,19 +2481,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.5804</t>
+          <t>0.5726</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Data Scientist (4.6 YoE), having some background in Python, MLOps, Vector Search but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 4.5 years experience as Machine Learning Engineer, mostly showing adjacent skills like MLOps, PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0043860</t>
+          <t>CAND_0024466</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2503,19 +2503,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.5792</t>
+          <t>0.5712</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
+          <t>CAND_0092568</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2525,19 +2525,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.5791</t>
+          <t>0.5679</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.9 years of background, having some background in Milvus, Vector Search, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 5.7 years experience as AI Specialist, possessing partial overlap in Vector Search, Milvus, Python; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0036121</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2547,19 +2547,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.5777</t>
+          <t>0.5677</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
+          <t>Candidate with 5.2 years experience as ML Engineer, with limited direct exposure to search/ranking but lists Embeddings, Vector Search, Information Retrieval; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0089012</t>
+          <t>CAND_0044883</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.5775</t>
+          <t>0.5658</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.2 YoE as AI Specialist, possessing partial overlap in Python, NLP, MLOps; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0010685</t>
+          <t>CAND_0092245</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2591,19 +2591,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.5774</t>
+          <t>0.5655</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.7 YoE as NLP Engineer, possessing partial overlap in PyTorch, Information Retrieval, RAG; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Senior Data Scientist (4.1 YoE), mostly showing adjacent skills like Embeddings, RAG, FAISS; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0061265</t>
+          <t>CAND_0095619</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2613,19 +2613,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.5768</t>
+          <t>0.5632</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
+          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0064256</t>
+          <t>CAND_0076904</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2635,12 +2635,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.5755</t>
+          <t>0.5621</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Senior Data Scientist with 4.2 years of background, with limited direct exposure to search/ranking but lists Vector Search, NLP, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
enforced YoE penalty and updated dependencies
</commit_message>
<xml_diff>
--- a/outputs/mohd_ibadullah.xlsx
+++ b/outputs/mohd_ibadullah.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.907</t>
+          <t>0.9074</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.8983</t>
+          <t>0.8985</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.8626</t>
+          <t>0.8627</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -545,7 +545,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.8543</t>
+          <t>0.855</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.8489</t>
+          <t>0.8493</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -579,7 +579,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0093547</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -589,19 +589,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.8309</t>
+          <t>0.8286</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Exceptional Senior Machine Learning Engineer offering 2.9 years of experience, offers solid expertise in RAG, Python, PyTorch which matches the core ranking mandate. Highly active on Redrob with a 75% recruiter response rate.</t>
+          <t>Highly relevant Lead AI Engineer with 6.7 years of background, demonstrates strong proficiency in Information Retrieval, PyTorch, Vector Search and alignment with the JD. Highly active on Redrob with a 73% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0092278</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.8276</t>
+          <t>0.814</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Highly relevant Lead AI Engineer with 6.7 years of background, demonstrates strong proficiency in Information Retrieval, PyTorch, Vector Search and alignment with the JD. Highly active on Redrob with a 73% recruiter response rate.</t>
+          <t>Exceptional Senior NLP Engineer offering 6.8 years of experience, offers solid expertise in TensorFlow, NLP, Vector Search which matches the core ranking mandate. Highly active on Redrob with a 7% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0092278</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -633,19 +633,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.8139</t>
+          <t>0.8079</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 6.8 years of experience, offers solid expertise in TensorFlow, NLP, Vector Search which matches the core ranking mandate. Highly active on Redrob with a 7% recruiter response rate.</t>
+          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in TensorFlow, FAISS, Embeddings and search infrastructure. Available quickly with a short notice period of 15 days.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0011687</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -655,19 +655,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.8073</t>
+          <t>0.7985</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in TensorFlow, FAISS, Embeddings and search infrastructure. Available quickly with a short notice period of 15 days.</t>
+          <t>Exceptional Senior AI Engineer offering 7.8 years of experience, offers solid expertise in Pinecone, Information Retrieval, Embeddings which matches the core ranking mandate. Highly active on Redrob with a 76% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -677,19 +677,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.7977</t>
+          <t>0.7978</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Exceptional Senior AI Engineer offering 7.8 years of experience, offers solid expertise in Pinecone, Information Retrieval, Embeddings which matches the core ranking mandate. Highly active on Redrob with a 76% recruiter response rate.</t>
+          <t>Exceptional Staff Machine Learning Engineer offering 8.6 years of experience, shows deep technical expertise in Pinecone, RAG, TensorFlow and search infrastructure. Highly active on Redrob with a 83% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -699,19 +699,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.7968</t>
+          <t>0.7917</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Exceptional Staff Machine Learning Engineer offering 8.6 years of experience, shows deep technical expertise in Pinecone, RAG, TensorFlow and search infrastructure. Highly active on Redrob with a 83% recruiter response rate.</t>
+          <t>Highly relevant Lead AI Engineer with 8.6 years of background, demonstrates strong proficiency in Vector Search, NLP, MLOps and alignment with the JD. Highly active on Redrob with a 11% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -721,19 +721,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.7909</t>
+          <t>0.7881</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Highly relevant Lead AI Engineer with 8.6 years of background, demonstrates strong proficiency in Vector Search, NLP, MLOps and alignment with the JD. Highly active on Redrob with a 11% recruiter response rate.</t>
+          <t>Exceptional Senior Machine Learning Engineer offering 7.2 years of experience, has successfully deployed systems involving Pinecone, Information Retrieval, Milvus at scale. Highly active on Redrob with a 61% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -743,19 +743,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.7871</t>
+          <t>0.782</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Exceptional Senior Machine Learning Engineer offering 7.2 years of experience, has successfully deployed systems involving Pinecone, Information Retrieval, Milvus at scale. Highly active on Redrob with a 61% recruiter response rate.</t>
+          <t>Highly relevant Senior NLP Engineer with 8.9 years of background, has successfully deployed systems involving Python, Pinecone at scale. Highly active on Redrob with a 78% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0046064</t>
+          <t>CAND_0039754</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -765,19 +765,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.7817</t>
+          <t>0.7805</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Highly relevant Senior NLP Engineer with 8.9 years of background, has successfully deployed systems involving Python, Pinecone at scale. Highly active on Redrob with a 78% recruiter response rate.</t>
+          <t>Exceptional Senior Applied Scientist offering 16.2 years of experience, offers solid expertise in NLP, Python, TensorFlow which matches the core ranking mandate. Highly active on Redrob with a 81% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0039754</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -787,19 +787,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.7794</t>
+          <t>0.7705</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Strong Senior Applied Scientist with 16.2 years of experience, possessing practical experience in NLP, Python, TensorFlow. Good overall behavioral signals.</t>
+          <t>Strong Senior Machine Learning Engineer with 6.1 years of experience, matching key job requirements like Information Retrieval, TensorFlow, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0095528</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -809,12 +809,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.7698</t>
+          <t>0.7678</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Strong Senior Machine Learning Engineer with 6.1 years of experience, matching key job requirements like Information Retrieval, TensorFlow, NLP. Good overall behavioral signals.</t>
+          <t>Competent Senior Data Scientist (5.3 YoE), matching key job requirements like PyTorch, Vector Search, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.7665</t>
+          <t>0.7671</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -843,7 +843,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0095528</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -853,19 +853,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.7662</t>
+          <t>0.7614</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Competent Senior Data Scientist (5.3 YoE), matching key job requirements like PyTorch, Vector Search, Python. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Staff Machine Learning Engineer with 7.0 years in the field, matching key job requirements like Pinecone, Information Retrieval, RAG. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0060072</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -875,19 +875,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.7605</t>
+          <t>0.7568</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Solid candidate working as Staff Machine Learning Engineer with 7.0 years in the field, matching key job requirements like Pinecone, Information Retrieval, RAG. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Staff Machine Learning Engineer with 5.7 years in the field, matching key job requirements like PyTorch, Milvus, Embeddings, though platform response rate is lower (10%).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0060072</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -897,19 +897,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.7556</t>
+          <t>0.7501</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Solid candidate working as Staff Machine Learning Engineer with 5.7 years in the field, matching key job requirements like PyTorch, Milvus, Embeddings, though platform response rate is lower (10%).</t>
+          <t>Well-qualified Senior AI Engineer showing 7.9 YoE, who brings relevant experience in NLP, Python, Ranking Systems. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0037944</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -919,19 +919,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.749</t>
+          <t>0.7362</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Well-qualified Senior AI Engineer showing 7.9 YoE, who brings relevant experience in NLP, Python, Ranking Systems. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Data Scientist with 4.9 years in the field, matching key job requirements like Vector Search, Embeddings, Python, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0041611</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -941,19 +941,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.7444</t>
+          <t>0.7358</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 4.9 years in the field, matching key job requirements like Vector Search, Embeddings, Python, slightly below the preferred 5+ years of experience.</t>
+          <t>Competent Staff Machine Learning Engineer (6.4 YoE), possessing practical experience in PyTorch, NLP, MLOps, though platform response rate is lower (7%).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0041611</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -963,19 +963,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.735</t>
+          <t>0.7274</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Competent Staff Machine Learning Engineer (6.4 YoE), possessing practical experience in PyTorch, NLP, MLOps, though platform response rate is lower (7%).</t>
+          <t>Competent AI Engineer (5.7 YoE), who brings relevant experience in Information Retrieval, PyTorch, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -985,19 +985,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.7251</t>
+          <t>0.7269</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (5.7 YoE), who brings relevant experience in Information Retrieval, PyTorch, Python. Good overall behavioral signals.</t>
+          <t>Competent Applied ML Engineer (14.1 YoE), matching key job requirements like PyTorch, NLP, Embeddings, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1007,19 +1007,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.7246</t>
+          <t>0.6978</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Competent Applied ML Engineer (14.1 YoE), matching key job requirements like PyTorch, NLP, Embeddings, note the longer notice period of 90 days.</t>
+          <t>Strong Lead AI Engineer with 6.4 years of experience, who brings relevant experience in Python, Ranking Systems, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1029,19 +1029,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.6957</t>
+          <t>0.6938</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Strong Lead AI Engineer with 6.4 years of experience, who brings relevant experience in Python, Ranking Systems, NLP. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior AI Engineer with 5.9 years in the field, matching key job requirements like Python, PyTorch, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1051,19 +1051,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.6923</t>
+          <t>0.6928</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior AI Engineer with 5.9 years in the field, matching key job requirements like Python, PyTorch, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Machine Learning Engineer with 7.2 years in the field, matching key job requirements like RAG, FAISS, Embeddings, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0049896</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1073,19 +1073,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.6901</t>
+          <t>0.6817</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Solid candidate working as Machine Learning Engineer with 7.2 years in the field, matching key job requirements like RAG, FAISS, Embeddings, note the longer notice period of 120 days.</t>
+          <t>Competent Search Engineer (7.3 YoE), with matching skills in PyTorch, Information Retrieval, NLP and solid backend fundamentals, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0061339</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1095,12 +1095,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.689</t>
+          <t>0.6787</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Strong Search Engineer with 4.2 years of experience, matching key job requirements like Information Retrieval, Milvus, TensorFlow, note the longer notice period of 90 days.</t>
+          <t>Competent AI Engineer (16.9 YoE), with matching skills in Information Retrieval, FAISS, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.6831</t>
+          <t>0.6757</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1129,7 +1129,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0049896</t>
+          <t>CAND_0083307</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1139,19 +1139,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.6792</t>
+          <t>0.6735</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (7.3 YoE), with matching skills in PyTorch, Information Retrieval, NLP and solid backend fundamentals, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Search Engineer with 7.8 years in the field, matching key job requirements like Embeddings, Pinecone, Python, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1161,19 +1161,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.676</t>
+          <t>0.6696</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (16.9 YoE), with matching skills in Information Retrieval, FAISS, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0083307</t>
+          <t>CAND_0065878</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1183,19 +1183,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.6712</t>
+          <t>0.6679</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 7.8 years in the field, matching key job requirements like Embeddings, Pinecone, Python, note the longer notice period of 120 days.</t>
+          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0042506</t>
+          <t>CAND_0032515</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.6703</t>
+          <t>0.6552</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 4.2 years in the field, with matching skills in TensorFlow, Information Retrieval, Milvus and solid backend fundamentals, slightly below the preferred 5+ years of experience.</t>
+          <t>Strong Machine Learning Engineer with 5.1 years of experience, who brings relevant experience in Milvus, Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0093912</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1227,19 +1227,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.6671</t>
+          <t>0.6485</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
+          <t>Well-qualified Senior Data Scientist showing 5.3 YoE, who brings relevant experience in Milvus, Embeddings, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0065878</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.6659</t>
+          <t>0.644</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0051615</t>
+          <t>CAND_0012632</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1271,19 +1271,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.6606</t>
+          <t>0.6394</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (4.6 YoE), matching key job requirements like RAG, Milvus, Vector Search, slightly below the preferred 5+ years of experience.</t>
+          <t>Competent AI Specialist (6.0 YoE), possessing practical experience in MLOps, Python, Pinecone, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0084681</t>
+          <t>CAND_0077285</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1293,19 +1293,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.6548</t>
+          <t>0.6364</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Specialist with 3.5 years in the field, matching key job requirements like Python, Information Retrieval, Vector Search, slightly below the preferred 5+ years of experience.</t>
+          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0032515</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1315,19 +1315,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.6526</t>
+          <t>0.6311</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Strong Machine Learning Engineer with 5.1 years of experience, who brings relevant experience in Milvus, Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Competent Search Engineer (7.2 YoE), matching key job requirements like Embeddings, Information Retrieval, PyTorch, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0092245</t>
+          <t>CAND_0039838</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1337,19 +1337,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.649</t>
+          <t>0.6307</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Strong Senior Data Scientist with 4.1 years of experience, matching key job requirements like Embeddings, RAG, FAISS, slightly below the preferred 5+ years of experience.</t>
+          <t>Strong Recommendation Systems Engineer with 4.9 years of experience, with matching skills in MLOps, Embeddings, RAG and solid backend fundamentals, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0093912</t>
+          <t>CAND_0030468</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1359,19 +1359,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.6462</t>
+          <t>0.6265</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 5.3 YoE, who brings relevant experience in Milvus, Embeddings, Vector Search. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Applied Scientist with 5.4 years in the field, matching key job requirements like TensorFlow, Ranking Systems, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0024620</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1381,19 +1381,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.6419</t>
+          <t>0.6264</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (5.9 YoE), possessing practical experience in Information Retrieval, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0039838</t>
+          <t>CAND_0064326</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1403,19 +1403,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.6376</t>
+          <t>0.6254</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Strong Recommendation Systems Engineer with 4.9 years of experience, with matching skills in MLOps, Embeddings, RAG and solid backend fundamentals, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Search Engineer with 7.6 years in the field, matching key job requirements like PyTorch, Milvus, RAG. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0012632</t>
+          <t>CAND_0051615</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1425,19 +1425,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.6369</t>
+          <t>0.6246</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Competent AI Specialist (6.0 YoE), possessing practical experience in MLOps, Python, Pinecone, note the longer notice period of 120 days.</t>
+          <t>Competent Search Engineer (4.6 YoE), matching key job requirements like RAG, Milvus, Vector Search, slightly below the preferred 5+ years of experience.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0076904</t>
+          <t>CAND_0036184</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1447,19 +1447,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.6363</t>
+          <t>0.624</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 4.2 YoE, possessing practical experience in Vector Search, NLP, MLOps, note the longer notice period of 90 days.</t>
+          <t>Strong Recommendation Systems Engineer with 6.0 years of experience, matching key job requirements like FAISS, MLOps, Embeddings. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0077285</t>
+          <t>CAND_0061175</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.6331</t>
+          <t>0.6225</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
+          <t>Solid candidate working as AI Research Engineer with 6.7 years in the field, with matching skills in Python, Milvus, Vector Search and solid backend fundamentals, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0099401</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1491,19 +1491,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.6284</t>
+          <t>0.6206</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (7.2 YoE), matching key job requirements like Embeddings, Information Retrieval, PyTorch, note the longer notice period of 120 days.</t>
+          <t>Strong NLP Engineer with 7.7 years of experience, who brings relevant experience in Embeddings, Information Retrieval, Python, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0008239</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.6257</t>
+          <t>0.6193</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Strong AI Engineer with 4.0 years of experience, matching key job requirements like Milvus, Vector Search, Python, slightly below the preferred 5+ years of experience.</t>
+          <t>Solid candidate working as AI Engineer with 6.7 years in the field, with matching skills in Embeddings, TensorFlow, Information Retrieval and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0054123</t>
+          <t>CAND_0070202</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1535,19 +1535,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.6248</t>
+          <t>0.6185</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Solid candidate working as Applied ML Engineer with 4.7 years in the field, matching key job requirements like Python, Vector Search, slightly below the preferred 5+ years of experience.</t>
+          <t>Competent Machine Learning Engineer (5.1 YoE), matching key job requirements like Embeddings, PyTorch, RAG, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0030468</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1557,19 +1557,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.624</t>
+          <t>0.6173</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.4 YoE as Senior Applied Scientist, mostly showing adjacent skills like TensorFlow, Ranking Systems, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0064326</t>
+          <t>CAND_0081686</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1579,19 +1579,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.6231</t>
+          <t>0.6153</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.6 YoE as Search Engineer, mostly showing adjacent skills like PyTorch, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 6.0 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, FAISS, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0036184</t>
+          <t>CAND_0061339</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1601,19 +1601,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.6211</t>
+          <t>0.614</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Recommendation Systems Engineer (6.0 YoE), mostly showing adjacent skills like FAISS, MLOps, Embeddings; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Search Engineer (4.2 YoE), mostly showing adjacent skills like Information Retrieval, Milvus, TensorFlow; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0051003</t>
+          <t>CAND_0051630</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1623,19 +1623,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.6207</t>
+          <t>0.6139</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.0 YoE as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists Embeddings, MLOps, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0061175</t>
+          <t>CAND_0006557</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1645,19 +1645,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.6203</t>
+          <t>0.613</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.7 YoE as AI Research Engineer, possessing partial overlap in Python, Milvus, Vector Search; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0099401</t>
+          <t>CAND_0052682</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1667,19 +1667,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.6183</t>
+          <t>0.6129</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as NLP Engineer (6.6 YoE), having some background in FAISS, PyTorch, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.6178</t>
+          <t>0.6128</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Candidate with 4.5 years experience as Machine Learning Engineer, mostly showing adjacent skills like MLOps, PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 8.8 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like MLOps, Python, Milvus; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1711,19 +1711,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.6167</t>
+          <t>0.6119</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.7 YoE as AI Engineer, possessing partial overlap in Embeddings, TensorFlow, Information Retrieval; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 7.9 YoE as Senior Machine Learning Engineer, possessing partial overlap in Ranking Systems, TensorFlow; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0070202</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1733,19 +1733,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.6155</t>
+          <t>0.6103</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Candidate with 5.1 years experience as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, PyTorch, RAG; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0072721</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1755,19 +1755,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.6155</t>
+          <t>0.6092</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Data Scientist (3.7 YoE), having some background in MLOps, Python, Embeddings but less specialized; included as potential pipeline filler.</t>
+          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1777,19 +1777,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.6144</t>
+          <t>0.6081</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0081686</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1799,19 +1799,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.6127</t>
+          <t>0.6062</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Candidate with 6.0 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, FAISS, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0051630</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1821,19 +1821,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.6109</t>
+          <t>0.6054</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
+          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0006557</t>
+          <t>CAND_0096172</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1843,19 +1843,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.6105</t>
+          <t>0.6036</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 5.2 YoE as NLP Engineer, possessing partial overlap in Python, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0058412</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1865,19 +1865,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.6101</t>
+          <t>0.6026</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Alternative profile showing 8.8 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like MLOps, Python, Milvus; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.6 YoE as Senior Software Engineer (ML), possessing partial overlap in Embeddings, Milvus, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0052682</t>
+          <t>CAND_0098454</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1887,19 +1887,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.6097</t>
+          <t>0.6022</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (6.6 YoE), having some background in FAISS, PyTorch, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.6094</t>
+          <t>0.6018</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.9 YoE as Senior Machine Learning Engineer, possessing partial overlap in Ranking Systems, TensorFlow; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, mostly showing adjacent skills like Milvus, TensorFlow, Python; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0029367</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1931,19 +1931,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.6071</t>
+          <t>0.6018</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0025971</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1953,19 +1953,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.6063</t>
+          <t>0.5987</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Junior ML Engineer with 5.4 years of background, having some background in FAISS, Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0032270</t>
+          <t>CAND_0054123</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1975,19 +1975,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.6059</t>
+          <t>0.5981</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Candidate with 4.4 years experience as Data Scientist, with limited direct exposure to search/ranking but lists Information Retrieval, Python, Embeddings; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 4.7 YoE as Applied ML Engineer, mostly showing adjacent skills like Python, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0089947</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1997,19 +1997,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.6048</t>
+          <t>0.5979</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Junior ML Engineer with 5.4 years of background, with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0042506</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2019,19 +2019,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.6031</t>
+          <t>0.5962</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 4.2 YoE as Search Engineer, possessing partial overlap in TensorFlow, Information Retrieval, Milvus; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2041,19 +2041,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.6028</t>
+          <t>0.5942</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
+          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0058412</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2063,19 +2063,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.6001</t>
+          <t>0.594</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Senior Software Engineer (ML), possessing partial overlap in Embeddings, Milvus, RAG; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.9 YoE as AI Engineer, mostly showing adjacent skills like Python, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0098454</t>
+          <t>CAND_0001930</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2085,19 +2085,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.5996</t>
+          <t>0.5913</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0087006</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.5994</t>
+          <t>0.5893</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.7 YoE as Senior Data Scientist, mostly showing adjacent skills like Embeddings, PyTorch, MLOps; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0077067</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.5993</t>
+          <t>0.5883</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, mostly showing adjacent skills like Milvus, TensorFlow, Python; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 5.4 YoE as AI Specialist, mostly showing adjacent skills like Python, Pinecone, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2151,19 +2151,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.5986</t>
+          <t>0.5855</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 7.3 YoE as AI Engineer, mostly showing adjacent skills like Pinecone, Vector Search, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0089947</t>
+          <t>CAND_0011125</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2173,19 +2173,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.5954</t>
+          <t>0.5851</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 5.4 years of background, with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 6.6 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, Embeddings, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0059240</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2195,19 +2195,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.5928</t>
+          <t>0.5843</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.0 YoE as Junior ML Engineer, possessing partial overlap in Milvus, NLP, Information Retrieval; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2217,19 +2217,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.5915</t>
+          <t>0.5818</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0081852</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2239,19 +2239,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.5915</t>
+          <t>0.5818</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.9 YoE as AI Engineer, mostly showing adjacent skills like Python, Vector Search; included as potential pipeline filler.</t>
+          <t>Senior Data Scientist with 5.9 years of background, having some background in Milvus, Vector Search, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2261,19 +2261,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.5887</t>
+          <t>0.5806</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0075439</t>
+          <t>CAND_0010685</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2283,19 +2283,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.5873</t>
+          <t>0.5802</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Machine Learning Engineer (4.3 YoE), with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.7 YoE as NLP Engineer, possessing partial overlap in PyTorch, Information Retrieval, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0087006</t>
+          <t>CAND_0061265</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2305,19 +2305,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.5866</t>
+          <t>0.5797</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0076831</t>
+          <t>CAND_0089498</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2327,19 +2327,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.5859</t>
+          <t>0.5791</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.0 YoE as Search Engineer, possessing partial overlap in MLOps, Milvus, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 5.8 YoE as AI Specialist, mostly showing adjacent skills like RAG, PyTorch, Python; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0007391</t>
+          <t>CAND_0064256</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.5838</t>
+          <t>0.5783</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.3 YoE as Data Scientist, possessing partial overlap in Python, Information Retrieval, TensorFlow; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0041568</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2371,19 +2371,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.5826</t>
+          <t>0.578</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.3 YoE as AI Engineer, mostly showing adjacent skills like Pinecone, Vector Search, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Search Engineer with 5.2 years of background, having some background in Vector Search, TensorFlow, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0003977</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2393,19 +2393,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.5821</t>
+          <t>0.5775</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 4.6 years of background, with limited direct exposure to search/ranking but lists NLP, Embeddings, PyTorch; included as potential pipeline filler.</t>
+          <t>Candidate with 6.8 years experience as AI Engineer, mostly showing adjacent skills like PyTorch, FAISS, NLP; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0011125</t>
+          <t>CAND_0051486</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2415,19 +2415,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.5821</t>
+          <t>0.5756</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, Embeddings, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>AI Specialist with 5.9 years of background, having some background in Pinecone, Vector Search, TensorFlow but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0002344</t>
+          <t>CAND_0091899</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2437,19 +2437,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.5812</t>
+          <t>0.5739</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Candidate with 4.7 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, TensorFlow, Pinecone; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 5.8 years experience as Senior Software Engineer (ML), possessing partial overlap in FAISS, NLP, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2459,19 +2459,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.5812</t>
+          <t>0.5736</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 4.7 YoE as Senior Data Scientist, mostly showing adjacent skills like Embeddings, PyTorch, MLOps; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0077504</t>
+          <t>CAND_0030348</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2481,19 +2481,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.5804</t>
+          <t>0.5726</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Data Scientist (4.6 YoE), having some background in Python, MLOps, Vector Search but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 4.5 years experience as Machine Learning Engineer, mostly showing adjacent skills like MLOps, PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0043860</t>
+          <t>CAND_0024466</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2503,19 +2503,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.5792</t>
+          <t>0.5712</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
+          <t>CAND_0092568</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2525,19 +2525,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.5791</t>
+          <t>0.5679</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.9 years of background, having some background in Milvus, Vector Search, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 5.7 years experience as AI Specialist, possessing partial overlap in Vector Search, Milvus, Python; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0036121</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2547,19 +2547,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.5777</t>
+          <t>0.5677</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
+          <t>Candidate with 5.2 years experience as ML Engineer, with limited direct exposure to search/ranking but lists Embeddings, Vector Search, Information Retrieval; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0089012</t>
+          <t>CAND_0044883</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.5775</t>
+          <t>0.5658</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.2 YoE as AI Specialist, possessing partial overlap in Python, NLP, MLOps; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0010685</t>
+          <t>CAND_0092245</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2591,19 +2591,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.5774</t>
+          <t>0.5655</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.7 YoE as NLP Engineer, possessing partial overlap in PyTorch, Information Retrieval, RAG; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Senior Data Scientist (4.1 YoE), mostly showing adjacent skills like Embeddings, RAG, FAISS; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0061265</t>
+          <t>CAND_0095619</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2613,19 +2613,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.5768</t>
+          <t>0.5632</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
+          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0064256</t>
+          <t>CAND_0076904</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2635,12 +2635,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.5755</t>
+          <t>0.5621</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Senior Data Scientist with 4.2 years of background, with limited direct exposure to search/ranking but lists Vector Search, NLP, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: complete win-ready ranking engine (hard YoE gating, career keywords bonus, behavioral signals, timeline honeypots)
</commit_message>
<xml_diff>
--- a/outputs/mohd_ibadullah.xlsx
+++ b/outputs/mohd_ibadullah.xlsx
@@ -457,7 +457,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.9305</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.9074</t>
+          <t>0.9684</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.8985</t>
+          <t>0.9593</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -513,7 +513,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0008425</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -523,19 +523,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.8627</t>
+          <t>0.9388</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in NLP, TensorFlow, Python and search infrastructure. Highly active on Redrob with a 66% recruiter response rate.</t>
+          <t>Highly relevant Senior AI Engineer with 5.9 years of background, offers solid expertise in FAISS, TensorFlow, NLP which matches the core ranking mandate. Excellent platform engagement with 80% response rate.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -545,19 +545,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.855</t>
+          <t>0.9179</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Highly relevant Senior AI Engineer with 5.9 years of background, offers solid expertise in FAISS, TensorFlow, NLP which matches the core ranking mandate. Excellent platform engagement with 80% response rate.</t>
+          <t>Highly relevant Lead AI Engineer with 6.7 years of background, demonstrates strong proficiency in Information Retrieval, PyTorch, Vector Search and alignment with the JD. Highly active on Redrob with a 73% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0007411</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -567,19 +567,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.8493</t>
+          <t>0.8996</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Top-tier candidate currently working as Senior Machine Learning Engineer (8.0 YoE), offers solid expertise in Vector Search, PyTorch, Information Retrieval which matches the core ranking mandate. Excellent platform engagement with 12% response rate.</t>
+          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in TensorFlow, FAISS, Embeddings and search infrastructure. Available quickly with a short notice period of 15 days.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0008425</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -589,19 +589,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.8286</t>
+          <t>0.8929</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Highly relevant Lead AI Engineer with 6.7 years of background, demonstrates strong proficiency in Information Retrieval, PyTorch, Vector Search and alignment with the JD. Highly active on Redrob with a 73% recruiter response rate.</t>
+          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in NLP, TensorFlow, Python and search infrastructure. Highly active on Redrob with a 66% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0092278</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.814</t>
+          <t>0.8909</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 6.8 years of experience, offers solid expertise in TensorFlow, NLP, Vector Search which matches the core ranking mandate. Highly active on Redrob with a 7% recruiter response rate.</t>
+          <t>Exceptional Senior AI Engineer offering 7.8 years of experience, offers solid expertise in Pinecone, Information Retrieval, Embeddings which matches the core ranking mandate. Highly active on Redrob with a 76% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0011687</t>
+          <t>CAND_0039754</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -633,19 +633,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.8079</t>
+          <t>0.8739</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in TensorFlow, FAISS, Embeddings and search infrastructure. Available quickly with a short notice period of 15 days.</t>
+          <t>Exceptional Senior Applied Scientist offering 16.2 years of experience, offers solid expertise in NLP, Python, TensorFlow which matches the core ranking mandate. Highly active on Redrob with a 81% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -655,19 +655,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.7985</t>
+          <t>0.8728</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Exceptional Senior AI Engineer offering 7.8 years of experience, offers solid expertise in Pinecone, Information Retrieval, Embeddings which matches the core ranking mandate. Highly active on Redrob with a 76% recruiter response rate.</t>
+          <t>Highly relevant Senior NLP Engineer with 8.9 years of background, has successfully deployed systems involving Python, Pinecone at scale. Highly active on Redrob with a 78% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -677,19 +677,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.7978</t>
+          <t>0.8624</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Exceptional Staff Machine Learning Engineer offering 8.6 years of experience, shows deep technical expertise in Pinecone, RAG, TensorFlow and search infrastructure. Highly active on Redrob with a 83% recruiter response rate.</t>
+          <t>Exceptional Senior Machine Learning Engineer offering 6.1 years of experience, demonstrates strong proficiency in Information Retrieval, TensorFlow, NLP and alignment with the JD. Highly active on Redrob with a 88% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -699,19 +699,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.7917</t>
+          <t>0.8605</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Highly relevant Lead AI Engineer with 8.6 years of background, demonstrates strong proficiency in Vector Search, NLP, MLOps and alignment with the JD. Highly active on Redrob with a 11% recruiter response rate.</t>
+          <t>Exceptional Staff Machine Learning Engineer offering 8.6 years of experience, shows deep technical expertise in Pinecone, RAG, TensorFlow and search infrastructure. Highly active on Redrob with a 83% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -721,19 +721,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.7881</t>
+          <t>0.8543</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Exceptional Senior Machine Learning Engineer offering 7.2 years of experience, has successfully deployed systems involving Pinecone, Information Retrieval, Milvus at scale. Highly active on Redrob with a 61% recruiter response rate.</t>
+          <t>Highly relevant Staff Machine Learning Engineer with 7.0 years of background, demonstrates strong proficiency in Pinecone, Information Retrieval, RAG and alignment with the JD. Highly active on Redrob with a 95% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0046064</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -743,19 +743,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.782</t>
+          <t>0.8511</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Highly relevant Senior NLP Engineer with 8.9 years of background, has successfully deployed systems involving Python, Pinecone at scale. Highly active on Redrob with a 78% recruiter response rate.</t>
+          <t>Exceptional Senior Machine Learning Engineer offering 7.2 years of experience, has successfully deployed systems involving Pinecone, Information Retrieval, Milvus at scale. Highly active on Redrob with a 61% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0039754</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -765,19 +765,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.7805</t>
+          <t>0.8433</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Exceptional Senior Applied Scientist offering 16.2 years of experience, offers solid expertise in NLP, Python, TensorFlow which matches the core ranking mandate. Highly active on Redrob with a 81% recruiter response rate.</t>
+          <t>Outstanding candidate as Senior AI Engineer showing 7.9 years of experience, shows deep technical expertise in NLP, Python, Ranking Systems and search infrastructure. Highly active on Redrob with a 79% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0095528</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -787,19 +787,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.7705</t>
+          <t>0.8324</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Strong Senior Machine Learning Engineer with 6.1 years of experience, matching key job requirements like Information Retrieval, TensorFlow, NLP. Good overall behavioral signals.</t>
+          <t>Competent Senior Data Scientist (5.3 YoE), matching key job requirements like PyTorch, Vector Search, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0095528</t>
+          <t>CAND_0033861</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -809,19 +809,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.7678</t>
+          <t>0.8289</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Competent Senior Data Scientist (5.3 YoE), matching key job requirements like PyTorch, Vector Search, Python. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior NLP Engineer with 8.0 years in the field, matching key job requirements like TensorFlow, Pinecone, Vector Search, though platform response rate is lower (16%).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0033861</t>
+          <t>CAND_0007411</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -831,19 +831,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.7671</t>
+          <t>0.8205</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior NLP Engineer with 8.0 years in the field, matching key job requirements like TensorFlow, Pinecone, Vector Search, though platform response rate is lower (16%).</t>
+          <t>Competent Senior Machine Learning Engineer (8.0 YoE), possessing practical experience in Vector Search, PyTorch, Information Retrieval, though platform response rate is lower (12%).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -853,19 +853,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.7614</t>
+          <t>0.7943</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Solid candidate working as Staff Machine Learning Engineer with 7.0 years in the field, matching key job requirements like Pinecone, Information Retrieval, RAG. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (5.7 YoE), who brings relevant experience in Information Retrieval, PyTorch, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0060072</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -875,19 +875,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.7568</t>
+          <t>0.794</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Solid candidate working as Staff Machine Learning Engineer with 5.7 years in the field, matching key job requirements like PyTorch, Milvus, Embeddings, though platform response rate is lower (10%).</t>
+          <t>Solid candidate working as Lead AI Engineer with 8.6 years in the field, matching key job requirements like Vector Search, NLP, MLOps, though platform response rate is lower (11%).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -897,19 +897,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.7501</t>
+          <t>0.7876</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Well-qualified Senior AI Engineer showing 7.9 YoE, who brings relevant experience in NLP, Python, Ranking Systems. Good overall behavioral signals.</t>
+          <t>Competent Applied ML Engineer (14.1 YoE), matching key job requirements like PyTorch, NLP, Embeddings, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -919,19 +919,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.7362</t>
+          <t>0.7766</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 4.9 years in the field, matching key job requirements like Vector Search, Embeddings, Python, slightly below the preferred 5+ years of experience.</t>
+          <t>Competent AI Engineer (16.9 YoE), with matching skills in Information Retrieval, FAISS, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0041611</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -941,19 +941,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.7358</t>
+          <t>0.7583</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Competent Staff Machine Learning Engineer (6.4 YoE), possessing practical experience in PyTorch, NLP, MLOps, though platform response rate is lower (7%).</t>
+          <t>Solid candidate working as Senior AI Engineer with 5.9 years in the field, matching key job requirements like Python, PyTorch, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -963,19 +963,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.7274</t>
+          <t>0.758</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (5.7 YoE), who brings relevant experience in Information Retrieval, PyTorch, Python. Good overall behavioral signals.</t>
+          <t>Strong Lead AI Engineer with 6.4 years of experience, who brings relevant experience in Python, Ranking Systems, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0083307</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -985,19 +985,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.7269</t>
+          <t>0.7402</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Competent Applied ML Engineer (14.1 YoE), matching key job requirements like PyTorch, NLP, Embeddings, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Search Engineer with 7.8 years in the field, matching key job requirements like Embeddings, Pinecone, Python, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1007,19 +1007,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.6978</t>
+          <t>0.7371</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Strong Lead AI Engineer with 6.4 years of experience, who brings relevant experience in Python, Ranking Systems, NLP. Good overall behavioral signals.</t>
+          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0065878</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1029,12 +1029,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.6938</t>
+          <t>0.7339</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior AI Engineer with 5.9 years in the field, matching key job requirements like Python, PyTorch, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.6928</t>
+          <t>0.7306</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1063,7 +1063,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0049896</t>
+          <t>CAND_0032515</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1073,19 +1073,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.6817</t>
+          <t>0.7226</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (7.3 YoE), with matching skills in PyTorch, Information Retrieval, NLP and solid backend fundamentals, note the longer notice period of 90 days.</t>
+          <t>Strong Machine Learning Engineer with 5.1 years of experience, who brings relevant experience in Milvus, Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0036184</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1095,19 +1095,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.6787</t>
+          <t>0.7224</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (16.9 YoE), with matching skills in Information Retrieval, FAISS, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Strong Recommendation Systems Engineer with 6.0 years of experience, matching key job requirements like FAISS, MLOps, Embeddings. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0064904</t>
+          <t>CAND_0064326</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1117,19 +1117,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.6757</t>
+          <t>0.7224</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Strong AI Engineer with 4.9 years of experience, who brings relevant experience in Embeddings, Python, MLOps, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Search Engineer with 7.6 years in the field, matching key job requirements like PyTorch, Milvus, RAG. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0083307</t>
+          <t>CAND_0049896</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1139,19 +1139,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.6735</t>
+          <t>0.7189</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 7.8 years in the field, matching key job requirements like Embeddings, Pinecone, Python, note the longer notice period of 120 days.</t>
+          <t>Competent Search Engineer (7.3 YoE), with matching skills in PyTorch, Information Retrieval, NLP and solid backend fundamentals, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0093912</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1161,19 +1161,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.6696</t>
+          <t>0.7154</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
+          <t>Well-qualified Senior Data Scientist showing 5.3 YoE, who brings relevant experience in Milvus, Embeddings, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0065878</t>
+          <t>CAND_0052682</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1183,19 +1183,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.6679</t>
+          <t>0.7123</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
+          <t>Strong NLP Engineer with 6.6 years of experience, who brings relevant experience in FAISS, PyTorch, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0032515</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.6552</t>
+          <t>0.711</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Strong Machine Learning Engineer with 5.1 years of experience, who brings relevant experience in Milvus, Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Solid candidate working as AI Engineer with 6.7 years in the field, with matching skills in Embeddings, TensorFlow, Information Retrieval and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0093912</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1227,19 +1227,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.6485</t>
+          <t>0.7042</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 5.3 YoE, who brings relevant experience in Milvus, Embeddings, Vector Search. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0077285</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.644</t>
+          <t>0.7002</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0012632</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1271,19 +1271,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.6394</t>
+          <t>0.6915</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Competent AI Specialist (6.0 YoE), possessing practical experience in MLOps, Python, Pinecone, note the longer notice period of 120 days.</t>
+          <t>Solid candidate working as AI Engineer with 6.9 years in the field, matching key job requirements like Python, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0077285</t>
+          <t>CAND_0024620</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1293,19 +1293,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.6364</t>
+          <t>0.6865</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (5.9 YoE), possessing practical experience in Information Retrieval, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1315,19 +1315,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.6311</t>
+          <t>0.6842</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (7.2 YoE), matching key job requirements like Embeddings, Information Retrieval, PyTorch, note the longer notice period of 120 days.</t>
+          <t>Solid candidate working as AI Engineer with 7.3 years in the field, matching key job requirements like Pinecone, Vector Search, RAG. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0039838</t>
+          <t>CAND_0081686</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1337,12 +1337,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.6307</t>
+          <t>0.6831</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Strong Recommendation Systems Engineer with 4.9 years of experience, with matching skills in MLOps, Embeddings, RAG and solid backend fundamentals, note the longer notice period of 90 days.</t>
+          <t>Competent Search Engineer (6.0 YoE), matching key job requirements like Embeddings, FAISS, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.6265</t>
+          <t>0.6818</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1371,7 +1371,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0024620</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1381,19 +1381,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.6264</t>
+          <t>0.6806</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (5.9 YoE), possessing practical experience in Information Retrieval, Python. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Staff Machine Learning Engineer with 8.8 years in the field, matching key job requirements like MLOps, Python, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0064326</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1403,19 +1403,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.6254</t>
+          <t>0.68</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 7.6 years in the field, matching key job requirements like PyTorch, Milvus, RAG. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Data Scientist with 5.7 years in the field, matching key job requirements like TensorFlow, FAISS, RAG, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0051615</t>
+          <t>CAND_0010685</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1425,19 +1425,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.6246</t>
+          <t>0.6782</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (4.6 YoE), matching key job requirements like RAG, Milvus, Vector Search, slightly below the preferred 5+ years of experience.</t>
+          <t>Solid candidate working as NLP Engineer with 6.7 years in the field, with matching skills in PyTorch, Information Retrieval, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0036184</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1447,19 +1447,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.624</t>
+          <t>0.6777</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Strong Recommendation Systems Engineer with 6.0 years of experience, matching key job requirements like FAISS, MLOps, Embeddings. Good overall behavioral signals.</t>
+          <t>Competent Recommendation Systems Engineer (5.8 YoE), matching key job requirements like FAISS, Vector Search, Milvus, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0061175</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.6225</t>
+          <t>0.6769</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Research Engineer with 6.7 years in the field, with matching skills in Python, Milvus, Vector Search and solid backend fundamentals, note the longer notice period of 120 days.</t>
+          <t>Competent AI Engineer (6.8 YoE), matching key job requirements like PyTorch, FAISS, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0099401</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1491,19 +1491,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.6206</t>
+          <t>0.6754</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Strong NLP Engineer with 7.7 years of experience, who brings relevant experience in Embeddings, Information Retrieval, Python, note the longer notice period of 90 days.</t>
+          <t>Strong Applied ML Engineer with 5.2 years of experience, who brings relevant experience in FAISS, Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0070525</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.6193</t>
+          <t>0.6751</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 6.7 years in the field, with matching skills in Embeddings, TensorFlow, Information Retrieval and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Strong Senior Software Engineer (ML) with 5.4 years of experience, who brings relevant experience in Python, Embeddings. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0070202</t>
+          <t>CAND_0096172</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1535,19 +1535,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.6185</t>
+          <t>0.6705</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Competent Machine Learning Engineer (5.1 YoE), matching key job requirements like Embeddings, PyTorch, RAG, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as NLP Engineer with 5.2 years in the field, with matching skills in Python, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0058412</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1557,19 +1557,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.6173</t>
+          <t>0.6698</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.6 YoE as Senior Software Engineer (ML), possessing partial overlap in Embeddings, Milvus, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0081686</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1579,19 +1579,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.6153</t>
+          <t>0.6691</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Candidate with 6.0 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, FAISS, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, mostly showing adjacent skills like Milvus, TensorFlow, Python; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0061339</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1601,19 +1601,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.614</t>
+          <t>0.6689</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Search Engineer (4.2 YoE), mostly showing adjacent skills like Information Retrieval, Milvus, TensorFlow; included as potential pipeline filler.</t>
+          <t>Candidate with 7.2 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, Information Retrieval, PyTorch; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0051630</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1623,19 +1623,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.6139</t>
+          <t>0.6671</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
+          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0006557</t>
+          <t>CAND_0061175</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1645,19 +1645,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.613</t>
+          <t>0.6588</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 6.7 YoE as AI Research Engineer, possessing partial overlap in Python, Milvus, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0052682</t>
+          <t>CAND_0098454</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1667,19 +1667,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.6129</t>
+          <t>0.658</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (6.6 YoE), having some background in FAISS, PyTorch, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0070202</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.6128</t>
+          <t>0.6576</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Alternative profile showing 8.8 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like MLOps, Python, Milvus; included as potential pipeline filler.</t>
+          <t>Candidate with 5.1 years experience as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, PyTorch, RAG; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0099401</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1711,19 +1711,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.6119</t>
+          <t>0.6575</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.9 YoE as Senior Machine Learning Engineer, possessing partial overlap in Ranking Systems, TensorFlow; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0029367</t>
+          <t>CAND_0025882</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1733,19 +1733,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.6103</t>
+          <t>0.6563</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 5.6 YoE as Senior Software Engineer (ML), possessing partial overlap in FAISS, Vector Search, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1755,19 +1755,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.6092</t>
+          <t>0.6559</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1777,19 +1777,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.6081</t>
+          <t>0.6559</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1799,19 +1799,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.6062</t>
+          <t>0.6556</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0000031</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1821,19 +1821,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.6054</t>
+          <t>0.6547</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
+          <t>Recommendation Systems Engineer with 6.0 years of background, possessing partial overlap in FAISS, Pinecone, MLOps; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0096172</t>
+          <t>CAND_0051630</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1843,19 +1843,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.6036</t>
+          <t>0.6529</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.2 YoE as NLP Engineer, possessing partial overlap in Python, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0058412</t>
+          <t>CAND_0012837</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1865,19 +1865,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.6026</t>
+          <t>0.6514</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Senior Software Engineer (ML), possessing partial overlap in Embeddings, Milvus, RAG; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.4 YoE as Junior ML Engineer, mostly showing adjacent skills like Vector Search, MLOps, NLP; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0098454</t>
+          <t>CAND_0006557</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1887,19 +1887,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.6022</t>
+          <t>0.6507</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.6018</t>
+          <t>0.6491</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, mostly showing adjacent skills like Milvus, TensorFlow, Python; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0061265</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1931,19 +1931,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.6018</t>
+          <t>0.6483</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0025971</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1953,19 +1953,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.5987</t>
+          <t>0.6477</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 5.4 years of background, having some background in FAISS, Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0054123</t>
+          <t>CAND_0095619</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1975,19 +1975,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.5981</t>
+          <t>0.6393</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.7 YoE as Applied ML Engineer, mostly showing adjacent skills like Python, Vector Search; included as potential pipeline filler.</t>
+          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0089947</t>
+          <t>CAND_0064256</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1997,19 +1997,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.5979</t>
+          <t>0.6345</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 5.4 years of background, with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0042506</t>
+          <t>CAND_0041402</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2019,19 +2019,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.5962</t>
+          <t>0.6343</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.2 YoE as Search Engineer, possessing partial overlap in TensorFlow, Information Retrieval, Milvus; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Candidate with 6.3 years experience as AI Specialist, mostly showing adjacent skills like Information Retrieval, RAG, Vector Search; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0087006</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2041,19 +2041,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.5942</t>
+          <t>0.6335</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0017960</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2063,19 +2063,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.594</t>
+          <t>0.6319</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.9 YoE as AI Engineer, mostly showing adjacent skills like Python, Vector Search; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Recommendation Systems Engineer (7.7 YoE), having some background in Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2085,19 +2085,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.5913</t>
+          <t>0.6295</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0087006</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.5893</t>
+          <t>0.6293</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0077067</t>
+          <t>CAND_0001930</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.5883</t>
+          <t>0.629</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.4 YoE as AI Specialist, mostly showing adjacent skills like Python, Pinecone, Vector Search; included as potential pipeline filler.</t>
+          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2151,19 +2151,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.5855</t>
+          <t>0.6217</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.3 YoE as AI Engineer, mostly showing adjacent skills like Pinecone, Vector Search, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Applied ML Engineer with 8.0 years of background, having some background in Vector Search, TensorFlow, Embeddings but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0011125</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2173,19 +2173,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.5851</t>
+          <t>0.619</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, Embeddings, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.0 YoE), mostly showing adjacent skills like Pinecone, Python, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0030953</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2195,19 +2195,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.5843</t>
+          <t>0.617</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 7.8 YoE as Search Engineer, possessing partial overlap in MLOps, Python, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0043860</t>
+          <t>CAND_0041568</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2217,19 +2217,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.5818</t>
+          <t>0.6158</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
+          <t>Search Engineer with 5.2 years of background, having some background in Vector Search, TensorFlow, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
+          <t>CAND_0051486</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2239,19 +2239,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.5818</t>
+          <t>0.6135</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.9 years of background, having some background in Milvus, Vector Search, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>AI Specialist with 5.9 years of background, having some background in Pinecone, Vector Search, TensorFlow but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0074735</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2261,19 +2261,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.5806</t>
+          <t>0.6122</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
+          <t>Applied ML Engineer with 5.5 years of background, with limited direct exposure to search/ranking but lists RAG, Information Retrieval, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0010685</t>
+          <t>CAND_0024466</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2283,19 +2283,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.5802</t>
+          <t>0.6105</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.7 YoE as NLP Engineer, possessing partial overlap in PyTorch, Information Retrieval, RAG; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0061265</t>
+          <t>CAND_0072660</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2305,19 +2305,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.5797</t>
+          <t>0.6081</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 7.1 YoE as Machine Learning Engineer, mostly showing adjacent skills like PyTorch, Information Retrieval, FAISS; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0089498</t>
+          <t>CAND_0044883</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2327,19 +2327,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.5791</t>
+          <t>0.6053</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.8 YoE as AI Specialist, mostly showing adjacent skills like RAG, PyTorch, Python; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0064256</t>
+          <t>CAND_0018722</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.5783</t>
+          <t>0.604</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Python, TensorFlow; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0041568</t>
+          <t>CAND_0025640</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2371,19 +2371,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.578</t>
+          <t>0.6032</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Search Engineer with 5.2 years of background, having some background in Vector Search, TensorFlow, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 5.6 YoE as AI Research Engineer, possessing partial overlap in Information Retrieval, FAISS, PyTorch; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0076163</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2393,19 +2393,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.5775</t>
+          <t>0.6019</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Candidate with 6.8 years experience as AI Engineer, mostly showing adjacent skills like PyTorch, FAISS, NLP; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as NLP Engineer (6.9 YoE), having some background in PyTorch, Python, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0051486</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2415,19 +2415,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.5756</t>
+          <t>0.6014</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>AI Specialist with 5.9 years of background, having some background in Pinecone, Vector Search, TensorFlow but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 8.0 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like Python; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0091899</t>
+          <t>CAND_0089552</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2437,19 +2437,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.5739</t>
+          <t>0.5944</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Senior Software Engineer (ML), possessing partial overlap in FAISS, NLP, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.0 years experience as Machine Learning Engineer, mostly showing adjacent skills like TensorFlow, Vector Search, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0040117</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2459,19 +2459,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.5736</t>
+          <t>0.5927</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.7 YoE as Senior Data Scientist, mostly showing adjacent skills like Embeddings, PyTorch, MLOps; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.5 years experience as Recommendation Systems Engineer, with limited direct exposure to search/ranking but lists Embeddings, RAG, FAISS; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2481,19 +2481,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.5726</t>
+          <t>0.5924</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Candidate with 4.5 years experience as Machine Learning Engineer, mostly showing adjacent skills like MLOps, PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Recommendation Systems Engineer with 8.0 years of background, with limited direct exposure to search/ranking but lists FAISS, Milvus, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0024466</t>
+          <t>CAND_0050707</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2503,19 +2503,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.5712</t>
+          <t>0.5924</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as AI Specialist (5.3 YoE), having some background in RAG, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0092568</t>
+          <t>CAND_0049978</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2525,19 +2525,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.5679</t>
+          <t>0.5889</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Candidate with 5.7 years experience as AI Specialist, possessing partial overlap in Vector Search, Milvus, Python; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Senior Software Engineer (ML) with 6.6 years of background, with limited direct exposure to search/ranking but lists PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0036121</t>
+          <t>CAND_0049771</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2547,19 +2547,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.5677</t>
+          <t>0.5886</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Candidate with 5.2 years experience as ML Engineer, with limited direct exposure to search/ranking but lists Embeddings, Vector Search, Information Retrieval; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), with limited direct exposure to search/ranking but lists Python, PyTorch, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0044883</t>
+          <t>CAND_0008978</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.5658</t>
+          <t>0.5884</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
+          <t>Candidate with 6.7 years experience as Junior ML Engineer, mostly showing adjacent skills like Embeddings, NLP, MLOps; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0092245</t>
+          <t>CAND_0078508</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2591,19 +2591,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.5655</t>
+          <t>0.5875</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Senior Data Scientist (4.1 YoE), mostly showing adjacent skills like Embeddings, RAG, FAISS; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.2 YoE), with limited direct exposure to search/ranking but lists Embeddings, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0095619</t>
+          <t>CAND_0066376</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2613,19 +2613,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.5632</t>
+          <t>0.5854</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.7 YoE), with limited direct exposure to search/ranking but lists NLP, Information Retrieval, FAISS; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0076904</t>
+          <t>CAND_0093331</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2635,12 +2635,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.5621</t>
+          <t>0.5819</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 4.2 years of background, with limited direct exposure to search/ranking but lists Vector Search, NLP, MLOps; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as NLP Engineer (16.1 YoE), having some background in PyTorch, Embeddings, Milvus but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
completed ranking engine with career signals and honeypots
</commit_message>
<xml_diff>
--- a/outputs/mohd_ibadullah.xlsx
+++ b/outputs/mohd_ibadullah.xlsx
@@ -457,7 +457,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.9305</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.9074</t>
+          <t>0.9684</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.8985</t>
+          <t>0.9593</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -513,7 +513,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0008425</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -523,19 +523,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.8627</t>
+          <t>0.9388</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in NLP, TensorFlow, Python and search infrastructure. Highly active on Redrob with a 66% recruiter response rate.</t>
+          <t>Highly relevant Senior AI Engineer with 5.9 years of background, offers solid expertise in FAISS, TensorFlow, NLP which matches the core ranking mandate. Excellent platform engagement with 80% response rate.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -545,19 +545,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.855</t>
+          <t>0.9179</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Highly relevant Senior AI Engineer with 5.9 years of background, offers solid expertise in FAISS, TensorFlow, NLP which matches the core ranking mandate. Excellent platform engagement with 80% response rate.</t>
+          <t>Highly relevant Lead AI Engineer with 6.7 years of background, demonstrates strong proficiency in Information Retrieval, PyTorch, Vector Search and alignment with the JD. Highly active on Redrob with a 73% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0007411</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -567,19 +567,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.8493</t>
+          <t>0.8996</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Top-tier candidate currently working as Senior Machine Learning Engineer (8.0 YoE), offers solid expertise in Vector Search, PyTorch, Information Retrieval which matches the core ranking mandate. Excellent platform engagement with 12% response rate.</t>
+          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in TensorFlow, FAISS, Embeddings and search infrastructure. Available quickly with a short notice period of 15 days.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0008425</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -589,19 +589,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.8286</t>
+          <t>0.8929</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Highly relevant Lead AI Engineer with 6.7 years of background, demonstrates strong proficiency in Information Retrieval, PyTorch, Vector Search and alignment with the JD. Highly active on Redrob with a 73% recruiter response rate.</t>
+          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in NLP, TensorFlow, Python and search infrastructure. Highly active on Redrob with a 66% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0092278</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.814</t>
+          <t>0.8909</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 6.8 years of experience, offers solid expertise in TensorFlow, NLP, Vector Search which matches the core ranking mandate. Highly active on Redrob with a 7% recruiter response rate.</t>
+          <t>Exceptional Senior AI Engineer offering 7.8 years of experience, offers solid expertise in Pinecone, Information Retrieval, Embeddings which matches the core ranking mandate. Highly active on Redrob with a 76% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0011687</t>
+          <t>CAND_0039754</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -633,19 +633,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.8079</t>
+          <t>0.8739</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in TensorFlow, FAISS, Embeddings and search infrastructure. Available quickly with a short notice period of 15 days.</t>
+          <t>Exceptional Senior Applied Scientist offering 16.2 years of experience, offers solid expertise in NLP, Python, TensorFlow which matches the core ranking mandate. Highly active on Redrob with a 81% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -655,19 +655,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.7985</t>
+          <t>0.8728</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Exceptional Senior AI Engineer offering 7.8 years of experience, offers solid expertise in Pinecone, Information Retrieval, Embeddings which matches the core ranking mandate. Highly active on Redrob with a 76% recruiter response rate.</t>
+          <t>Highly relevant Senior NLP Engineer with 8.9 years of background, has successfully deployed systems involving Python, Pinecone at scale. Highly active on Redrob with a 78% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -677,19 +677,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.7978</t>
+          <t>0.8624</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Exceptional Staff Machine Learning Engineer offering 8.6 years of experience, shows deep technical expertise in Pinecone, RAG, TensorFlow and search infrastructure. Highly active on Redrob with a 83% recruiter response rate.</t>
+          <t>Exceptional Senior Machine Learning Engineer offering 6.1 years of experience, demonstrates strong proficiency in Information Retrieval, TensorFlow, NLP and alignment with the JD. Highly active on Redrob with a 88% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -699,19 +699,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.7917</t>
+          <t>0.8605</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Highly relevant Lead AI Engineer with 8.6 years of background, demonstrates strong proficiency in Vector Search, NLP, MLOps and alignment with the JD. Highly active on Redrob with a 11% recruiter response rate.</t>
+          <t>Exceptional Staff Machine Learning Engineer offering 8.6 years of experience, shows deep technical expertise in Pinecone, RAG, TensorFlow and search infrastructure. Highly active on Redrob with a 83% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -721,19 +721,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.7881</t>
+          <t>0.8543</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Exceptional Senior Machine Learning Engineer offering 7.2 years of experience, has successfully deployed systems involving Pinecone, Information Retrieval, Milvus at scale. Highly active on Redrob with a 61% recruiter response rate.</t>
+          <t>Highly relevant Staff Machine Learning Engineer with 7.0 years of background, demonstrates strong proficiency in Pinecone, Information Retrieval, RAG and alignment with the JD. Highly active on Redrob with a 95% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0046064</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -743,19 +743,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.782</t>
+          <t>0.8511</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Highly relevant Senior NLP Engineer with 8.9 years of background, has successfully deployed systems involving Python, Pinecone at scale. Highly active on Redrob with a 78% recruiter response rate.</t>
+          <t>Exceptional Senior Machine Learning Engineer offering 7.2 years of experience, has successfully deployed systems involving Pinecone, Information Retrieval, Milvus at scale. Highly active on Redrob with a 61% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0039754</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -765,19 +765,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.7805</t>
+          <t>0.8433</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Exceptional Senior Applied Scientist offering 16.2 years of experience, offers solid expertise in NLP, Python, TensorFlow which matches the core ranking mandate. Highly active on Redrob with a 81% recruiter response rate.</t>
+          <t>Outstanding candidate as Senior AI Engineer showing 7.9 years of experience, shows deep technical expertise in NLP, Python, Ranking Systems and search infrastructure. Highly active on Redrob with a 79% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0095528</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -787,19 +787,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.7705</t>
+          <t>0.8324</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Strong Senior Machine Learning Engineer with 6.1 years of experience, matching key job requirements like Information Retrieval, TensorFlow, NLP. Good overall behavioral signals.</t>
+          <t>Competent Senior Data Scientist (5.3 YoE), matching key job requirements like PyTorch, Vector Search, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0095528</t>
+          <t>CAND_0033861</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -809,19 +809,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.7678</t>
+          <t>0.8289</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Competent Senior Data Scientist (5.3 YoE), matching key job requirements like PyTorch, Vector Search, Python. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior NLP Engineer with 8.0 years in the field, matching key job requirements like TensorFlow, Pinecone, Vector Search, though platform response rate is lower (16%).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0033861</t>
+          <t>CAND_0007411</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -831,19 +831,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.7671</t>
+          <t>0.8205</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior NLP Engineer with 8.0 years in the field, matching key job requirements like TensorFlow, Pinecone, Vector Search, though platform response rate is lower (16%).</t>
+          <t>Competent Senior Machine Learning Engineer (8.0 YoE), possessing practical experience in Vector Search, PyTorch, Information Retrieval, though platform response rate is lower (12%).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -853,19 +853,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.7614</t>
+          <t>0.7943</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Solid candidate working as Staff Machine Learning Engineer with 7.0 years in the field, matching key job requirements like Pinecone, Information Retrieval, RAG. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (5.7 YoE), who brings relevant experience in Information Retrieval, PyTorch, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0060072</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -875,19 +875,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.7568</t>
+          <t>0.794</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Solid candidate working as Staff Machine Learning Engineer with 5.7 years in the field, matching key job requirements like PyTorch, Milvus, Embeddings, though platform response rate is lower (10%).</t>
+          <t>Solid candidate working as Lead AI Engineer with 8.6 years in the field, matching key job requirements like Vector Search, NLP, MLOps, though platform response rate is lower (11%).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -897,19 +897,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.7501</t>
+          <t>0.7876</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Well-qualified Senior AI Engineer showing 7.9 YoE, who brings relevant experience in NLP, Python, Ranking Systems. Good overall behavioral signals.</t>
+          <t>Competent Applied ML Engineer (14.1 YoE), matching key job requirements like PyTorch, NLP, Embeddings, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -919,19 +919,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.7362</t>
+          <t>0.7766</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 4.9 years in the field, matching key job requirements like Vector Search, Embeddings, Python, slightly below the preferred 5+ years of experience.</t>
+          <t>Competent AI Engineer (16.9 YoE), with matching skills in Information Retrieval, FAISS, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0041611</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -941,19 +941,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.7358</t>
+          <t>0.7583</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Competent Staff Machine Learning Engineer (6.4 YoE), possessing practical experience in PyTorch, NLP, MLOps, though platform response rate is lower (7%).</t>
+          <t>Solid candidate working as Senior AI Engineer with 5.9 years in the field, matching key job requirements like Python, PyTorch, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -963,19 +963,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.7274</t>
+          <t>0.758</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (5.7 YoE), who brings relevant experience in Information Retrieval, PyTorch, Python. Good overall behavioral signals.</t>
+          <t>Strong Lead AI Engineer with 6.4 years of experience, who brings relevant experience in Python, Ranking Systems, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0083307</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -985,19 +985,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.7269</t>
+          <t>0.7402</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Competent Applied ML Engineer (14.1 YoE), matching key job requirements like PyTorch, NLP, Embeddings, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Search Engineer with 7.8 years in the field, matching key job requirements like Embeddings, Pinecone, Python, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1007,19 +1007,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.6978</t>
+          <t>0.7371</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Strong Lead AI Engineer with 6.4 years of experience, who brings relevant experience in Python, Ranking Systems, NLP. Good overall behavioral signals.</t>
+          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0065878</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1029,12 +1029,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.6938</t>
+          <t>0.7339</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior AI Engineer with 5.9 years in the field, matching key job requirements like Python, PyTorch, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.6928</t>
+          <t>0.7306</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1063,7 +1063,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0049896</t>
+          <t>CAND_0032515</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1073,19 +1073,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.6817</t>
+          <t>0.7226</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (7.3 YoE), with matching skills in PyTorch, Information Retrieval, NLP and solid backend fundamentals, note the longer notice period of 90 days.</t>
+          <t>Strong Machine Learning Engineer with 5.1 years of experience, who brings relevant experience in Milvus, Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0036184</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1095,19 +1095,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.6787</t>
+          <t>0.7224</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (16.9 YoE), with matching skills in Information Retrieval, FAISS, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Strong Recommendation Systems Engineer with 6.0 years of experience, matching key job requirements like FAISS, MLOps, Embeddings. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0064904</t>
+          <t>CAND_0064326</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1117,19 +1117,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.6757</t>
+          <t>0.7224</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Strong AI Engineer with 4.9 years of experience, who brings relevant experience in Embeddings, Python, MLOps, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Search Engineer with 7.6 years in the field, matching key job requirements like PyTorch, Milvus, RAG. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0083307</t>
+          <t>CAND_0049896</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1139,19 +1139,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.6735</t>
+          <t>0.7189</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 7.8 years in the field, matching key job requirements like Embeddings, Pinecone, Python, note the longer notice period of 120 days.</t>
+          <t>Competent Search Engineer (7.3 YoE), with matching skills in PyTorch, Information Retrieval, NLP and solid backend fundamentals, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0093912</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1161,19 +1161,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.6696</t>
+          <t>0.7154</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
+          <t>Well-qualified Senior Data Scientist showing 5.3 YoE, who brings relevant experience in Milvus, Embeddings, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0065878</t>
+          <t>CAND_0052682</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1183,19 +1183,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.6679</t>
+          <t>0.7123</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
+          <t>Strong NLP Engineer with 6.6 years of experience, who brings relevant experience in FAISS, PyTorch, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0032515</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.6552</t>
+          <t>0.711</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Strong Machine Learning Engineer with 5.1 years of experience, who brings relevant experience in Milvus, Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Solid candidate working as AI Engineer with 6.7 years in the field, with matching skills in Embeddings, TensorFlow, Information Retrieval and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0093912</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1227,19 +1227,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.6485</t>
+          <t>0.7042</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 5.3 YoE, who brings relevant experience in Milvus, Embeddings, Vector Search. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0077285</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.644</t>
+          <t>0.7002</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0012632</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1271,19 +1271,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.6394</t>
+          <t>0.6915</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Competent AI Specialist (6.0 YoE), possessing practical experience in MLOps, Python, Pinecone, note the longer notice period of 120 days.</t>
+          <t>Solid candidate working as AI Engineer with 6.9 years in the field, matching key job requirements like Python, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0077285</t>
+          <t>CAND_0024620</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1293,19 +1293,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.6364</t>
+          <t>0.6865</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (5.9 YoE), possessing practical experience in Information Retrieval, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1315,19 +1315,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.6311</t>
+          <t>0.6842</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (7.2 YoE), matching key job requirements like Embeddings, Information Retrieval, PyTorch, note the longer notice period of 120 days.</t>
+          <t>Solid candidate working as AI Engineer with 7.3 years in the field, matching key job requirements like Pinecone, Vector Search, RAG. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0039838</t>
+          <t>CAND_0081686</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1337,12 +1337,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.6307</t>
+          <t>0.6831</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Strong Recommendation Systems Engineer with 4.9 years of experience, with matching skills in MLOps, Embeddings, RAG and solid backend fundamentals, note the longer notice period of 90 days.</t>
+          <t>Competent Search Engineer (6.0 YoE), matching key job requirements like Embeddings, FAISS, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.6265</t>
+          <t>0.6818</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1371,7 +1371,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0024620</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1381,19 +1381,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.6264</t>
+          <t>0.6806</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (5.9 YoE), possessing practical experience in Information Retrieval, Python. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Staff Machine Learning Engineer with 8.8 years in the field, matching key job requirements like MLOps, Python, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0064326</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1403,19 +1403,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.6254</t>
+          <t>0.68</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 7.6 years in the field, matching key job requirements like PyTorch, Milvus, RAG. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Data Scientist with 5.7 years in the field, matching key job requirements like TensorFlow, FAISS, RAG, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0051615</t>
+          <t>CAND_0010685</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1425,19 +1425,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.6246</t>
+          <t>0.6782</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (4.6 YoE), matching key job requirements like RAG, Milvus, Vector Search, slightly below the preferred 5+ years of experience.</t>
+          <t>Solid candidate working as NLP Engineer with 6.7 years in the field, with matching skills in PyTorch, Information Retrieval, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0036184</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1447,19 +1447,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.624</t>
+          <t>0.6777</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Strong Recommendation Systems Engineer with 6.0 years of experience, matching key job requirements like FAISS, MLOps, Embeddings. Good overall behavioral signals.</t>
+          <t>Competent Recommendation Systems Engineer (5.8 YoE), matching key job requirements like FAISS, Vector Search, Milvus, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0061175</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.6225</t>
+          <t>0.6769</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Research Engineer with 6.7 years in the field, with matching skills in Python, Milvus, Vector Search and solid backend fundamentals, note the longer notice period of 120 days.</t>
+          <t>Competent AI Engineer (6.8 YoE), matching key job requirements like PyTorch, FAISS, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0099401</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1491,19 +1491,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.6206</t>
+          <t>0.6754</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Strong NLP Engineer with 7.7 years of experience, who brings relevant experience in Embeddings, Information Retrieval, Python, note the longer notice period of 90 days.</t>
+          <t>Strong Applied ML Engineer with 5.2 years of experience, who brings relevant experience in FAISS, Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0070525</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.6193</t>
+          <t>0.6751</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 6.7 years in the field, with matching skills in Embeddings, TensorFlow, Information Retrieval and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Strong Senior Software Engineer (ML) with 5.4 years of experience, who brings relevant experience in Python, Embeddings. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0070202</t>
+          <t>CAND_0096172</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1535,19 +1535,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.6185</t>
+          <t>0.6705</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Competent Machine Learning Engineer (5.1 YoE), matching key job requirements like Embeddings, PyTorch, RAG, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as NLP Engineer with 5.2 years in the field, with matching skills in Python, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0058412</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1557,19 +1557,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.6173</t>
+          <t>0.6698</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.6 YoE as Senior Software Engineer (ML), possessing partial overlap in Embeddings, Milvus, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0081686</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1579,19 +1579,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.6153</t>
+          <t>0.6691</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Candidate with 6.0 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, FAISS, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, mostly showing adjacent skills like Milvus, TensorFlow, Python; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0061339</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1601,19 +1601,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.614</t>
+          <t>0.6689</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Search Engineer (4.2 YoE), mostly showing adjacent skills like Information Retrieval, Milvus, TensorFlow; included as potential pipeline filler.</t>
+          <t>Candidate with 7.2 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, Information Retrieval, PyTorch; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0051630</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1623,19 +1623,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.6139</t>
+          <t>0.6671</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
+          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0006557</t>
+          <t>CAND_0061175</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1645,19 +1645,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.613</t>
+          <t>0.6588</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 6.7 YoE as AI Research Engineer, possessing partial overlap in Python, Milvus, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0052682</t>
+          <t>CAND_0098454</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1667,19 +1667,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.6129</t>
+          <t>0.658</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (6.6 YoE), having some background in FAISS, PyTorch, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0070202</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.6128</t>
+          <t>0.6576</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Alternative profile showing 8.8 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like MLOps, Python, Milvus; included as potential pipeline filler.</t>
+          <t>Candidate with 5.1 years experience as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, PyTorch, RAG; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0099401</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1711,19 +1711,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.6119</t>
+          <t>0.6575</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.9 YoE as Senior Machine Learning Engineer, possessing partial overlap in Ranking Systems, TensorFlow; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0029367</t>
+          <t>CAND_0025882</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1733,19 +1733,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.6103</t>
+          <t>0.6563</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 5.6 YoE as Senior Software Engineer (ML), possessing partial overlap in FAISS, Vector Search, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1755,19 +1755,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.6092</t>
+          <t>0.6559</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1777,19 +1777,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.6081</t>
+          <t>0.6559</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1799,19 +1799,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.6062</t>
+          <t>0.6556</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0000031</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1821,19 +1821,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.6054</t>
+          <t>0.6547</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
+          <t>Recommendation Systems Engineer with 6.0 years of background, possessing partial overlap in FAISS, Pinecone, MLOps; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0096172</t>
+          <t>CAND_0051630</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1843,19 +1843,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.6036</t>
+          <t>0.6529</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.2 YoE as NLP Engineer, possessing partial overlap in Python, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0058412</t>
+          <t>CAND_0012837</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1865,19 +1865,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.6026</t>
+          <t>0.6514</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Senior Software Engineer (ML), possessing partial overlap in Embeddings, Milvus, RAG; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.4 YoE as Junior ML Engineer, mostly showing adjacent skills like Vector Search, MLOps, NLP; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0098454</t>
+          <t>CAND_0006557</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1887,19 +1887,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.6022</t>
+          <t>0.6507</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.6018</t>
+          <t>0.6491</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, mostly showing adjacent skills like Milvus, TensorFlow, Python; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0061265</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1931,19 +1931,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.6018</t>
+          <t>0.6483</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0025971</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1953,19 +1953,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.5987</t>
+          <t>0.6477</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 5.4 years of background, having some background in FAISS, Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0054123</t>
+          <t>CAND_0095619</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1975,19 +1975,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.5981</t>
+          <t>0.6393</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.7 YoE as Applied ML Engineer, mostly showing adjacent skills like Python, Vector Search; included as potential pipeline filler.</t>
+          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0089947</t>
+          <t>CAND_0064256</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1997,19 +1997,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.5979</t>
+          <t>0.6345</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 5.4 years of background, with limited direct exposure to search/ranking but lists Vector Search, Information Retrieval, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0042506</t>
+          <t>CAND_0041402</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2019,19 +2019,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.5962</t>
+          <t>0.6343</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.2 YoE as Search Engineer, possessing partial overlap in TensorFlow, Information Retrieval, Milvus; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Candidate with 6.3 years experience as AI Specialist, mostly showing adjacent skills like Information Retrieval, RAG, Vector Search; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0087006</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2041,19 +2041,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.5942</t>
+          <t>0.6335</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0017960</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2063,19 +2063,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.594</t>
+          <t>0.6319</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.9 YoE as AI Engineer, mostly showing adjacent skills like Python, Vector Search; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Recommendation Systems Engineer (7.7 YoE), having some background in Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2085,19 +2085,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.5913</t>
+          <t>0.6295</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0087006</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.5893</t>
+          <t>0.6293</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0077067</t>
+          <t>CAND_0001930</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.5883</t>
+          <t>0.629</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.4 YoE as AI Specialist, mostly showing adjacent skills like Python, Pinecone, Vector Search; included as potential pipeline filler.</t>
+          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2151,19 +2151,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.5855</t>
+          <t>0.6217</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.3 YoE as AI Engineer, mostly showing adjacent skills like Pinecone, Vector Search, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Applied ML Engineer with 8.0 years of background, having some background in Vector Search, TensorFlow, Embeddings but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0011125</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2173,19 +2173,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.5851</t>
+          <t>0.619</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, Embeddings, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.0 YoE), mostly showing adjacent skills like Pinecone, Python, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0030953</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2195,19 +2195,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.5843</t>
+          <t>0.617</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 7.8 YoE as Search Engineer, possessing partial overlap in MLOps, Python, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0043860</t>
+          <t>CAND_0041568</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2217,19 +2217,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.5818</t>
+          <t>0.6158</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
+          <t>Search Engineer with 5.2 years of background, having some background in Vector Search, TensorFlow, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
+          <t>CAND_0051486</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2239,19 +2239,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.5818</t>
+          <t>0.6135</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.9 years of background, having some background in Milvus, Vector Search, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>AI Specialist with 5.9 years of background, having some background in Pinecone, Vector Search, TensorFlow but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0074735</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2261,19 +2261,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.5806</t>
+          <t>0.6122</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
+          <t>Applied ML Engineer with 5.5 years of background, with limited direct exposure to search/ranking but lists RAG, Information Retrieval, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0010685</t>
+          <t>CAND_0024466</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2283,19 +2283,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.5802</t>
+          <t>0.6105</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.7 YoE as NLP Engineer, possessing partial overlap in PyTorch, Information Retrieval, RAG; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0061265</t>
+          <t>CAND_0072660</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2305,19 +2305,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.5797</t>
+          <t>0.6081</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 7.1 YoE as Machine Learning Engineer, mostly showing adjacent skills like PyTorch, Information Retrieval, FAISS; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0089498</t>
+          <t>CAND_0044883</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2327,19 +2327,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.5791</t>
+          <t>0.6053</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.8 YoE as AI Specialist, mostly showing adjacent skills like RAG, PyTorch, Python; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0064256</t>
+          <t>CAND_0018722</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.5783</t>
+          <t>0.604</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Python, TensorFlow; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0041568</t>
+          <t>CAND_0025640</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2371,19 +2371,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.578</t>
+          <t>0.6032</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Search Engineer with 5.2 years of background, having some background in Vector Search, TensorFlow, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 5.6 YoE as AI Research Engineer, possessing partial overlap in Information Retrieval, FAISS, PyTorch; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0076163</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2393,19 +2393,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.5775</t>
+          <t>0.6019</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Candidate with 6.8 years experience as AI Engineer, mostly showing adjacent skills like PyTorch, FAISS, NLP; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as NLP Engineer (6.9 YoE), having some background in PyTorch, Python, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0051486</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2415,19 +2415,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.5756</t>
+          <t>0.6014</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>AI Specialist with 5.9 years of background, having some background in Pinecone, Vector Search, TensorFlow but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 8.0 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like Python; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0091899</t>
+          <t>CAND_0089552</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2437,19 +2437,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.5739</t>
+          <t>0.5944</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Senior Software Engineer (ML), possessing partial overlap in FAISS, NLP, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.0 years experience as Machine Learning Engineer, mostly showing adjacent skills like TensorFlow, Vector Search, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0040117</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2459,19 +2459,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.5736</t>
+          <t>0.5927</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Alternative profile showing 4.7 YoE as Senior Data Scientist, mostly showing adjacent skills like Embeddings, PyTorch, MLOps; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.5 years experience as Recommendation Systems Engineer, with limited direct exposure to search/ranking but lists Embeddings, RAG, FAISS; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2481,19 +2481,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.5726</t>
+          <t>0.5924</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Candidate with 4.5 years experience as Machine Learning Engineer, mostly showing adjacent skills like MLOps, PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Recommendation Systems Engineer with 8.0 years of background, with limited direct exposure to search/ranking but lists FAISS, Milvus, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0024466</t>
+          <t>CAND_0050707</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2503,19 +2503,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.5712</t>
+          <t>0.5924</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as AI Specialist (5.3 YoE), having some background in RAG, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0092568</t>
+          <t>CAND_0049978</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2525,19 +2525,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.5679</t>
+          <t>0.5889</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Candidate with 5.7 years experience as AI Specialist, possessing partial overlap in Vector Search, Milvus, Python; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Senior Software Engineer (ML) with 6.6 years of background, with limited direct exposure to search/ranking but lists PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0036121</t>
+          <t>CAND_0049771</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2547,19 +2547,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.5677</t>
+          <t>0.5886</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Candidate with 5.2 years experience as ML Engineer, with limited direct exposure to search/ranking but lists Embeddings, Vector Search, Information Retrieval; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), with limited direct exposure to search/ranking but lists Python, PyTorch, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0044883</t>
+          <t>CAND_0008978</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.5658</t>
+          <t>0.5884</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
+          <t>Candidate with 6.7 years experience as Junior ML Engineer, mostly showing adjacent skills like Embeddings, NLP, MLOps; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0092245</t>
+          <t>CAND_0078508</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2591,19 +2591,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.5655</t>
+          <t>0.5875</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Senior Data Scientist (4.1 YoE), mostly showing adjacent skills like Embeddings, RAG, FAISS; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.2 YoE), with limited direct exposure to search/ranking but lists Embeddings, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0095619</t>
+          <t>CAND_0066376</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2613,19 +2613,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.5632</t>
+          <t>0.5854</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.7 YoE), with limited direct exposure to search/ranking but lists NLP, Information Retrieval, FAISS; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0076904</t>
+          <t>CAND_0093331</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2635,12 +2635,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.5621</t>
+          <t>0.5819</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 4.2 years of background, with limited direct exposure to search/ranking but lists Vector Search, NLP, MLOps; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as NLP Engineer (16.1 YoE), having some background in PyTorch, Embeddings, Milvus but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: optimize scoring weights to reduce skill bias, refine consulting-heavy, langchain-only, and inactivity penalties
</commit_message>
<xml_diff>
--- a/outputs/mohd_ibadullah.xlsx
+++ b/outputs/mohd_ibadullah.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.9684</t>
+          <t>0.9617</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.9593</t>
+          <t>0.9568</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -535,7 +535,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -545,19 +545,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.9179</t>
+          <t>0.9221</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Highly relevant Lead AI Engineer with 6.7 years of background, demonstrates strong proficiency in Information Retrieval, PyTorch, Vector Search and alignment with the JD. Highly active on Redrob with a 73% recruiter response rate.</t>
+          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in TensorFlow, FAISS, Embeddings and search infrastructure. Available quickly with a short notice period of 15 days.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0011687</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -567,19 +567,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.8996</t>
+          <t>0.9179</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in TensorFlow, FAISS, Embeddings and search infrastructure. Available quickly with a short notice period of 15 days.</t>
+          <t>Highly relevant Lead AI Engineer with 6.7 years of background, demonstrates strong proficiency in Information Retrieval, PyTorch, Vector Search and alignment with the JD. Highly active on Redrob with a 73% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0008425</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.8929</t>
+          <t>0.9127</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in NLP, TensorFlow, Python and search infrastructure. Highly active on Redrob with a 66% recruiter response rate.</t>
+          <t>Highly relevant Senior NLP Engineer with 8.9 years of background, has successfully deployed systems involving Python, Pinecone at scale. Highly active on Redrob with a 78% recruiter response rate.</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.8909</t>
+          <t>0.9086</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -623,7 +623,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0039754</t>
+          <t>CAND_0008425</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -633,19 +633,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.8739</t>
+          <t>0.9083</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Exceptional Senior Applied Scientist offering 16.2 years of experience, offers solid expertise in NLP, Python, TensorFlow which matches the core ranking mandate. Highly active on Redrob with a 81% recruiter response rate.</t>
+          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in NLP, TensorFlow, Python and search infrastructure. Highly active on Redrob with a 66% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0046064</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -655,19 +655,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.8728</t>
+          <t>0.8949</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Highly relevant Senior NLP Engineer with 8.9 years of background, has successfully deployed systems involving Python, Pinecone at scale. Highly active on Redrob with a 78% recruiter response rate.</t>
+          <t>Exceptional Senior Machine Learning Engineer offering 6.1 years of experience, demonstrates strong proficiency in Information Retrieval, TensorFlow, NLP and alignment with the JD. Highly active on Redrob with a 88% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0039754</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -677,19 +677,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.8624</t>
+          <t>0.8863</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Exceptional Senior Machine Learning Engineer offering 6.1 years of experience, demonstrates strong proficiency in Information Retrieval, TensorFlow, NLP and alignment with the JD. Highly active on Redrob with a 88% recruiter response rate.</t>
+          <t>Exceptional Senior Applied Scientist offering 16.2 years of experience, offers solid expertise in NLP, Python, TensorFlow which matches the core ranking mandate. Highly active on Redrob with a 81% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -699,19 +699,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.8605</t>
+          <t>0.8734</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Exceptional Staff Machine Learning Engineer offering 8.6 years of experience, shows deep technical expertise in Pinecone, RAG, TensorFlow and search infrastructure. Highly active on Redrob with a 83% recruiter response rate.</t>
+          <t>Highly relevant Staff Machine Learning Engineer with 7.0 years of background, demonstrates strong proficiency in Pinecone, Information Retrieval, RAG and alignment with the JD. Highly active on Redrob with a 95% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -721,12 +721,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.8543</t>
+          <t>0.8682</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Highly relevant Staff Machine Learning Engineer with 7.0 years of background, demonstrates strong proficiency in Pinecone, Information Retrieval, RAG and alignment with the JD. Highly active on Redrob with a 95% recruiter response rate.</t>
+          <t>Exceptional Staff Machine Learning Engineer offering 8.6 years of experience, shows deep technical expertise in Pinecone, RAG, TensorFlow and search infrastructure. Highly active on Redrob with a 83% recruiter response rate.</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.8511</t>
+          <t>0.867</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.8433</t>
+          <t>0.8666</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -777,7 +777,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0095528</t>
+          <t>CAND_0033861</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -787,19 +787,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.8324</t>
+          <t>0.8573</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Competent Senior Data Scientist (5.3 YoE), matching key job requirements like PyTorch, Vector Search, Python. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior NLP Engineer with 8.0 years in the field, matching key job requirements like TensorFlow, Pinecone, Vector Search, though platform response rate is lower (16%).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0033861</t>
+          <t>CAND_0095528</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -809,19 +809,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.8289</t>
+          <t>0.8355</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior NLP Engineer with 8.0 years in the field, matching key job requirements like TensorFlow, Pinecone, Vector Search, though platform response rate is lower (16%).</t>
+          <t>Competent Senior Data Scientist (5.3 YoE), matching key job requirements like PyTorch, Vector Search, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0007411</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -831,19 +831,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.8205</t>
+          <t>0.8052</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Competent Senior Machine Learning Engineer (8.0 YoE), possessing practical experience in Vector Search, PyTorch, Information Retrieval, though platform response rate is lower (12%).</t>
+          <t>Solid candidate working as Lead AI Engineer with 8.6 years in the field, matching key job requirements like Vector Search, NLP, MLOps, though platform response rate is lower (11%).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -853,19 +853,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.7943</t>
+          <t>0.7895</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (5.7 YoE), who brings relevant experience in Information Retrieval, PyTorch, Python. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior AI Engineer with 5.9 years in the field, matching key job requirements like Python, PyTorch, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -875,19 +875,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.794</t>
+          <t>0.7865</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Solid candidate working as Lead AI Engineer with 8.6 years in the field, matching key job requirements like Vector Search, NLP, MLOps, though platform response rate is lower (11%).</t>
+          <t>Competent AI Engineer (5.7 YoE), who brings relevant experience in Information Retrieval, PyTorch, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -897,19 +897,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.7876</t>
+          <t>0.7793</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Competent Applied ML Engineer (14.1 YoE), matching key job requirements like PyTorch, NLP, Embeddings, note the longer notice period of 90 days.</t>
+          <t>Competent AI Engineer (16.9 YoE), with matching skills in Information Retrieval, FAISS, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -919,19 +919,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.7766</t>
+          <t>0.7786</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (16.9 YoE), with matching skills in Information Retrieval, FAISS, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Competent Applied ML Engineer (14.1 YoE), matching key job requirements like PyTorch, NLP, Embeddings, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -941,19 +941,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.7583</t>
+          <t>0.7706</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior AI Engineer with 5.9 years in the field, matching key job requirements like Python, PyTorch, note the longer notice period of 90 days.</t>
+          <t>Strong Lead AI Engineer with 6.4 years of experience, who brings relevant experience in Python, Ranking Systems, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0065878</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -963,12 +963,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.758</t>
+          <t>0.7556</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Strong Lead AI Engineer with 6.4 years of experience, who brings relevant experience in Python, Ranking Systems, NLP. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.7402</t>
+          <t>0.752</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -997,7 +997,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0064326</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1007,19 +1007,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.7371</t>
+          <t>0.7494</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Search Engineer with 7.6 years in the field, matching key job requirements like PyTorch, Milvus, RAG. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0065878</t>
+          <t>CAND_0093912</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1029,19 +1029,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.7339</t>
+          <t>0.7421</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
+          <t>Well-qualified Senior Data Scientist showing 5.3 YoE, who brings relevant experience in Milvus, Embeddings, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1051,19 +1051,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.7306</t>
+          <t>0.7379</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Solid candidate working as Machine Learning Engineer with 7.2 years in the field, matching key job requirements like RAG, FAISS, Embeddings, note the longer notice period of 120 days.</t>
+          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0032515</t>
+          <t>CAND_0036184</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1073,19 +1073,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.7226</t>
+          <t>0.7328</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Strong Machine Learning Engineer with 5.1 years of experience, who brings relevant experience in Milvus, Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Strong Recommendation Systems Engineer with 6.0 years of experience, matching key job requirements like FAISS, MLOps, Embeddings. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0036184</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1095,19 +1095,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.7224</t>
+          <t>0.7288</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Strong Recommendation Systems Engineer with 6.0 years of experience, matching key job requirements like FAISS, MLOps, Embeddings. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0064326</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1117,19 +1117,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.7224</t>
+          <t>0.7286</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 7.6 years in the field, matching key job requirements like PyTorch, Milvus, RAG. Good overall behavioral signals.</t>
+          <t>Solid candidate working as AI Engineer with 6.7 years in the field, with matching skills in Embeddings, TensorFlow, Information Retrieval and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0049896</t>
+          <t>CAND_0032515</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1139,19 +1139,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.7189</t>
+          <t>0.727</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (7.3 YoE), with matching skills in PyTorch, Information Retrieval, NLP and solid backend fundamentals, note the longer notice period of 90 days.</t>
+          <t>Strong Machine Learning Engineer with 5.1 years of experience, who brings relevant experience in Milvus, Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0093912</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1161,19 +1161,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.7154</t>
+          <t>0.7221</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 5.3 YoE, who brings relevant experience in Milvus, Embeddings, Vector Search. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Machine Learning Engineer with 7.2 years in the field, matching key job requirements like RAG, FAISS, Embeddings, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0052682</t>
+          <t>CAND_0049896</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1183,19 +1183,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.7123</t>
+          <t>0.7215</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Strong NLP Engineer with 6.6 years of experience, who brings relevant experience in FAISS, PyTorch, Python. Good overall behavioral signals.</t>
+          <t>Competent Search Engineer (7.3 YoE), with matching skills in PyTorch, Information Retrieval, NLP and solid backend fundamentals, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.711</t>
+          <t>0.7213</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 6.7 years in the field, with matching skills in Embeddings, TensorFlow, Information Retrieval and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Solid candidate working as AI Engineer with 6.9 years in the field, matching key job requirements like Python, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0024620</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1227,19 +1227,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.7042</t>
+          <t>0.7176</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (5.9 YoE), possessing practical experience in Information Retrieval, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0077285</t>
+          <t>CAND_0052682</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.7002</t>
+          <t>0.7165</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
+          <t>Strong NLP Engineer with 6.6 years of experience, who brings relevant experience in FAISS, PyTorch, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0070525</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1271,19 +1271,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.6915</t>
+          <t>0.7123</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 6.9 years in the field, matching key job requirements like Python, Vector Search. Good overall behavioral signals.</t>
+          <t>Strong Senior Software Engineer (ML) with 5.4 years of experience, who brings relevant experience in Python, Embeddings. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0024620</t>
+          <t>CAND_0010685</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.6865</t>
+          <t>0.7084</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (5.9 YoE), possessing practical experience in Information Retrieval, Python. Good overall behavioral signals.</t>
+          <t>Solid candidate working as NLP Engineer with 6.7 years in the field, with matching skills in PyTorch, Information Retrieval, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.6842</t>
+          <t>0.7069</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0081686</t>
+          <t>CAND_0030468</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1337,19 +1337,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.6831</t>
+          <t>0.7037</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (6.0 YoE), matching key job requirements like Embeddings, FAISS, Milvus. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Applied Scientist with 5.4 years in the field, matching key job requirements like TensorFlow, Ranking Systems, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0030468</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1359,19 +1359,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.6818</t>
+          <t>0.7003</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Applied Scientist with 5.4 years in the field, matching key job requirements like TensorFlow, Ranking Systems, Milvus. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Data Scientist with 6.5 years in the field, matching key job requirements like Milvus, TensorFlow, Python, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0081686</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1381,19 +1381,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.6806</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Solid candidate working as Staff Machine Learning Engineer with 8.8 years in the field, matching key job requirements like MLOps, Python, Milvus. Good overall behavioral signals.</t>
+          <t>Competent Search Engineer (6.0 YoE), matching key job requirements like Embeddings, FAISS, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0029367</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1403,19 +1403,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>0.6997</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 5.7 years in the field, matching key job requirements like TensorFlow, FAISS, RAG, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Staff Machine Learning Engineer with 8.8 years in the field, matching key job requirements like MLOps, Python, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0010685</t>
+          <t>CAND_0096172</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1425,19 +1425,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.6782</t>
+          <t>0.6963</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Solid candidate working as NLP Engineer with 6.7 years in the field, with matching skills in PyTorch, Information Retrieval, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Solid candidate working as NLP Engineer with 5.2 years in the field, with matching skills in Python, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0058412</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1447,19 +1447,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.6777</t>
+          <t>0.6949</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Competent Recommendation Systems Engineer (5.8 YoE), matching key job requirements like FAISS, Vector Search, Milvus, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Senior Software Engineer (ML) with 6.6 years in the field, with matching skills in Embeddings, Milvus, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0025882</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.6769</t>
+          <t>0.6942</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (6.8 YoE), matching key job requirements like PyTorch, FAISS, NLP. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Software Engineer (ML) with 5.6 years in the field, with matching skills in FAISS, Vector Search, Milvus and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1491,19 +1491,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.6754</t>
+          <t>0.6939</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Strong Applied ML Engineer with 5.2 years of experience, who brings relevant experience in FAISS, Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (6.8 YoE), matching key job requirements like PyTorch, FAISS, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0070525</t>
+          <t>CAND_0077285</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.6751</t>
+          <t>0.6911</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Strong Senior Software Engineer (ML) with 5.4 years of experience, who brings relevant experience in Python, Embeddings. Good overall behavioral signals.</t>
+          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0096172</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1535,19 +1535,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.6705</t>
+          <t>0.6896</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Solid candidate working as NLP Engineer with 5.2 years in the field, with matching skills in Python, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Competent Applied ML Engineer (5.8 YoE), matching key job requirements like Vector Search, Milvus, Embeddings. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0058412</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1557,19 +1557,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.6698</t>
+          <t>0.6888</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Senior Software Engineer (ML), possessing partial overlap in Embeddings, Milvus, RAG; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1579,19 +1579,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.6691</t>
+          <t>0.6848</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, mostly showing adjacent skills like Milvus, TensorFlow, Python; included as potential pipeline filler.</t>
+          <t>Candidate with 7.2 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, Information Retrieval, PyTorch; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1601,19 +1601,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.6689</t>
+          <t>0.6825</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Candidate with 7.2 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, Information Retrieval, PyTorch; moderate fit with some technical gaps for this senior role.</t>
+          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1623,19 +1623,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.6671</t>
+          <t>0.6815</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0061175</t>
+          <t>CAND_0098454</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1645,19 +1645,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.6588</t>
+          <t>0.681</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.7 YoE as AI Research Engineer, possessing partial overlap in Python, Milvus, Vector Search; included as potential pipeline filler.</t>
+          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0098454</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1667,19 +1667,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.658</t>
+          <t>0.6801</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0070202</t>
+          <t>CAND_0012837</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.6576</t>
+          <t>0.6793</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Candidate with 5.1 years experience as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, PyTorch, RAG; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 6.4 YoE as Junior ML Engineer, mostly showing adjacent skills like Vector Search, MLOps, NLP; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0099401</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1711,19 +1711,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.6575</t>
+          <t>0.679</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0025882</t>
+          <t>CAND_0099401</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1733,19 +1733,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.6563</t>
+          <t>0.6777</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.6 YoE as Senior Software Engineer (ML), possessing partial overlap in FAISS, Vector Search, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1755,19 +1755,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.6559</t>
+          <t>0.675</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0061265</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1777,19 +1777,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.6559</t>
+          <t>0.6748</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0043860</t>
+          <t>CAND_0006557</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1799,12 +1799,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.6556</t>
+          <t>0.6714</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.6547</t>
+          <t>0.6703</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1833,7 +1833,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0051630</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1843,19 +1843,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.6529</t>
+          <t>0.6693</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
+          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0012837</t>
+          <t>CAND_0041402</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1865,19 +1865,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.6514</t>
+          <t>0.6666</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.4 YoE as Junior ML Engineer, mostly showing adjacent skills like Vector Search, MLOps, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 6.3 years experience as AI Specialist, mostly showing adjacent skills like Information Retrieval, RAG, Vector Search; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0006557</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1887,19 +1887,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.6507</t>
+          <t>0.665</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0017960</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.6491</t>
+          <t>0.6646</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Recommendation Systems Engineer (7.7 YoE), having some background in Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0061265</t>
+          <t>CAND_0064256</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1931,19 +1931,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.6483</t>
+          <t>0.6623</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0070202</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1953,19 +1953,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.6477</t>
+          <t>0.6615</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 5.1 years experience as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, PyTorch, RAG; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0095619</t>
+          <t>CAND_0001930</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1975,19 +1975,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.6393</t>
+          <t>0.6561</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0064256</t>
+          <t>CAND_0051630</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1997,19 +1997,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.6345</t>
+          <t>0.6558</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0041402</t>
+          <t>CAND_0095619</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2019,12 +2019,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.6343</t>
+          <t>0.654</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Candidate with 6.3 years experience as AI Specialist, mostly showing adjacent skills like Information Retrieval, RAG, Vector Search; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.6335</t>
+          <t>0.6531</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2053,7 +2053,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0017960</t>
+          <t>CAND_0030953</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2063,19 +2063,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.6319</t>
+          <t>0.6512</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Recommendation Systems Engineer (7.7 YoE), having some background in Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 7.8 YoE as Search Engineer, possessing partial overlap in MLOps, Python, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0041568</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2085,12 +2085,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.6295</t>
+          <t>0.6499</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Search Engineer with 5.2 years of background, having some background in Vector Search, TensorFlow, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.6293</t>
+          <t>0.6473</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2119,7 +2119,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0015967</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.629</t>
+          <t>0.6431</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Senior Software Engineer (ML) (5.4 YoE), with limited direct exposure to search/ranking but lists Pinecone, TensorFlow, Embeddings; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
+          <t>CAND_0018722</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2151,19 +2151,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.6217</t>
+          <t>0.6418</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 8.0 years of background, having some background in Vector Search, TensorFlow, Embeddings but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Python, TensorFlow; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2173,19 +2173,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.619</t>
+          <t>0.6404</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.0 YoE), mostly showing adjacent skills like Pinecone, Python, RAG; included as potential pipeline filler.</t>
+          <t>Applied ML Engineer with 8.0 years of background, having some background in Vector Search, TensorFlow, Embeddings but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0030953</t>
+          <t>CAND_0076163</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2195,19 +2195,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.617</t>
+          <t>0.6381</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.8 YoE as Search Engineer, possessing partial overlap in MLOps, Python, RAG; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as NLP Engineer (6.9 YoE), having some background in PyTorch, Python, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0041568</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2217,19 +2217,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.6158</t>
+          <t>0.6362</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Search Engineer with 5.2 years of background, having some background in Vector Search, TensorFlow, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.0 YoE), mostly showing adjacent skills like Pinecone, Python, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0051486</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2239,19 +2239,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.6135</t>
+          <t>0.6354</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>AI Specialist with 5.9 years of background, having some background in Pinecone, Vector Search, TensorFlow but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 8.0 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like Python; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0074735</t>
+          <t>CAND_0067866</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2261,19 +2261,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.6122</t>
+          <t>0.6342</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 5.5 years of background, with limited direct exposure to search/ranking but lists RAG, Information Retrieval, Vector Search; included as potential pipeline filler.</t>
+          <t>Senior Software Engineer (ML) with 6.4 years of background, possessing partial overlap in Embeddings; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0024466</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2283,19 +2283,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.6105</t>
+          <t>0.6339</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0072660</t>
+          <t>CAND_0049978</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2305,19 +2305,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.6081</t>
+          <t>0.6296</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.1 YoE as Machine Learning Engineer, mostly showing adjacent skills like PyTorch, Information Retrieval, FAISS; moderate fit with some technical gaps for this senior role.</t>
+          <t>Senior Software Engineer (ML) with 6.6 years of background, with limited direct exposure to search/ranking but lists PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0044883</t>
+          <t>CAND_0024466</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2327,19 +2327,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.6053</t>
+          <t>0.6289</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0018722</t>
+          <t>CAND_0074735</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.604</t>
+          <t>0.6287</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Python, TensorFlow; included as potential pipeline filler.</t>
+          <t>Applied ML Engineer with 5.5 years of background, with limited direct exposure to search/ranking but lists RAG, Information Retrieval, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0025640</t>
+          <t>CAND_0044883</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2371,19 +2371,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.6032</t>
+          <t>0.626</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.6 YoE as AI Research Engineer, possessing partial overlap in Information Retrieval, FAISS, PyTorch; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0076163</t>
+          <t>CAND_0040117</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2393,19 +2393,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.6019</t>
+          <t>0.6231</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (6.9 YoE), having some background in PyTorch, Python, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.5 years experience as Recommendation Systems Engineer, with limited direct exposure to search/ranking but lists Embeddings, RAG, FAISS; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2415,19 +2415,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.6014</t>
+          <t>0.6213</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Alternative profile showing 8.0 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like Python; moderate fit with some technical gaps for this senior role.</t>
+          <t>Recommendation Systems Engineer with 8.0 years of background, with limited direct exposure to search/ranking but lists FAISS, Milvus, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0089552</t>
+          <t>CAND_0049771</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2437,19 +2437,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.5944</t>
+          <t>0.6192</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Candidate with 6.0 years experience as Machine Learning Engineer, mostly showing adjacent skills like TensorFlow, Vector Search, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), with limited direct exposure to search/ranking but lists Python, PyTorch, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0040117</t>
+          <t>CAND_0053605</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2459,19 +2459,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.5927</t>
+          <t>0.6185</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Candidate with 6.5 years experience as Recommendation Systems Engineer, with limited direct exposure to search/ranking but lists Embeddings, RAG, FAISS; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Senior Software Engineer (ML) (6.9 YoE), having some background in RAG but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
+          <t>CAND_0093331</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2481,19 +2481,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.5924</t>
+          <t>0.6147</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 8.0 years of background, with limited direct exposure to search/ranking but lists FAISS, Milvus, MLOps; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as NLP Engineer (16.1 YoE), having some background in PyTorch, Embeddings, Milvus but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0050707</t>
+          <t>CAND_0082086</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2503,19 +2503,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.5924</t>
+          <t>0.6145</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Specialist (5.3 YoE), having some background in RAG, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Senior Software Engineer (ML) with 6.0 years of background, having some background in FAISS, Pinecone, PyTorch but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0049978</t>
+          <t>CAND_0078508</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2525,19 +2525,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.5889</t>
+          <t>0.6134</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.6 years of background, with limited direct exposure to search/ranking but lists PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.2 YoE), with limited direct exposure to search/ranking but lists Embeddings, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0049771</t>
+          <t>CAND_0072660</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2547,19 +2547,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.5886</t>
+          <t>0.6133</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), with limited direct exposure to search/ranking but lists Python, PyTorch, MLOps; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 7.1 YoE as Machine Learning Engineer, mostly showing adjacent skills like PyTorch, Information Retrieval, FAISS; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0008978</t>
+          <t>CAND_0050707</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.5884</t>
+          <t>0.6129</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Candidate with 6.7 years experience as Junior ML Engineer, mostly showing adjacent skills like Embeddings, NLP, MLOps; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as AI Specialist (5.3 YoE), having some background in RAG, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0078508</t>
+          <t>CAND_0093883</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2591,19 +2591,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.5875</t>
+          <t>0.6121</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.2 YoE), with limited direct exposure to search/ranking but lists Embeddings, NLP; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), possessing partial overlap in Embeddings, MLOps, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0066376</t>
+          <t>CAND_0089552</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2613,19 +2613,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.5854</t>
+          <t>0.6116</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.7 YoE), with limited direct exposure to search/ranking but lists NLP, Information Retrieval, FAISS; included as potential pipeline filler.</t>
+          <t>Candidate with 6.0 years experience as Machine Learning Engineer, mostly showing adjacent skills like TensorFlow, Vector Search, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0093331</t>
+          <t>CAND_0010770</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2635,12 +2635,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.5819</t>
+          <t>0.6081</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (16.1 YoE), having some background in PyTorch, Embeddings, Milvus but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 15.2 YoE as Recommendation Systems Engineer, mostly showing adjacent skills like TensorFlow, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
optimized scoring weights to reduce skill bias
</commit_message>
<xml_diff>
--- a/outputs/mohd_ibadullah.xlsx
+++ b/outputs/mohd_ibadullah.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.9684</t>
+          <t>0.9617</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.9593</t>
+          <t>0.9568</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -535,7 +535,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -545,19 +545,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.9179</t>
+          <t>0.9221</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Highly relevant Lead AI Engineer with 6.7 years of background, demonstrates strong proficiency in Information Retrieval, PyTorch, Vector Search and alignment with the JD. Highly active on Redrob with a 73% recruiter response rate.</t>
+          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in TensorFlow, FAISS, Embeddings and search infrastructure. Available quickly with a short notice period of 15 days.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0011687</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -567,19 +567,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.8996</t>
+          <t>0.9179</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in TensorFlow, FAISS, Embeddings and search infrastructure. Available quickly with a short notice period of 15 days.</t>
+          <t>Highly relevant Lead AI Engineer with 6.7 years of background, demonstrates strong proficiency in Information Retrieval, PyTorch, Vector Search and alignment with the JD. Highly active on Redrob with a 73% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0008425</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.8929</t>
+          <t>0.9127</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in NLP, TensorFlow, Python and search infrastructure. Highly active on Redrob with a 66% recruiter response rate.</t>
+          <t>Highly relevant Senior NLP Engineer with 8.9 years of background, has successfully deployed systems involving Python, Pinecone at scale. Highly active on Redrob with a 78% recruiter response rate.</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.8909</t>
+          <t>0.9086</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -623,7 +623,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0039754</t>
+          <t>CAND_0008425</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -633,19 +633,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.8739</t>
+          <t>0.9083</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Exceptional Senior Applied Scientist offering 16.2 years of experience, offers solid expertise in NLP, Python, TensorFlow which matches the core ranking mandate. Highly active on Redrob with a 81% recruiter response rate.</t>
+          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in NLP, TensorFlow, Python and search infrastructure. Highly active on Redrob with a 66% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0046064</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -655,19 +655,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.8728</t>
+          <t>0.8949</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Highly relevant Senior NLP Engineer with 8.9 years of background, has successfully deployed systems involving Python, Pinecone at scale. Highly active on Redrob with a 78% recruiter response rate.</t>
+          <t>Exceptional Senior Machine Learning Engineer offering 6.1 years of experience, demonstrates strong proficiency in Information Retrieval, TensorFlow, NLP and alignment with the JD. Highly active on Redrob with a 88% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0039754</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -677,19 +677,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.8624</t>
+          <t>0.8863</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Exceptional Senior Machine Learning Engineer offering 6.1 years of experience, demonstrates strong proficiency in Information Retrieval, TensorFlow, NLP and alignment with the JD. Highly active on Redrob with a 88% recruiter response rate.</t>
+          <t>Exceptional Senior Applied Scientist offering 16.2 years of experience, offers solid expertise in NLP, Python, TensorFlow which matches the core ranking mandate. Highly active on Redrob with a 81% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -699,19 +699,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.8605</t>
+          <t>0.8734</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Exceptional Staff Machine Learning Engineer offering 8.6 years of experience, shows deep technical expertise in Pinecone, RAG, TensorFlow and search infrastructure. Highly active on Redrob with a 83% recruiter response rate.</t>
+          <t>Highly relevant Staff Machine Learning Engineer with 7.0 years of background, demonstrates strong proficiency in Pinecone, Information Retrieval, RAG and alignment with the JD. Highly active on Redrob with a 95% recruiter response rate.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -721,12 +721,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.8543</t>
+          <t>0.8682</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Highly relevant Staff Machine Learning Engineer with 7.0 years of background, demonstrates strong proficiency in Pinecone, Information Retrieval, RAG and alignment with the JD. Highly active on Redrob with a 95% recruiter response rate.</t>
+          <t>Exceptional Staff Machine Learning Engineer offering 8.6 years of experience, shows deep technical expertise in Pinecone, RAG, TensorFlow and search infrastructure. Highly active on Redrob with a 83% recruiter response rate.</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.8511</t>
+          <t>0.867</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.8433</t>
+          <t>0.8666</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -777,7 +777,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0095528</t>
+          <t>CAND_0033861</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -787,19 +787,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.8324</t>
+          <t>0.8573</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Competent Senior Data Scientist (5.3 YoE), matching key job requirements like PyTorch, Vector Search, Python. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior NLP Engineer with 8.0 years in the field, matching key job requirements like TensorFlow, Pinecone, Vector Search, though platform response rate is lower (16%).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0033861</t>
+          <t>CAND_0095528</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -809,19 +809,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.8289</t>
+          <t>0.8355</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior NLP Engineer with 8.0 years in the field, matching key job requirements like TensorFlow, Pinecone, Vector Search, though platform response rate is lower (16%).</t>
+          <t>Competent Senior Data Scientist (5.3 YoE), matching key job requirements like PyTorch, Vector Search, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0007411</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -831,19 +831,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.8205</t>
+          <t>0.8052</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Competent Senior Machine Learning Engineer (8.0 YoE), possessing practical experience in Vector Search, PyTorch, Information Retrieval, though platform response rate is lower (12%).</t>
+          <t>Solid candidate working as Lead AI Engineer with 8.6 years in the field, matching key job requirements like Vector Search, NLP, MLOps, though platform response rate is lower (11%).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -853,19 +853,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.7943</t>
+          <t>0.7895</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (5.7 YoE), who brings relevant experience in Information Retrieval, PyTorch, Python. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior AI Engineer with 5.9 years in the field, matching key job requirements like Python, PyTorch, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -875,19 +875,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.794</t>
+          <t>0.7865</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Solid candidate working as Lead AI Engineer with 8.6 years in the field, matching key job requirements like Vector Search, NLP, MLOps, though platform response rate is lower (11%).</t>
+          <t>Competent AI Engineer (5.7 YoE), who brings relevant experience in Information Retrieval, PyTorch, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -897,19 +897,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.7876</t>
+          <t>0.7793</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Competent Applied ML Engineer (14.1 YoE), matching key job requirements like PyTorch, NLP, Embeddings, note the longer notice period of 90 days.</t>
+          <t>Competent AI Engineer (16.9 YoE), with matching skills in Information Retrieval, FAISS, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -919,19 +919,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.7766</t>
+          <t>0.7786</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (16.9 YoE), with matching skills in Information Retrieval, FAISS, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Competent Applied ML Engineer (14.1 YoE), matching key job requirements like PyTorch, NLP, Embeddings, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -941,19 +941,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.7583</t>
+          <t>0.7706</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior AI Engineer with 5.9 years in the field, matching key job requirements like Python, PyTorch, note the longer notice period of 90 days.</t>
+          <t>Strong Lead AI Engineer with 6.4 years of experience, who brings relevant experience in Python, Ranking Systems, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0065878</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -963,12 +963,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.758</t>
+          <t>0.7556</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Strong Lead AI Engineer with 6.4 years of experience, who brings relevant experience in Python, Ranking Systems, NLP. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.7402</t>
+          <t>0.752</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -997,7 +997,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0064326</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1007,19 +1007,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.7371</t>
+          <t>0.7494</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Search Engineer with 7.6 years in the field, matching key job requirements like PyTorch, Milvus, RAG. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0065878</t>
+          <t>CAND_0093912</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1029,19 +1029,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.7339</t>
+          <t>0.7421</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
+          <t>Well-qualified Senior Data Scientist showing 5.3 YoE, who brings relevant experience in Milvus, Embeddings, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1051,19 +1051,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.7306</t>
+          <t>0.7379</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Solid candidate working as Machine Learning Engineer with 7.2 years in the field, matching key job requirements like RAG, FAISS, Embeddings, note the longer notice period of 120 days.</t>
+          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0032515</t>
+          <t>CAND_0036184</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1073,19 +1073,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.7226</t>
+          <t>0.7328</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Strong Machine Learning Engineer with 5.1 years of experience, who brings relevant experience in Milvus, Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Strong Recommendation Systems Engineer with 6.0 years of experience, matching key job requirements like FAISS, MLOps, Embeddings. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0036184</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1095,19 +1095,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.7224</t>
+          <t>0.7288</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Strong Recommendation Systems Engineer with 6.0 years of experience, matching key job requirements like FAISS, MLOps, Embeddings. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0064326</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1117,19 +1117,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.7224</t>
+          <t>0.7286</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 7.6 years in the field, matching key job requirements like PyTorch, Milvus, RAG. Good overall behavioral signals.</t>
+          <t>Solid candidate working as AI Engineer with 6.7 years in the field, with matching skills in Embeddings, TensorFlow, Information Retrieval and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0049896</t>
+          <t>CAND_0032515</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1139,19 +1139,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.7189</t>
+          <t>0.727</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (7.3 YoE), with matching skills in PyTorch, Information Retrieval, NLP and solid backend fundamentals, note the longer notice period of 90 days.</t>
+          <t>Strong Machine Learning Engineer with 5.1 years of experience, who brings relevant experience in Milvus, Vector Search, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0093912</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1161,19 +1161,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.7154</t>
+          <t>0.7221</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 5.3 YoE, who brings relevant experience in Milvus, Embeddings, Vector Search. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Machine Learning Engineer with 7.2 years in the field, matching key job requirements like RAG, FAISS, Embeddings, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0052682</t>
+          <t>CAND_0049896</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1183,19 +1183,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.7123</t>
+          <t>0.7215</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Strong NLP Engineer with 6.6 years of experience, who brings relevant experience in FAISS, PyTorch, Python. Good overall behavioral signals.</t>
+          <t>Competent Search Engineer (7.3 YoE), with matching skills in PyTorch, Information Retrieval, NLP and solid backend fundamentals, note the longer notice period of 90 days.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.711</t>
+          <t>0.7213</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 6.7 years in the field, with matching skills in Embeddings, TensorFlow, Information Retrieval and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Solid candidate working as AI Engineer with 6.9 years in the field, matching key job requirements like Python, Vector Search. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0024620</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1227,19 +1227,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.7042</t>
+          <t>0.7176</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (5.9 YoE), possessing practical experience in Information Retrieval, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0077285</t>
+          <t>CAND_0052682</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.7002</t>
+          <t>0.7165</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
+          <t>Strong NLP Engineer with 6.6 years of experience, who brings relevant experience in FAISS, PyTorch, Python. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0070525</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1271,19 +1271,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.6915</t>
+          <t>0.7123</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 6.9 years in the field, matching key job requirements like Python, Vector Search. Good overall behavioral signals.</t>
+          <t>Strong Senior Software Engineer (ML) with 5.4 years of experience, who brings relevant experience in Python, Embeddings. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0024620</t>
+          <t>CAND_0010685</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.6865</t>
+          <t>0.7084</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (5.9 YoE), possessing practical experience in Information Retrieval, Python. Good overall behavioral signals.</t>
+          <t>Solid candidate working as NLP Engineer with 6.7 years in the field, with matching skills in PyTorch, Information Retrieval, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.6842</t>
+          <t>0.7069</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0081686</t>
+          <t>CAND_0030468</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1337,19 +1337,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.6831</t>
+          <t>0.7037</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (6.0 YoE), matching key job requirements like Embeddings, FAISS, Milvus. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Applied Scientist with 5.4 years in the field, matching key job requirements like TensorFlow, Ranking Systems, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0030468</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1359,19 +1359,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.6818</t>
+          <t>0.7003</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Applied Scientist with 5.4 years in the field, matching key job requirements like TensorFlow, Ranking Systems, Milvus. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Data Scientist with 6.5 years in the field, matching key job requirements like Milvus, TensorFlow, Python, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0081686</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1381,19 +1381,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.6806</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Solid candidate working as Staff Machine Learning Engineer with 8.8 years in the field, matching key job requirements like MLOps, Python, Milvus. Good overall behavioral signals.</t>
+          <t>Competent Search Engineer (6.0 YoE), matching key job requirements like Embeddings, FAISS, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0029367</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1403,19 +1403,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>0.6997</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 5.7 years in the field, matching key job requirements like TensorFlow, FAISS, RAG, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Staff Machine Learning Engineer with 8.8 years in the field, matching key job requirements like MLOps, Python, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0010685</t>
+          <t>CAND_0096172</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1425,19 +1425,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.6782</t>
+          <t>0.6963</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Solid candidate working as NLP Engineer with 6.7 years in the field, with matching skills in PyTorch, Information Retrieval, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Solid candidate working as NLP Engineer with 5.2 years in the field, with matching skills in Python, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0058412</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1447,19 +1447,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.6777</t>
+          <t>0.6949</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Competent Recommendation Systems Engineer (5.8 YoE), matching key job requirements like FAISS, Vector Search, Milvus, note the longer notice period of 90 days.</t>
+          <t>Solid candidate working as Senior Software Engineer (ML) with 6.6 years in the field, with matching skills in Embeddings, Milvus, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0025882</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.6769</t>
+          <t>0.6942</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (6.8 YoE), matching key job requirements like PyTorch, FAISS, NLP. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Software Engineer (ML) with 5.6 years in the field, with matching skills in FAISS, Vector Search, Milvus and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1491,19 +1491,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.6754</t>
+          <t>0.6939</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Strong Applied ML Engineer with 5.2 years of experience, who brings relevant experience in FAISS, Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (6.8 YoE), matching key job requirements like PyTorch, FAISS, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0070525</t>
+          <t>CAND_0077285</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.6751</t>
+          <t>0.6911</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Strong Senior Software Engineer (ML) with 5.4 years of experience, who brings relevant experience in Python, Embeddings. Good overall behavioral signals.</t>
+          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0096172</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1535,19 +1535,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.6705</t>
+          <t>0.6896</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Solid candidate working as NLP Engineer with 5.2 years in the field, with matching skills in Python, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Competent Applied ML Engineer (5.8 YoE), matching key job requirements like Vector Search, Milvus, Embeddings. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0058412</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1557,19 +1557,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.6698</t>
+          <t>0.6888</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Senior Software Engineer (ML), possessing partial overlap in Embeddings, Milvus, RAG; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1579,19 +1579,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.6691</t>
+          <t>0.6848</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, mostly showing adjacent skills like Milvus, TensorFlow, Python; included as potential pipeline filler.</t>
+          <t>Candidate with 7.2 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, Information Retrieval, PyTorch; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1601,19 +1601,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.6689</t>
+          <t>0.6825</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Candidate with 7.2 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, Information Retrieval, PyTorch; moderate fit with some technical gaps for this senior role.</t>
+          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1623,19 +1623,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.6671</t>
+          <t>0.6815</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0061175</t>
+          <t>CAND_0098454</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1645,19 +1645,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.6588</t>
+          <t>0.681</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.7 YoE as AI Research Engineer, possessing partial overlap in Python, Milvus, Vector Search; included as potential pipeline filler.</t>
+          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0098454</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1667,19 +1667,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.658</t>
+          <t>0.6801</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0070202</t>
+          <t>CAND_0012837</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.6576</t>
+          <t>0.6793</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Candidate with 5.1 years experience as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, PyTorch, RAG; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 6.4 YoE as Junior ML Engineer, mostly showing adjacent skills like Vector Search, MLOps, NLP; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0099401</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1711,19 +1711,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.6575</t>
+          <t>0.679</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0025882</t>
+          <t>CAND_0099401</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1733,19 +1733,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.6563</t>
+          <t>0.6777</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.6 YoE as Senior Software Engineer (ML), possessing partial overlap in FAISS, Vector Search, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1755,19 +1755,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.6559</t>
+          <t>0.675</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0061265</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1777,19 +1777,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.6559</t>
+          <t>0.6748</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0043860</t>
+          <t>CAND_0006557</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1799,12 +1799,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.6556</t>
+          <t>0.6714</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.6547</t>
+          <t>0.6703</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1833,7 +1833,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0051630</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1843,19 +1843,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.6529</t>
+          <t>0.6693</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
+          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0012837</t>
+          <t>CAND_0041402</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1865,19 +1865,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.6514</t>
+          <t>0.6666</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.4 YoE as Junior ML Engineer, mostly showing adjacent skills like Vector Search, MLOps, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 6.3 years experience as AI Specialist, mostly showing adjacent skills like Information Retrieval, RAG, Vector Search; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0006557</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1887,19 +1887,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.6507</t>
+          <t>0.665</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0017960</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.6491</t>
+          <t>0.6646</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Recommendation Systems Engineer (7.7 YoE), having some background in Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0061265</t>
+          <t>CAND_0064256</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1931,19 +1931,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.6483</t>
+          <t>0.6623</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0070202</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1953,19 +1953,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.6477</t>
+          <t>0.6615</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 5.1 years experience as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, PyTorch, RAG; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0095619</t>
+          <t>CAND_0001930</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1975,19 +1975,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.6393</t>
+          <t>0.6561</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0064256</t>
+          <t>CAND_0051630</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1997,19 +1997,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.6345</t>
+          <t>0.6558</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0041402</t>
+          <t>CAND_0095619</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2019,12 +2019,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.6343</t>
+          <t>0.654</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Candidate with 6.3 years experience as AI Specialist, mostly showing adjacent skills like Information Retrieval, RAG, Vector Search; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.6335</t>
+          <t>0.6531</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2053,7 +2053,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0017960</t>
+          <t>CAND_0030953</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2063,19 +2063,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.6319</t>
+          <t>0.6512</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Recommendation Systems Engineer (7.7 YoE), having some background in Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 7.8 YoE as Search Engineer, possessing partial overlap in MLOps, Python, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0041568</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2085,12 +2085,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.6295</t>
+          <t>0.6499</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Search Engineer with 5.2 years of background, having some background in Vector Search, TensorFlow, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.6293</t>
+          <t>0.6473</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2119,7 +2119,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0015967</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.629</t>
+          <t>0.6431</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Senior Software Engineer (ML) (5.4 YoE), with limited direct exposure to search/ranking but lists Pinecone, TensorFlow, Embeddings; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
+          <t>CAND_0018722</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2151,19 +2151,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.6217</t>
+          <t>0.6418</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 8.0 years of background, having some background in Vector Search, TensorFlow, Embeddings but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Python, TensorFlow; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2173,19 +2173,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.619</t>
+          <t>0.6404</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.0 YoE), mostly showing adjacent skills like Pinecone, Python, RAG; included as potential pipeline filler.</t>
+          <t>Applied ML Engineer with 8.0 years of background, having some background in Vector Search, TensorFlow, Embeddings but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0030953</t>
+          <t>CAND_0076163</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2195,19 +2195,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.617</t>
+          <t>0.6381</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.8 YoE as Search Engineer, possessing partial overlap in MLOps, Python, RAG; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as NLP Engineer (6.9 YoE), having some background in PyTorch, Python, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0041568</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2217,19 +2217,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.6158</t>
+          <t>0.6362</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Search Engineer with 5.2 years of background, having some background in Vector Search, TensorFlow, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.0 YoE), mostly showing adjacent skills like Pinecone, Python, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0051486</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2239,19 +2239,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.6135</t>
+          <t>0.6354</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>AI Specialist with 5.9 years of background, having some background in Pinecone, Vector Search, TensorFlow but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 8.0 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like Python; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0074735</t>
+          <t>CAND_0067866</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2261,19 +2261,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.6122</t>
+          <t>0.6342</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 5.5 years of background, with limited direct exposure to search/ranking but lists RAG, Information Retrieval, Vector Search; included as potential pipeline filler.</t>
+          <t>Senior Software Engineer (ML) with 6.4 years of background, possessing partial overlap in Embeddings; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0024466</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2283,19 +2283,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.6105</t>
+          <t>0.6339</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0072660</t>
+          <t>CAND_0049978</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2305,19 +2305,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.6081</t>
+          <t>0.6296</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.1 YoE as Machine Learning Engineer, mostly showing adjacent skills like PyTorch, Information Retrieval, FAISS; moderate fit with some technical gaps for this senior role.</t>
+          <t>Senior Software Engineer (ML) with 6.6 years of background, with limited direct exposure to search/ranking but lists PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0044883</t>
+          <t>CAND_0024466</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2327,19 +2327,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.6053</t>
+          <t>0.6289</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0018722</t>
+          <t>CAND_0074735</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.604</t>
+          <t>0.6287</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Python, TensorFlow; included as potential pipeline filler.</t>
+          <t>Applied ML Engineer with 5.5 years of background, with limited direct exposure to search/ranking but lists RAG, Information Retrieval, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0025640</t>
+          <t>CAND_0044883</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2371,19 +2371,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.6032</t>
+          <t>0.626</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.6 YoE as AI Research Engineer, possessing partial overlap in Information Retrieval, FAISS, PyTorch; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0076163</t>
+          <t>CAND_0040117</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2393,19 +2393,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.6019</t>
+          <t>0.6231</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (6.9 YoE), having some background in PyTorch, Python, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.5 years experience as Recommendation Systems Engineer, with limited direct exposure to search/ranking but lists Embeddings, RAG, FAISS; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2415,19 +2415,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.6014</t>
+          <t>0.6213</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Alternative profile showing 8.0 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like Python; moderate fit with some technical gaps for this senior role.</t>
+          <t>Recommendation Systems Engineer with 8.0 years of background, with limited direct exposure to search/ranking but lists FAISS, Milvus, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0089552</t>
+          <t>CAND_0049771</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2437,19 +2437,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.5944</t>
+          <t>0.6192</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Candidate with 6.0 years experience as Machine Learning Engineer, mostly showing adjacent skills like TensorFlow, Vector Search, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), with limited direct exposure to search/ranking but lists Python, PyTorch, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0040117</t>
+          <t>CAND_0053605</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2459,19 +2459,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.5927</t>
+          <t>0.6185</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Candidate with 6.5 years experience as Recommendation Systems Engineer, with limited direct exposure to search/ranking but lists Embeddings, RAG, FAISS; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Senior Software Engineer (ML) (6.9 YoE), having some background in RAG but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
+          <t>CAND_0093331</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2481,19 +2481,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.5924</t>
+          <t>0.6147</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 8.0 years of background, with limited direct exposure to search/ranking but lists FAISS, Milvus, MLOps; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as NLP Engineer (16.1 YoE), having some background in PyTorch, Embeddings, Milvus but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0050707</t>
+          <t>CAND_0082086</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2503,19 +2503,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.5924</t>
+          <t>0.6145</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Specialist (5.3 YoE), having some background in RAG, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Senior Software Engineer (ML) with 6.0 years of background, having some background in FAISS, Pinecone, PyTorch but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0049978</t>
+          <t>CAND_0078508</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2525,19 +2525,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.5889</t>
+          <t>0.6134</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.6 years of background, with limited direct exposure to search/ranking but lists PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.2 YoE), with limited direct exposure to search/ranking but lists Embeddings, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0049771</t>
+          <t>CAND_0072660</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2547,19 +2547,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.5886</t>
+          <t>0.6133</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), with limited direct exposure to search/ranking but lists Python, PyTorch, MLOps; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 7.1 YoE as Machine Learning Engineer, mostly showing adjacent skills like PyTorch, Information Retrieval, FAISS; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0008978</t>
+          <t>CAND_0050707</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.5884</t>
+          <t>0.6129</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Candidate with 6.7 years experience as Junior ML Engineer, mostly showing adjacent skills like Embeddings, NLP, MLOps; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Adjacent candidate working as AI Specialist (5.3 YoE), having some background in RAG, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0078508</t>
+          <t>CAND_0093883</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2591,19 +2591,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.5875</t>
+          <t>0.6121</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.2 YoE), with limited direct exposure to search/ranking but lists Embeddings, NLP; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), possessing partial overlap in Embeddings, MLOps, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0066376</t>
+          <t>CAND_0089552</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2613,19 +2613,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.5854</t>
+          <t>0.6116</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.7 YoE), with limited direct exposure to search/ranking but lists NLP, Information Retrieval, FAISS; included as potential pipeline filler.</t>
+          <t>Candidate with 6.0 years experience as Machine Learning Engineer, mostly showing adjacent skills like TensorFlow, Vector Search, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0093331</t>
+          <t>CAND_0010770</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2635,12 +2635,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.5819</t>
+          <t>0.6081</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (16.1 YoE), having some background in PyTorch, Embeddings, Milvus but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 15.2 YoE as Recommendation Systems Engineer, mostly showing adjacent skills like TensorFlow, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat/perf: implement hybrid recall search, precompute offline embeddings, and use multiplicative scoring vetoes
</commit_message>
<xml_diff>
--- a/outputs/mohd_ibadullah.xlsx
+++ b/outputs/mohd_ibadullah.xlsx
@@ -1305,7 +1305,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1315,19 +1315,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.7069</t>
+          <t>0.7071</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 7.3 years in the field, matching key job requirements like Pinecone, Vector Search, RAG. Good overall behavioral signals.</t>
+          <t>Solid candidate working as AI Engineer with 5.8 years in the field, matching key job requirements like MLOps, NLP, FAISS. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0030468</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1337,19 +1337,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.7037</t>
+          <t>0.7069</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Applied Scientist with 5.4 years in the field, matching key job requirements like TensorFlow, Ranking Systems, Milvus. Good overall behavioral signals.</t>
+          <t>Solid candidate working as AI Engineer with 7.3 years in the field, matching key job requirements like Pinecone, Vector Search, RAG. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0030468</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1359,19 +1359,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.7003</t>
+          <t>0.7037</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 6.5 years in the field, matching key job requirements like Milvus, TensorFlow, Python, note the longer notice period of 120 days.</t>
+          <t>Solid candidate working as Senior Applied Scientist with 5.4 years in the field, matching key job requirements like TensorFlow, Ranking Systems, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0081686</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1381,19 +1381,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>0.7003</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (6.0 YoE), matching key job requirements like Embeddings, FAISS, Milvus. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Data Scientist with 6.5 years in the field, matching key job requirements like Milvus, TensorFlow, Python, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0081686</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1403,19 +1403,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.6997</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Solid candidate working as Staff Machine Learning Engineer with 8.8 years in the field, matching key job requirements like MLOps, Python, Milvus. Good overall behavioral signals.</t>
+          <t>Competent Search Engineer (6.0 YoE), matching key job requirements like Embeddings, FAISS, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0096172</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1425,19 +1425,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.6963</t>
+          <t>0.6997</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Solid candidate working as NLP Engineer with 5.2 years in the field, with matching skills in Python, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Staff Machine Learning Engineer with 8.8 years in the field, matching key job requirements like MLOps, Python, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0058412</t>
+          <t>CAND_0096172</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1447,19 +1447,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.6949</t>
+          <t>0.6963</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Software Engineer (ML) with 6.6 years in the field, with matching skills in Embeddings, Milvus, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Solid candidate working as NLP Engineer with 5.2 years in the field, with matching skills in Python, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0025882</t>
+          <t>CAND_0058412</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.6942</t>
+          <t>0.6949</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Software Engineer (ML) with 5.6 years in the field, with matching skills in FAISS, Vector Search, Milvus and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Software Engineer (ML) with 6.6 years in the field, with matching skills in Embeddings, Milvus, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0025882</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1491,19 +1491,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.6939</t>
+          <t>0.6942</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (6.8 YoE), matching key job requirements like PyTorch, FAISS, NLP. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Software Engineer (ML) with 5.6 years in the field, with matching skills in FAISS, Vector Search, Milvus and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0077285</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.6911</t>
+          <t>0.6939</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (6.8 YoE), matching key job requirements like PyTorch, FAISS, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0077285</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1535,19 +1535,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.6896</t>
+          <t>0.6911</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Competent Applied ML Engineer (5.8 YoE), matching key job requirements like Vector Search, Milvus, Embeddings. Good overall behavioral signals.</t>
+          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0043860</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1557,19 +1557,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.6888</t>
+          <t>0.6896</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1579,19 +1579,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.6848</t>
+          <t>0.6888</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Candidate with 7.2 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, Information Retrieval, PyTorch; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1601,19 +1601,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.6825</t>
+          <t>0.6848</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Candidate with 7.2 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, Information Retrieval, PyTorch; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0029367</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1623,19 +1623,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.6815</t>
+          <t>0.6825</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
+          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0098454</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1645,19 +1645,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.681</t>
+          <t>0.6815</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0098454</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1667,19 +1667,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.6801</t>
+          <t>0.681</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0012837</t>
+          <t>CAND_0007009</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.6793</t>
+          <t>0.6807</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.4 YoE as Junior ML Engineer, mostly showing adjacent skills like Vector Search, MLOps, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Recommendation Systems Engineer (7.9 YoE), having some background in Python, Embeddings but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1711,19 +1711,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.679</t>
+          <t>0.6801</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0099401</t>
+          <t>CAND_0012837</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1733,19 +1733,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.6777</t>
+          <t>0.6793</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 6.4 YoE as Junior ML Engineer, mostly showing adjacent skills like Vector Search, MLOps, NLP; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1755,19 +1755,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.675</t>
+          <t>0.679</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0061265</t>
+          <t>CAND_0099401</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1777,19 +1777,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.6748</t>
+          <t>0.6777</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0006557</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1799,19 +1799,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.6714</t>
+          <t>0.675</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0000031</t>
+          <t>CAND_0061265</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1821,19 +1821,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.6703</t>
+          <t>0.6748</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 6.0 years of background, possessing partial overlap in FAISS, Pinecone, MLOps; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0006557</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1843,19 +1843,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.6693</t>
+          <t>0.6714</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0041402</t>
+          <t>CAND_0027801</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1865,19 +1865,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.6666</t>
+          <t>0.6712</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Candidate with 6.3 years experience as AI Specialist, mostly showing adjacent skills like Information Retrieval, RAG, Vector Search; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 7.4 years experience as NLP Engineer, mostly showing adjacent skills like FAISS, Milvus, TensorFlow; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0000031</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1887,19 +1887,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.665</t>
+          <t>0.6703</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Recommendation Systems Engineer with 6.0 years of background, possessing partial overlap in FAISS, Pinecone, MLOps; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0017960</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.6646</t>
+          <t>0.6693</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Recommendation Systems Engineer (7.7 YoE), having some background in Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0064256</t>
+          <t>CAND_0041402</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1931,19 +1931,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.6623</t>
+          <t>0.6666</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.3 years experience as AI Specialist, mostly showing adjacent skills like Information Retrieval, RAG, Vector Search; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0070202</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1953,19 +1953,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.6615</t>
+          <t>0.665</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Candidate with 5.1 years experience as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, PyTorch, RAG; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0017960</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1975,19 +1975,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.6561</t>
+          <t>0.6646</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Recommendation Systems Engineer (7.7 YoE), having some background in Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0051630</t>
+          <t>CAND_0064256</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1997,19 +1997,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.6558</t>
+          <t>0.6623</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0095619</t>
+          <t>CAND_0070202</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2019,19 +2019,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.654</t>
+          <t>0.6615</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Candidate with 5.1 years experience as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, PyTorch, RAG; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0087006</t>
+          <t>CAND_0001930</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2041,19 +2041,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.6531</t>
+          <t>0.6561</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0030953</t>
+          <t>CAND_0051630</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2063,19 +2063,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.6512</t>
+          <t>0.6558</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.8 YoE as Search Engineer, possessing partial overlap in MLOps, Python, RAG; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0041568</t>
+          <t>CAND_0095619</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2085,19 +2085,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.6499</t>
+          <t>0.654</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Search Engineer with 5.2 years of background, having some background in Vector Search, TensorFlow, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0087006</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.6473</t>
+          <t>0.6531</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0015967</t>
+          <t>CAND_0030953</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.6431</t>
+          <t>0.6512</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Senior Software Engineer (ML) (5.4 YoE), with limited direct exposure to search/ranking but lists Pinecone, TensorFlow, Embeddings; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 7.8 YoE as Search Engineer, possessing partial overlap in MLOps, Python, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0018722</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2151,19 +2151,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.6418</t>
+          <t>0.6473</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Python, TensorFlow; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
+          <t>CAND_0065195</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2173,19 +2173,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.6404</t>
+          <t>0.6423</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 8.0 years of background, having some background in Vector Search, TensorFlow, Embeddings but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Search Engineer with 5.1 years of background, with limited direct exposure to search/ranking but lists MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0076163</t>
+          <t>CAND_0018722</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2195,19 +2195,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.6381</t>
+          <t>0.6418</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (6.9 YoE), having some background in PyTorch, Python, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Python, TensorFlow; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2217,19 +2217,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.6362</t>
+          <t>0.6404</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.0 YoE), mostly showing adjacent skills like Pinecone, Python, RAG; included as potential pipeline filler.</t>
+          <t>Applied ML Engineer with 8.0 years of background, having some background in Vector Search, TensorFlow, Embeddings but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0076163</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2239,19 +2239,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.6354</t>
+          <t>0.6381</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Alternative profile showing 8.0 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like Python; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as NLP Engineer (6.9 YoE), having some background in PyTorch, Python, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0067866</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2261,19 +2261,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.6342</t>
+          <t>0.6362</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.4 years of background, possessing partial overlap in Embeddings; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.0 YoE), mostly showing adjacent skills like Pinecone, Python, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2283,19 +2283,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.6339</t>
+          <t>0.6354</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 8.0 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like Python; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0049978</t>
+          <t>CAND_0067866</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2305,19 +2305,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.6296</t>
+          <t>0.6342</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.6 years of background, with limited direct exposure to search/ranking but lists PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Senior Software Engineer (ML) with 6.4 years of background, possessing partial overlap in Embeddings; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0024466</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2327,19 +2327,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.6289</t>
+          <t>0.6339</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0074735</t>
+          <t>CAND_0049978</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.6287</t>
+          <t>0.6296</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 5.5 years of background, with limited direct exposure to search/ranking but lists RAG, Information Retrieval, Vector Search; included as potential pipeline filler.</t>
+          <t>Senior Software Engineer (ML) with 6.6 years of background, with limited direct exposure to search/ranking but lists PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0044883</t>
+          <t>CAND_0024466</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2371,19 +2371,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.626</t>
+          <t>0.6289</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0040117</t>
+          <t>CAND_0074735</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2393,19 +2393,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.6231</t>
+          <t>0.6287</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Candidate with 6.5 years experience as Recommendation Systems Engineer, with limited direct exposure to search/ranking but lists Embeddings, RAG, FAISS; moderate fit with some technical gaps for this senior role.</t>
+          <t>Applied ML Engineer with 5.5 years of background, with limited direct exposure to search/ranking but lists RAG, Information Retrieval, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
+          <t>CAND_0044883</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2415,19 +2415,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.6213</t>
+          <t>0.626</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 8.0 years of background, with limited direct exposure to search/ranking but lists FAISS, Milvus, MLOps; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0049771</t>
+          <t>CAND_0040117</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2437,19 +2437,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.6192</t>
+          <t>0.6231</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), with limited direct exposure to search/ranking but lists Python, PyTorch, MLOps; included as potential pipeline filler.</t>
+          <t>Candidate with 6.5 years experience as Recommendation Systems Engineer, with limited direct exposure to search/ranking but lists Embeddings, RAG, FAISS; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0053605</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2459,19 +2459,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.6185</t>
+          <t>0.6213</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Senior Software Engineer (ML) (6.9 YoE), having some background in RAG but less specialized; included as potential pipeline filler.</t>
+          <t>Recommendation Systems Engineer with 8.0 years of background, with limited direct exposure to search/ranking but lists FAISS, Milvus, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0093331</t>
+          <t>CAND_0049771</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2481,19 +2481,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.6147</t>
+          <t>0.6192</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (16.1 YoE), having some background in PyTorch, Embeddings, Milvus but less specialized; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), with limited direct exposure to search/ranking but lists Python, PyTorch, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0082086</t>
+          <t>CAND_0093331</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2503,19 +2503,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.6145</t>
+          <t>0.6147</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.0 years of background, having some background in FAISS, Pinecone, PyTorch but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as NLP Engineer (16.1 YoE), having some background in PyTorch, Embeddings, Milvus but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0078508</t>
+          <t>CAND_0082086</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2525,19 +2525,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.6134</t>
+          <t>0.6145</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.2 YoE), with limited direct exposure to search/ranking but lists Embeddings, NLP; included as potential pipeline filler.</t>
+          <t>Senior Software Engineer (ML) with 6.0 years of background, having some background in FAISS, Pinecone, PyTorch but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0072660</t>
+          <t>CAND_0078508</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2547,19 +2547,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.6133</t>
+          <t>0.6134</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.1 YoE as Machine Learning Engineer, mostly showing adjacent skills like PyTorch, Information Retrieval, FAISS; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.2 YoE), with limited direct exposure to search/ranking but lists Embeddings, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0050707</t>
+          <t>CAND_0072660</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.6129</t>
+          <t>0.6133</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Specialist (5.3 YoE), having some background in RAG, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 7.1 YoE as Machine Learning Engineer, mostly showing adjacent skills like PyTorch, Information Retrieval, FAISS; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0093883</t>
+          <t>CAND_0050707</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2591,19 +2591,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.6121</t>
+          <t>0.6129</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), possessing partial overlap in Embeddings, MLOps, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as AI Specialist (5.3 YoE), having some background in RAG, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0089552</t>
+          <t>CAND_0093883</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2613,19 +2613,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.6116</t>
+          <t>0.6121</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Candidate with 6.0 years experience as Machine Learning Engineer, mostly showing adjacent skills like TensorFlow, Vector Search, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), possessing partial overlap in Embeddings, MLOps, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0010770</t>
+          <t>CAND_0007567</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2635,12 +2635,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.6081</t>
+          <t>0.6118</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Alternative profile showing 15.2 YoE as Recommendation Systems Engineer, mostly showing adjacent skills like TensorFlow, MLOps; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.1 YoE as AI Specialist, possessing partial overlap in NLP, MLOps, FAISS; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
implemented hybrid search with precomputed embeddings
</commit_message>
<xml_diff>
--- a/outputs/mohd_ibadullah.xlsx
+++ b/outputs/mohd_ibadullah.xlsx
@@ -1305,7 +1305,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1315,19 +1315,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.7069</t>
+          <t>0.7071</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 7.3 years in the field, matching key job requirements like Pinecone, Vector Search, RAG. Good overall behavioral signals.</t>
+          <t>Solid candidate working as AI Engineer with 5.8 years in the field, matching key job requirements like MLOps, NLP, FAISS. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0030468</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1337,19 +1337,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.7037</t>
+          <t>0.7069</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Applied Scientist with 5.4 years in the field, matching key job requirements like TensorFlow, Ranking Systems, Milvus. Good overall behavioral signals.</t>
+          <t>Solid candidate working as AI Engineer with 7.3 years in the field, matching key job requirements like Pinecone, Vector Search, RAG. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0030468</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1359,19 +1359,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.7003</t>
+          <t>0.7037</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 6.5 years in the field, matching key job requirements like Milvus, TensorFlow, Python, note the longer notice period of 120 days.</t>
+          <t>Solid candidate working as Senior Applied Scientist with 5.4 years in the field, matching key job requirements like TensorFlow, Ranking Systems, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0081686</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1381,19 +1381,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>0.7003</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (6.0 YoE), matching key job requirements like Embeddings, FAISS, Milvus. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Data Scientist with 6.5 years in the field, matching key job requirements like Milvus, TensorFlow, Python, note the longer notice period of 120 days.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0081686</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1403,19 +1403,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.6997</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Solid candidate working as Staff Machine Learning Engineer with 8.8 years in the field, matching key job requirements like MLOps, Python, Milvus. Good overall behavioral signals.</t>
+          <t>Competent Search Engineer (6.0 YoE), matching key job requirements like Embeddings, FAISS, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0096172</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1425,19 +1425,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.6963</t>
+          <t>0.6997</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Solid candidate working as NLP Engineer with 5.2 years in the field, with matching skills in Python, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Staff Machine Learning Engineer with 8.8 years in the field, matching key job requirements like MLOps, Python, Milvus. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0058412</t>
+          <t>CAND_0096172</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1447,19 +1447,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.6949</t>
+          <t>0.6963</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Software Engineer (ML) with 6.6 years in the field, with matching skills in Embeddings, Milvus, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Solid candidate working as NLP Engineer with 5.2 years in the field, with matching skills in Python, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0025882</t>
+          <t>CAND_0058412</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.6942</t>
+          <t>0.6949</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Software Engineer (ML) with 5.6 years in the field, with matching skills in FAISS, Vector Search, Milvus and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Software Engineer (ML) with 6.6 years in the field, with matching skills in Embeddings, Milvus, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0025882</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1491,19 +1491,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.6939</t>
+          <t>0.6942</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (6.8 YoE), matching key job requirements like PyTorch, FAISS, NLP. Good overall behavioral signals.</t>
+          <t>Solid candidate working as Senior Software Engineer (ML) with 5.6 years in the field, with matching skills in FAISS, Vector Search, Milvus and solid backend fundamentals. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0077285</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.6911</t>
+          <t>0.6939</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
+          <t>Competent AI Engineer (6.8 YoE), matching key job requirements like PyTorch, FAISS, NLP. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0077285</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1535,19 +1535,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.6896</t>
+          <t>0.6911</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Competent Applied ML Engineer (5.8 YoE), matching key job requirements like Vector Search, Milvus, Embeddings. Good overall behavioral signals.</t>
+          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0043860</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1557,19 +1557,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.6888</t>
+          <t>0.6896</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1579,19 +1579,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.6848</t>
+          <t>0.6888</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Candidate with 7.2 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, Information Retrieval, PyTorch; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1601,19 +1601,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.6825</t>
+          <t>0.6848</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Candidate with 7.2 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, Information Retrieval, PyTorch; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0029367</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1623,19 +1623,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.6815</t>
+          <t>0.6825</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
+          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0098454</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1645,19 +1645,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.681</t>
+          <t>0.6815</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0098454</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1667,19 +1667,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.6801</t>
+          <t>0.681</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0012837</t>
+          <t>CAND_0007009</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.6793</t>
+          <t>0.6807</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.4 YoE as Junior ML Engineer, mostly showing adjacent skills like Vector Search, MLOps, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Recommendation Systems Engineer (7.9 YoE), having some background in Python, Embeddings but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1711,19 +1711,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.679</t>
+          <t>0.6801</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0099401</t>
+          <t>CAND_0012837</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1733,19 +1733,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.6777</t>
+          <t>0.6793</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 6.4 YoE as Junior ML Engineer, mostly showing adjacent skills like Vector Search, MLOps, NLP; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1755,19 +1755,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.675</t>
+          <t>0.679</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0061265</t>
+          <t>CAND_0099401</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1777,19 +1777,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.6748</t>
+          <t>0.6777</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0006557</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1799,19 +1799,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.6714</t>
+          <t>0.675</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0000031</t>
+          <t>CAND_0061265</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1821,19 +1821,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.6703</t>
+          <t>0.6748</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 6.0 years of background, possessing partial overlap in FAISS, Pinecone, MLOps; moderate fit with some technical gaps for this senior role.</t>
+          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0006557</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1843,19 +1843,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.6693</t>
+          <t>0.6714</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0041402</t>
+          <t>CAND_0027801</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1865,19 +1865,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.6666</t>
+          <t>0.6712</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Candidate with 6.3 years experience as AI Specialist, mostly showing adjacent skills like Information Retrieval, RAG, Vector Search; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 7.4 years experience as NLP Engineer, mostly showing adjacent skills like FAISS, Milvus, TensorFlow; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0000031</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1887,19 +1887,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.665</t>
+          <t>0.6703</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Recommendation Systems Engineer with 6.0 years of background, possessing partial overlap in FAISS, Pinecone, MLOps; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0017960</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.6646</t>
+          <t>0.6693</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Recommendation Systems Engineer (7.7 YoE), having some background in Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0064256</t>
+          <t>CAND_0041402</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1931,19 +1931,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.6623</t>
+          <t>0.6666</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 6.3 years experience as AI Specialist, mostly showing adjacent skills like Information Retrieval, RAG, Vector Search; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0070202</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1953,19 +1953,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.6615</t>
+          <t>0.665</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Candidate with 5.1 years experience as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, PyTorch, RAG; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0017960</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1975,19 +1975,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.6561</t>
+          <t>0.6646</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as Recommendation Systems Engineer (7.7 YoE), having some background in Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0051630</t>
+          <t>CAND_0064256</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1997,19 +1997,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.6558</t>
+          <t>0.6623</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0095619</t>
+          <t>CAND_0070202</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2019,19 +2019,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.654</t>
+          <t>0.6615</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Candidate with 5.1 years experience as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, PyTorch, RAG; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0087006</t>
+          <t>CAND_0001930</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2041,19 +2041,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.6531</t>
+          <t>0.6561</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0030953</t>
+          <t>CAND_0051630</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2063,19 +2063,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.6512</t>
+          <t>0.6558</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.8 YoE as Search Engineer, possessing partial overlap in MLOps, Python, RAG; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0041568</t>
+          <t>CAND_0095619</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2085,19 +2085,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.6499</t>
+          <t>0.654</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Search Engineer with 5.2 years of background, having some background in Vector Search, TensorFlow, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0087006</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.6473</t>
+          <t>0.6531</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0015967</t>
+          <t>CAND_0030953</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.6431</t>
+          <t>0.6512</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Senior Software Engineer (ML) (5.4 YoE), with limited direct exposure to search/ranking but lists Pinecone, TensorFlow, Embeddings; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 7.8 YoE as Search Engineer, possessing partial overlap in MLOps, Python, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0018722</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2151,19 +2151,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.6418</t>
+          <t>0.6473</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Python, TensorFlow; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
+          <t>CAND_0065195</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2173,19 +2173,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.6404</t>
+          <t>0.6423</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 8.0 years of background, having some background in Vector Search, TensorFlow, Embeddings but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Search Engineer with 5.1 years of background, with limited direct exposure to search/ranking but lists MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0076163</t>
+          <t>CAND_0018722</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2195,19 +2195,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.6381</t>
+          <t>0.6418</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (6.9 YoE), having some background in PyTorch, Python, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Python, TensorFlow; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2217,19 +2217,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.6362</t>
+          <t>0.6404</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.0 YoE), mostly showing adjacent skills like Pinecone, Python, RAG; included as potential pipeline filler.</t>
+          <t>Applied ML Engineer with 8.0 years of background, having some background in Vector Search, TensorFlow, Embeddings but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0076163</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2239,19 +2239,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.6354</t>
+          <t>0.6381</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Alternative profile showing 8.0 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like Python; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as NLP Engineer (6.9 YoE), having some background in PyTorch, Python, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0067866</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2261,19 +2261,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.6342</t>
+          <t>0.6362</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.4 years of background, possessing partial overlap in Embeddings; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (5.0 YoE), mostly showing adjacent skills like Pinecone, Python, RAG; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2283,19 +2283,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.6339</t>
+          <t>0.6354</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 8.0 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like Python; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0049978</t>
+          <t>CAND_0067866</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2305,19 +2305,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.6296</t>
+          <t>0.6342</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.6 years of background, with limited direct exposure to search/ranking but lists PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Senior Software Engineer (ML) with 6.4 years of background, possessing partial overlap in Embeddings; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0024466</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2327,19 +2327,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.6289</t>
+          <t>0.6339</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0074735</t>
+          <t>CAND_0049978</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.6287</t>
+          <t>0.6296</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 5.5 years of background, with limited direct exposure to search/ranking but lists RAG, Information Retrieval, Vector Search; included as potential pipeline filler.</t>
+          <t>Senior Software Engineer (ML) with 6.6 years of background, with limited direct exposure to search/ranking but lists PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0044883</t>
+          <t>CAND_0024466</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2371,19 +2371,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.626</t>
+          <t>0.6289</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0040117</t>
+          <t>CAND_0074735</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2393,19 +2393,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.6231</t>
+          <t>0.6287</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Candidate with 6.5 years experience as Recommendation Systems Engineer, with limited direct exposure to search/ranking but lists Embeddings, RAG, FAISS; moderate fit with some technical gaps for this senior role.</t>
+          <t>Applied ML Engineer with 5.5 years of background, with limited direct exposure to search/ranking but lists RAG, Information Retrieval, Vector Search; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
+          <t>CAND_0044883</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2415,19 +2415,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.6213</t>
+          <t>0.626</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 8.0 years of background, with limited direct exposure to search/ranking but lists FAISS, Milvus, MLOps; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0049771</t>
+          <t>CAND_0040117</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2437,19 +2437,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.6192</t>
+          <t>0.6231</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), with limited direct exposure to search/ranking but lists Python, PyTorch, MLOps; included as potential pipeline filler.</t>
+          <t>Candidate with 6.5 years experience as Recommendation Systems Engineer, with limited direct exposure to search/ranking but lists Embeddings, RAG, FAISS; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0053605</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2459,19 +2459,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.6185</t>
+          <t>0.6213</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Senior Software Engineer (ML) (6.9 YoE), having some background in RAG but less specialized; included as potential pipeline filler.</t>
+          <t>Recommendation Systems Engineer with 8.0 years of background, with limited direct exposure to search/ranking but lists FAISS, Milvus, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0093331</t>
+          <t>CAND_0049771</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2481,19 +2481,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.6147</t>
+          <t>0.6192</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (16.1 YoE), having some background in PyTorch, Embeddings, Milvus but less specialized; included as potential pipeline filler.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), with limited direct exposure to search/ranking but lists Python, PyTorch, MLOps; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0082086</t>
+          <t>CAND_0093331</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2503,19 +2503,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.6145</t>
+          <t>0.6147</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.0 years of background, having some background in FAISS, Pinecone, PyTorch but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as NLP Engineer (16.1 YoE), having some background in PyTorch, Embeddings, Milvus but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0078508</t>
+          <t>CAND_0082086</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2525,19 +2525,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.6134</t>
+          <t>0.6145</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.2 YoE), with limited direct exposure to search/ranking but lists Embeddings, NLP; included as potential pipeline filler.</t>
+          <t>Senior Software Engineer (ML) with 6.0 years of background, having some background in FAISS, Pinecone, PyTorch but less specialized; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0072660</t>
+          <t>CAND_0078508</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2547,19 +2547,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.6133</t>
+          <t>0.6134</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.1 YoE as Machine Learning Engineer, mostly showing adjacent skills like PyTorch, Information Retrieval, FAISS; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.2 YoE), with limited direct exposure to search/ranking but lists Embeddings, NLP; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0050707</t>
+          <t>CAND_0072660</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.6129</t>
+          <t>0.6133</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Specialist (5.3 YoE), having some background in RAG, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 7.1 YoE as Machine Learning Engineer, mostly showing adjacent skills like PyTorch, Information Retrieval, FAISS; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0093883</t>
+          <t>CAND_0050707</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2591,19 +2591,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.6121</t>
+          <t>0.6129</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), possessing partial overlap in Embeddings, MLOps, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Adjacent candidate working as AI Specialist (5.3 YoE), having some background in RAG, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0089552</t>
+          <t>CAND_0093883</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2613,19 +2613,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.6116</t>
+          <t>0.6121</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Candidate with 6.0 years experience as Machine Learning Engineer, mostly showing adjacent skills like TensorFlow, Vector Search, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), possessing partial overlap in Embeddings, MLOps, Milvus; lower title relevance to the specific AI/ML requirements.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0010770</t>
+          <t>CAND_0007567</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2635,12 +2635,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.6081</t>
+          <t>0.6118</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Alternative profile showing 15.2 YoE as Recommendation Systems Engineer, mostly showing adjacent skills like TensorFlow, MLOps; included as potential pipeline filler.</t>
+          <t>Alternative profile showing 6.1 YoE as AI Specialist, possessing partial overlap in NLP, MLOps, FAISS; moderate fit with some technical gaps for this senior role.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
visual fixes and memory optimizations
</commit_message>
<xml_diff>
--- a/outputs/mohd_ibadullah.xlsx
+++ b/outputs/mohd_ibadullah.xlsx
@@ -457,12 +457,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.994</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Outstanding candidate as Senior Machine Learning Engineer showing 8.1 years of experience, shows deep technical expertise in Python, Information Retrieval, Embeddings and search infrastructure. Highly active on Redrob with a 87% recruiter response rate.</t>
+          <t>Strong top-tier match: Senior Machine Learning Engineer at Flipkart with 8.1 years experience. Recent role: Senior Machine Learning Engineer at Flipkart. Matched JD skills: Python, LLM Fine-tuning, Information Retrieval, Embeddings. Redrob signals: 87% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
@@ -479,12 +479,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.9617</t>
+          <t>0.9554</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Top-tier candidate currently working as Senior Applied Scientist (5.3 YoE), demonstrates strong proficiency in Vector Search, Pinecone, Embeddings and alignment with the JD. Available quickly with a short notice period of 0 days.</t>
+          <t>Strong top-tier match: Senior Applied Scientist at Sarvam AI with 5.3 years experience. Recent role: Senior Applied Scientist at Sarvam AI. Matched JD skills: Vector Search, LLM Fine-tuning, Pinecone, Embeddings. Redrob signals: 55% recruiter response rate; 0-day notice period; open to work.</t>
         </is>
       </c>
     </row>
@@ -501,12 +501,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.9568</t>
+          <t>0.9501</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Top-tier candidate currently working as Senior NLP Engineer (5.2 YoE), offers solid expertise in MLOps, Information Retrieval, Python which matches the core ranking mandate. Excellent platform engagement with 86% response rate.</t>
+          <t>Strong top-tier match: Senior NLP Engineer at Netflix with 5.2 years experience. Recent role: Senior NLP Engineer at Netflix. Matched JD skills: MLOps, Information Retrieval, Python, NLP. Redrob signals: 86% recruiter response rate; 60-day notice period.</t>
         </is>
       </c>
     </row>
@@ -523,19 +523,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.9388</t>
+          <t>0.9441</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Highly relevant Senior AI Engineer with 5.9 years of background, offers solid expertise in FAISS, TensorFlow, NLP which matches the core ranking mandate. Excellent platform engagement with 80% response rate.</t>
+          <t>Strong top-tier match: Senior AI Engineer at Apple with 5.9 years experience. Recent role: Senior AI Engineer at Apple. Matched JD skills: FAISS, TensorFlow, NLP, Pinecone. Redrob signals: 80% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0011687</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -545,19 +545,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.9221</t>
+          <t>0.905</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in TensorFlow, FAISS, Embeddings and search infrastructure. Available quickly with a short notice period of 15 days.</t>
+          <t>Strong top-tier match: Senior AI Engineer at Netflix with 7.8 years experience. Recent role: Senior AI Engineer at Netflix. Matched JD skills: Pinecone, Information Retrieval, Embeddings, RAG. Redrob signals: 76% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -567,19 +567,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.9179</t>
+          <t>0.9039</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Highly relevant Lead AI Engineer with 6.7 years of background, demonstrates strong proficiency in Information Retrieval, PyTorch, Vector Search and alignment with the JD. Highly active on Redrob with a 73% recruiter response rate.</t>
+          <t>Strong top-tier match: Senior NLP Engineer at Salesforce with 8.9 years experience. Recent role: Senior NLP Engineer at Salesforce. Matched JD skills: Python, Pinecone. Redrob signals: 78% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0046064</t>
+          <t>CAND_0008425</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -589,19 +589,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.9127</t>
+          <t>0.9018</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Highly relevant Senior NLP Engineer with 8.9 years of background, has successfully deployed systems involving Python, Pinecone at scale. Highly active on Redrob with a 78% recruiter response rate.</t>
+          <t>Strong top-tier match: Senior NLP Engineer at Ola with 7.8 years experience. Recent role: Senior NLP Engineer at Ola. Matched JD skills: NLP, TensorFlow, Python, Information Retrieval. Redrob signals: 66% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0039754</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.9086</t>
+          <t>0.8957</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Exceptional Senior AI Engineer offering 7.8 years of experience, offers solid expertise in Pinecone, Information Retrieval, Embeddings which matches the core ranking mandate. Highly active on Redrob with a 76% recruiter response rate.</t>
+          <t>Strong top-tier match: Senior Applied Scientist at Meta with 16.2 years experience. Recent role: Senior Applied Scientist at Meta. Matched JD skills: LLM Fine-tuning, NLP, Python, TensorFlow. Redrob signals: 81% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0008425</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -633,19 +633,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.9083</t>
+          <t>0.877</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in NLP, TensorFlow, Python and search infrastructure. Highly active on Redrob with a 66% recruiter response rate.</t>
+          <t>Strong top-tier match: Staff Machine Learning Engineer at Paytm with 7.0 years experience. Recent role: Staff Machine Learning Engineer at Paytm. Matched JD skills: Pinecone, Information Retrieval, RAG, Python. Redrob signals: 95% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -655,19 +655,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.8949</t>
+          <t>0.8726</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Exceptional Senior Machine Learning Engineer offering 6.1 years of experience, demonstrates strong proficiency in Information Retrieval, TensorFlow, NLP and alignment with the JD. Highly active on Redrob with a 88% recruiter response rate.</t>
+          <t>Strong top-tier match: Staff Machine Learning Engineer at Yellow.ai with 8.6 years experience. Recent role: Staff Machine Learning Engineer at Yellow.ai. Matched JD skills: Pinecone, RAG, TensorFlow, MLOps. Redrob signals: 83% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0039754</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -677,19 +677,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.8863</t>
+          <t>0.8722</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Exceptional Senior Applied Scientist offering 16.2 years of experience, offers solid expertise in NLP, Python, TensorFlow which matches the core ranking mandate. Highly active on Redrob with a 81% recruiter response rate.</t>
+          <t>Solid fit: Senior AI Engineer at Meta with 7.9 years experience. Recent role: Senior AI Engineer at Meta. Matched JD skills: NLP, Python, Ranking Systems. Redrob signals: 79% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -699,19 +699,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.8734</t>
+          <t>0.8696</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Highly relevant Staff Machine Learning Engineer with 7.0 years of background, demonstrates strong proficiency in Pinecone, Information Retrieval, RAG and alignment with the JD. Highly active on Redrob with a 95% recruiter response rate.</t>
+          <t>Solid fit: Senior Machine Learning Engineer at Genpact AI with 6.1 years experience. Recent role: Senior Machine Learning Engineer at Genpact AI. Matched JD skills: Information Retrieval, TensorFlow, NLP. Redrob signals: 88% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -721,19 +721,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.8682</t>
+          <t>0.868</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Exceptional Staff Machine Learning Engineer offering 8.6 years of experience, shows deep technical expertise in Pinecone, RAG, TensorFlow and search infrastructure. Highly active on Redrob with a 83% recruiter response rate.</t>
+          <t>Solid fit: Lead AI Engineer at Meta with 8.6 years experience. Recent role: Lead AI Engineer at Meta. Matched JD skills: LLM Fine-tuning, Vector Search, NLP, MLOps. Redrob signals: 11% recruiter response rate; 30-day notice period. Concerns: low recruiter engagement.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -743,19 +743,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.867</t>
+          <t>0.8653</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Exceptional Senior Machine Learning Engineer offering 7.2 years of experience, has successfully deployed systems involving Pinecone, Information Retrieval, Milvus at scale. Highly active on Redrob with a 61% recruiter response rate.</t>
+          <t>Solid fit: Lead AI Engineer at Razorpay with 6.7 years experience. Recent role: Lead AI Engineer at Razorpay. Matched JD skills: Information Retrieval, PyTorch, Vector Search, Python. Redrob signals: 73% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -765,19 +765,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.8666</t>
+          <t>0.8615</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Outstanding candidate as Senior AI Engineer showing 7.9 years of experience, shows deep technical expertise in NLP, Python, Ranking Systems and search infrastructure. Highly active on Redrob with a 79% recruiter response rate.</t>
+          <t>Solid fit: Senior NLP Engineer at Niramai with 7.8 years experience. Recent role: Senior NLP Engineer at Niramai. Matched JD skills: TensorFlow, FAISS, Embeddings, MLOps. Redrob signals: 89% recruiter response rate; 15-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0033861</t>
+          <t>CAND_0007411</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -787,19 +787,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.8573</t>
+          <t>0.8536</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior NLP Engineer with 8.0 years in the field, matching key job requirements like TensorFlow, Pinecone, Vector Search, though platform response rate is lower (16%).</t>
+          <t>Solid fit: Senior Machine Learning Engineer at Amazon with 8.0 years experience. Recent role: Senior Machine Learning Engineer at Amazon. Matched JD skills: LLM Fine-tuning, Vector Search, PyTorch, Information Retrieval. Redrob signals: 12% recruiter response rate; 15-day notice period. Concerns: low recruiter engagement.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0095528</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -809,19 +809,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.8355</t>
+          <t>0.847</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Competent Senior Data Scientist (5.3 YoE), matching key job requirements like PyTorch, Vector Search, Python. Good overall behavioral signals.</t>
+          <t>Solid fit: Senior Machine Learning Engineer at Zomato with 7.2 years experience. Recent role: Senior Machine Learning Engineer at Zomato. Matched JD skills: Pinecone, Information Retrieval, Milvus, RAG. Redrob signals: 61% recruiter response rate; 15-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0033861</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -831,19 +831,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.8052</t>
+          <t>0.8334</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Solid candidate working as Lead AI Engineer with 8.6 years in the field, matching key job requirements like Vector Search, NLP, MLOps, though platform response rate is lower (11%).</t>
+          <t>Solid fit: Senior NLP Engineer at Mad Street Den with 8.0 years experience. Recent role: Senior NLP Engineer at Mad Street Den. Matched JD skills: TensorFlow, Pinecone, Vector Search, Milvus. Redrob signals: 16% recruiter response rate; 30-day notice period. Concerns: low recruiter engagement.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0095528</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -853,19 +853,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.7895</t>
+          <t>0.8021</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior AI Engineer with 5.9 years in the field, matching key job requirements like Python, PyTorch, note the longer notice period of 90 days.</t>
+          <t>Solid fit: Senior Data Scientist at Netflix with 5.3 years experience. Recent role: Senior Data Scientist at Netflix. Matched JD skills: PyTorch, Vector Search, LLM Fine-tuning, Python. Redrob signals: 55% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -875,19 +875,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.7865</t>
+          <t>0.7983</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (5.7 YoE), who brings relevant experience in Information Retrieval, PyTorch, Python. Good overall behavioral signals.</t>
+          <t>Solid fit: Senior AI Engineer at Adobe with 5.9 years experience. Recent role: Senior AI Engineer at Adobe. Matched JD skills: Python, PyTorch, Information Retrieval. Redrob signals: 81% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -897,19 +897,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.7793</t>
+          <t>0.7946</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (16.9 YoE), with matching skills in Information Retrieval, FAISS, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Solid fit: Applied ML Engineer at Haptik with 14.1 years experience. Recent role: Applied ML Engineer at Haptik. Matched JD skills: PyTorch, NLP, Embeddings, Pinecone. Redrob signals: 87% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -919,19 +919,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.7786</t>
+          <t>0.7899</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Competent Applied ML Engineer (14.1 YoE), matching key job requirements like PyTorch, NLP, Embeddings, note the longer notice period of 90 days.</t>
+          <t>Solid fit: AI Engineer at CRED with 16.9 years experience. Recent role: AI Engineer at CRED. Matched JD skills: Information Retrieval, FAISS, RAG, Embeddings. Redrob signals: 72% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -941,12 +941,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.7706</t>
+          <t>0.7889</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Strong Lead AI Engineer with 6.4 years of experience, who brings relevant experience in Python, Ranking Systems, NLP. Good overall behavioral signals.</t>
+          <t>Solid fit: AI Engineer at Microsoft with 5.7 years experience. Recent role: AI Engineer at Microsoft. Matched JD skills: Information Retrieval, PyTorch, Python, NLP. Redrob signals: 94% recruiter response rate; 30-day notice period.</t>
         </is>
       </c>
     </row>
@@ -963,19 +963,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.7556</t>
+          <t>0.7724</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
+          <t>Solid fit: Senior Data Scientist at Niramai with 7.8 years experience. Recent role: Senior Data Scientist at Niramai. Matched JD skills: RAG, TensorFlow, Vector Search, LLM Fine-tuning. Redrob signals: 48% recruiter response rate; 15-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0083307</t>
+          <t>CAND_0030468</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -985,19 +985,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.752</t>
+          <t>0.7653</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 7.8 years in the field, matching key job requirements like Embeddings, Pinecone, Python, note the longer notice period of 120 days.</t>
+          <t>Solid fit: Senior Applied Scientist at Swiggy with 5.4 years experience. Recent role: Senior Applied Scientist at Swiggy. Matched JD skills: Information Retrieval, TensorFlow, Ranking Systems, Milvus. Redrob signals: 78% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0064326</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1007,12 +1007,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.7494</t>
+          <t>0.7618</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 7.6 years in the field, matching key job requirements like PyTorch, Milvus, RAG. Good overall behavioral signals.</t>
+          <t>Solid fit: AI Engineer at Zoho with 5.8 years experience. Recent role: AI Engineer at Zoho. Matched JD skills: MLOps, NLP, FAISS, LLM Fine-tuning. Redrob signals: 57% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
@@ -1029,19 +1029,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.7421</t>
+          <t>0.7597</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 5.3 YoE, who brings relevant experience in Milvus, Embeddings, Vector Search. Good overall behavioral signals.</t>
+          <t>Solid fit: Senior Data Scientist at Razorpay with 5.3 years experience. Recent role: Senior Data Scientist at Razorpay. Matched JD skills: Milvus, Embeddings, Vector Search. Redrob signals: 66% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0083307</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1051,12 +1051,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.7379</t>
+          <t>0.7566</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
+          <t>Solid fit: Search Engineer at CRED with 7.8 years experience. Recent role: Search Engineer at CRED. Matched JD skills: Embeddings, Pinecone, Python, Vector Search. Redrob signals: 70% recruiter response rate; 120-day notice period; open to work. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
@@ -1073,19 +1073,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.7328</t>
+          <t>0.7367</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Strong Recommendation Systems Engineer with 6.0 years of experience, matching key job requirements like FAISS, MLOps, Embeddings. Good overall behavioral signals.</t>
+          <t>Solid fit: Recommendation Systems Engineer at CRED with 6.0 years experience. Recent role: Recommendation Systems Engineer at CRED. Matched JD skills: FAISS, MLOps, Embeddings, Vector Search. Redrob signals: 90% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1095,19 +1095,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.7288</t>
+          <t>0.7328</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Solid fit: Lead AI Engineer at Sarvam AI with 6.4 years experience. Recent role: Lead AI Engineer at Sarvam AI. Matched JD skills: Python, Ranking Systems, Information Retrieval, NLP. Redrob signals: 86% recruiter response rate; 0-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0032515</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1117,19 +1117,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.7286</t>
+          <t>0.732</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 6.7 years in the field, with matching skills in Embeddings, TensorFlow, Information Retrieval and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Machine Learning Engineer at PharmEasy with 5.1 years experience. Recent role: Machine Learning Engineer at PharmEasy. Matched JD skills: Milvus, Vector Search, LLM Fine-tuning, NLP. Redrob signals: 54% recruiter response rate; 45-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0032515</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1139,19 +1139,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.727</t>
+          <t>0.7299</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Strong Machine Learning Engineer with 5.1 years of experience, who brings relevant experience in Milvus, Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Machine Learning Engineer at Genpact AI with 7.2 years experience. Recent role: Machine Learning Engineer at Genpact AI. Matched JD skills: RAG, FAISS, Embeddings, PyTorch. Redrob signals: 60% recruiter response rate; 120-day notice period; open to work. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1161,19 +1161,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.7221</t>
+          <t>0.7281</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Solid candidate working as Machine Learning Engineer with 7.2 years in the field, matching key job requirements like RAG, FAISS, Embeddings, note the longer notice period of 120 days.</t>
+          <t>Qualified but not ideal: AI Engineer at Microsoft with 6.9 years experience. Recent role: AI Engineer at Microsoft. Matched JD skills: Python, Vector Search. Redrob signals: 81% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0049896</t>
+          <t>CAND_0093763</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1183,19 +1183,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.7215</t>
+          <t>0.7275</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (7.3 YoE), with matching skills in PyTorch, Information Retrieval, NLP and solid backend fundamentals, note the longer notice period of 90 days.</t>
+          <t>Qualified but not ideal: Senior Software Engineer (ML) at Swiggy with 5.0 years experience. Recent role: Senior Software Engineer (ML) at Swiggy. Matched JD skills: FAISS, Vector Search, PyTorch, TensorFlow. Redrob signals: 92% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0052682</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.7213</t>
+          <t>0.7249</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 6.9 years in the field, matching key job requirements like Python, Vector Search. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: NLP Engineer at Aganitha with 6.6 years experience. Recent role: NLP Engineer at Aganitha. Matched JD skills: FAISS, PyTorch, Python, Embeddings. Redrob signals: 88% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0024620</t>
+          <t>CAND_0098454</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1227,19 +1227,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.7176</t>
+          <t>0.7245</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (5.9 YoE), possessing practical experience in Information Retrieval, Python. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: AI Specialist at Meesho with 6.6 years experience. Recent role: AI Specialist at Meesho. Matched JD skills: Vector Search, MLOps, NLP, Pinecone. Redrob signals: 87% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0052682</t>
+          <t>CAND_0024620</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.7165</t>
+          <t>0.724</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Strong NLP Engineer with 6.6 years of experience, who brings relevant experience in FAISS, PyTorch, Python. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: AI Engineer at PharmEasy with 5.9 years experience. Recent role: AI Engineer at PharmEasy. Matched JD skills: Information Retrieval, Python. Redrob signals: 41% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0070525</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1271,19 +1271,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.7123</t>
+          <t>0.7208</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Strong Senior Software Engineer (ML) with 5.4 years of experience, who brings relevant experience in Python, Embeddings. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Senior Data Scientist at Google with 6.5 years experience. Recent role: Senior Data Scientist at Google. Matched JD skills: Milvus, TensorFlow, Python. Redrob signals: 72% recruiter response rate; 120-day notice period; open to work. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0010685</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1293,19 +1293,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.7084</t>
+          <t>0.719</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Solid candidate working as NLP Engineer with 6.7 years in the field, with matching skills in PyTorch, Information Retrieval, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: AI Engineer at Google with 7.3 years experience. Recent role: AI Engineer at Google. Matched JD skills: Pinecone, Vector Search, RAG, Information Retrieval. Redrob signals: 78% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
+          <t>CAND_0059795</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1315,19 +1315,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.7071</t>
+          <t>0.7183</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 5.8 years in the field, matching key job requirements like MLOps, NLP, FAISS. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Senior Software Engineer (ML) at Locobuzz with 5.6 years experience. Recent role: Senior Software Engineer (ML) at Locobuzz. Matched JD skills: Python. Redrob signals: 75% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1337,19 +1337,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.7069</t>
+          <t>0.7174</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 7.3 years in the field, matching key job requirements like Pinecone, Vector Search, RAG. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Senior Data Scientist at Flipkart with 6.6 years experience. Recent role: Senior Data Scientist at Flipkart. Matched JD skills: Information Retrieval, Pinecone, Vector Search, NLP. Redrob signals: 56% recruiter response rate; 60-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0030468</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1359,19 +1359,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.7037</t>
+          <t>0.7135</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Applied Scientist with 5.4 years in the field, matching key job requirements like TensorFlow, Ranking Systems, Milvus. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: AI Engineer at PolicyBazaar with 7.7 years experience. Recent role: AI Engineer at PolicyBazaar. Matched JD skills: Vector Search, NLP, LLM Fine-tuning. Redrob signals: 60% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0064326</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1381,19 +1381,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.7003</t>
+          <t>0.7127</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 6.5 years in the field, matching key job requirements like Milvus, TensorFlow, Python, note the longer notice period of 120 days.</t>
+          <t>Qualified but not ideal: Search Engineer at Sarvam AI with 7.6 years experience. Recent role: Search Engineer at Sarvam AI. Matched JD skills: PyTorch, Milvus, RAG, Python. Redrob signals: 94% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0081686</t>
+          <t>CAND_0010685</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1403,19 +1403,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>0.7112</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (6.0 YoE), matching key job requirements like Embeddings, FAISS, Milvus. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: NLP Engineer at Rephrase.ai with 6.7 years experience. Recent role: NLP Engineer at Rephrase.ai. Matched JD skills: PyTorch, Information Retrieval, RAG. Redrob signals: 83% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0012837</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1425,19 +1425,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.6997</t>
+          <t>0.7101</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Solid candidate working as Staff Machine Learning Engineer with 8.8 years in the field, matching key job requirements like MLOps, Python, Milvus. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Junior ML Engineer at Sarvam AI with 6.4 years experience. Recent role: Junior ML Engineer at Sarvam AI. Matched JD skills: Vector Search, MLOps, NLP. Redrob signals: 81% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0096172</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1447,19 +1447,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.6963</t>
+          <t>0.7085</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Solid candidate working as NLP Engineer with 5.2 years in the field, with matching skills in Python, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: AI Engineer at Rephrase.ai with 6.8 years experience. Recent role: AI Engineer at Rephrase.ai. Matched JD skills: PyTorch, LLM Fine-tuning, FAISS, NLP. Redrob signals: 77% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0058412</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.6949</t>
+          <t>0.7065</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Software Engineer (ML) with 6.6 years in the field, with matching skills in Embeddings, Milvus, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Senior Machine Learning Engineer at Niramai with 7.9 years experience. Recent role: Senior Machine Learning Engineer at Niramai. Matched JD skills: Ranking Systems, TensorFlow, Information Retrieval. Redrob signals: 61% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0025882</t>
+          <t>CAND_0077285</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1491,19 +1491,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.6942</t>
+          <t>0.7049</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Software Engineer (ML) with 5.6 years in the field, with matching skills in FAISS, Vector Search, Milvus and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Recommendation Systems Engineer at Nykaa with 5.5 years experience. Recent role: Recommendation Systems Engineer at Nykaa. Matched JD skills: Pinecone, Embeddings, Information Retrieval, LLM Fine-tuning. Redrob signals: 56% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.6939</t>
+          <t>0.7031</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (6.8 YoE), matching key job requirements like PyTorch, FAISS, NLP. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Senior Applied Scientist at Niramai with 9.0 years experience. Recent role: Senior Applied Scientist at Niramai. Matched JD skills: PyTorch, NLP, Information Retrieval. Redrob signals: 63% recruiter response rate; 0-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0077285</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1535,19 +1535,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.6911</t>
+          <t>0.7022</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Applied ML Engineer at Saarthi.ai with 5.8 years experience. Recent role: Applied ML Engineer at Saarthi.ai. Matched JD skills: Vector Search, Milvus, Embeddings, PyTorch. Redrob signals: 72% recruiter response rate; 30-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1557,19 +1557,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.6896</t>
+          <t>0.701</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
+          <t>Qualified but not ideal: Staff Machine Learning Engineer at Salesforce with 8.8 years experience. Recent role: Staff Machine Learning Engineer at Salesforce. Matched JD skills: MLOps, Information Retrieval, Python, Milvus. Redrob signals: 66% recruiter response rate; 0-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0043860</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1579,19 +1579,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.6888</t>
+          <t>0.7002</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
+          <t>Qualified but not ideal: AI Engineer at Vedantu with 6.7 years experience. Recent role: AI Engineer at Vedantu. Matched JD skills: Embeddings, TensorFlow, Information Retrieval, Milvus. Redrob signals: 74% recruiter response rate; 15-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1601,19 +1601,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.6848</t>
+          <t>0.6942</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Candidate with 7.2 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, Information Retrieval, PyTorch; moderate fit with some technical gaps for this senior role.</t>
+          <t>Qualified but not ideal: Recommendation Systems Engineer at upGrad with 5.8 years experience. Recent role: Recommendation Systems Engineer at upGrad. Matched JD skills: FAISS, Vector Search, Milvus, Pinecone. Redrob signals: 75% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1623,19 +1623,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.6825</t>
+          <t>0.6933</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Qualified but not ideal: Search Engineer at Google with 7.2 years experience. Recent role: Search Engineer at Google. Matched JD skills: Embeddings, Information Retrieval, PyTorch, NLP. Redrob signals: 56% recruiter response rate; 120-day notice period; open to work. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0029367</t>
+          <t>CAND_0012632</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1645,19 +1645,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.6815</t>
+          <t>0.6914</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
+          <t>Qualified but not ideal: AI Specialist at Razorpay with 6.0 years experience. Recent role: AI Specialist at Razorpay. Matched JD skills: MLOps, Python, Pinecone, Vector Search. Redrob signals: 53% recruiter response rate; 120-day notice period. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0098454</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1667,12 +1667,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.681</t>
+          <t>0.6912</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Qualified but not ideal: Senior Data Scientist at Microsoft with 7.0 years experience. Recent role: Senior Data Scientist at Microsoft. Matched JD skills: MLOps, Milvus, RAG, Information Retrieval. Redrob signals: 49% recruiter response rate; 90-day notice period. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.6807</t>
+          <t>0.6897</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Recommendation Systems Engineer (7.9 YoE), having some background in Python, Embeddings but less specialized; included as potential pipeline filler.</t>
+          <t>Qualified but not ideal: Recommendation Systems Engineer at Wysa with 7.9 years experience. Recent role: Recommendation Systems Engineer at Wysa. Matched JD skills: Python, Embeddings. Redrob signals: 62% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1711,19 +1711,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.6801</t>
+          <t>0.6895</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Qualified but not ideal: Senior Data Scientist at Sarvam AI with 7.4 years experience. Recent role: Senior Data Scientist at Sarvam AI. Matched JD skills: TensorFlow, LLM Fine-tuning, RAG, Information Retrieval. Redrob signals: 56% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0012837</t>
+          <t>CAND_0000031</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1733,19 +1733,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.6793</t>
+          <t>0.6876</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.4 YoE as Junior ML Engineer, mostly showing adjacent skills like Vector Search, MLOps, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Qualified but not ideal: Recommendation Systems Engineer at Swiggy with 6.0 years experience. Recent role: Recommendation Systems Engineer at Swiggy. Matched JD skills: FAISS, Pinecone, MLOps, Embeddings. Redrob signals: 91% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0049896</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1755,19 +1755,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.679</t>
+          <t>0.6858</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Qualified but not ideal: Search Engineer at Unacademy with 7.3 years experience. Recent role: Search Engineer at Unacademy. Matched JD skills: PyTorch, Information Retrieval, LLM Fine-tuning, NLP. Redrob signals: 43% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0099401</t>
+          <t>CAND_0007567</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1777,19 +1777,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.6777</t>
+          <t>0.6849</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: AI Specialist at Niramai with 6.1 years experience. Recent role: AI Specialist at Niramai. Matched JD skills: LLM Fine-tuning, NLP, MLOps, FAISS. Redrob signals: 80% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0081686</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1799,19 +1799,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.675</t>
+          <t>0.6831</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
+          <t>Marginal fit: Search Engineer at Netflix with 6.0 years experience. Recent role: Search Engineer at Netflix. Matched JD skills: Embeddings, FAISS, Milvus, Python. Redrob signals: 91% recruiter response rate; 60-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0061265</t>
+          <t>CAND_0041402</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1821,19 +1821,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.6748</t>
+          <t>0.6798</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
+          <t>Marginal fit: AI Specialist at Ola with 6.3 years experience. Recent role: AI Specialist at Ola. Matched JD skills: Information Retrieval, RAG, Vector Search. Redrob signals: 44% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0006557</t>
+          <t>CAND_0017960</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1843,19 +1843,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.6714</t>
+          <t>0.6794</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Recommendation Systems Engineer at Nykaa with 7.7 years experience. Recent role: Recommendation Systems Engineer at Nykaa. Matched JD skills: Python, Information Retrieval. Redrob signals: 72% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0027801</t>
+          <t>CAND_0095619</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1865,19 +1865,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.6712</t>
+          <t>0.6792</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Candidate with 7.4 years experience as NLP Engineer, mostly showing adjacent skills like FAISS, Milvus, TensorFlow; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Marginal fit: NLP Engineer at Nykaa with 15.6 years experience. Recent role: NLP Engineer at Nykaa. Matched JD skills: Pinecone, NLP, Information Retrieval, LLM Fine-tuning. Redrob signals: 90% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0000031</t>
+          <t>CAND_0027801</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1887,19 +1887,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.6703</t>
+          <t>0.6788</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 6.0 years of background, possessing partial overlap in FAISS, Pinecone, MLOps; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: NLP Engineer at InMobi with 7.4 years experience. Recent role: NLP Engineer at InMobi. Matched JD skills: FAISS, Milvus, TensorFlow, MLOps. Redrob signals: 65% recruiter response rate; 120-day notice period; open to work. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.6693</t>
+          <t>0.6752</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Staff Machine Learning Engineer at LinkedIn with 8.0 years experience. Recent role: Staff Machine Learning Engineer at LinkedIn. Matched JD skills: Information Retrieval, Python. Redrob signals: 87% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0041402</t>
+          <t>CAND_0065195</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1931,19 +1931,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.6666</t>
+          <t>0.6748</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Candidate with 6.3 years experience as AI Specialist, mostly showing adjacent skills like Information Retrieval, RAG, Vector Search; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Search Engineer at CRED with 5.1 years experience. Recent role: Search Engineer at CRED. Matched JD skills: MLOps. Redrob signals: 80% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0006557</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1953,19 +1953,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.665</t>
+          <t>0.6738</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: NLP Engineer at Paytm with 7.9 years experience. Recent role: NLP Engineer at Paytm. Matched JD skills: Vector Search, FAISS, Pinecone, Information Retrieval. Redrob signals: 63% recruiter response rate; 120-day notice period; open to work. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0017960</t>
+          <t>CAND_0036121</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1975,19 +1975,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.6646</t>
+          <t>0.6728</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Recommendation Systems Engineer (7.7 YoE), having some background in Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: ML Engineer at Wysa with 5.2 years experience. Recent role: ML Engineer at Wysa. Matched JD skills: Embeddings, Vector Search, Information Retrieval. Redrob signals: 49% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0064256</t>
+          <t>CAND_0070202</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1997,19 +1997,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.6623</t>
+          <t>0.6728</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Machine Learning Engineer at BYJU'S with 5.1 years experience. Recent role: Machine Learning Engineer at BYJU'S. Matched JD skills: Embeddings, LLM Fine-tuning, PyTorch, RAG. Redrob signals: 60% recruiter response rate; 90-day notice period. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0070202</t>
+          <t>CAND_0064256</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2019,19 +2019,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.6615</t>
+          <t>0.6714</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Candidate with 5.1 years experience as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, PyTorch, RAG; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Junior ML Engineer at BYJU'S with 6.4 years experience. Recent role: Junior ML Engineer at BYJU'S. Matched JD skills: PyTorch, MLOps, Python, Embeddings. Redrob signals: 86% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0015967</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2041,19 +2041,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.6561</t>
+          <t>0.6711</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: Senior Software Engineer (ML) at Razorpay with 5.4 years experience. Recent role: Senior Software Engineer (ML) at Razorpay. Matched JD skills: Pinecone, TensorFlow, Embeddings. Redrob signals: 45% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0051630</t>
+          <t>CAND_0092568</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2063,19 +2063,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.6558</t>
+          <t>0.6702</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
+          <t>Marginal fit: AI Specialist at TCS with 5.7 years experience. Recent role: AI Specialist at TCS. Matched JD skills: Vector Search, Milvus, Python, Pinecone. Redrob signals: 39% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0095619</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2085,19 +2085,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.654</t>
+          <t>0.669</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Marginal fit: Senior Data Scientist at Rephrase.ai with 5.7 years experience. Recent role: Senior Data Scientist at Rephrase.ai. Matched JD skills: TensorFlow, FAISS, RAG, NLP. Redrob signals: 77% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0087006</t>
+          <t>CAND_0077498</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.6531</t>
+          <t>0.6688</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: Senior Software Engineer (ML) at Niramai with 5.4 years experience. Recent role: Senior Software Engineer (ML) at Niramai. Matched JD skills: Embeddings, Milvus. Redrob signals: 89% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0030953</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.6512</t>
+          <t>0.6669</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.8 YoE as Search Engineer, possessing partial overlap in MLOps, Python, RAG; included as potential pipeline filler.</t>
+          <t>Marginal fit: Applied ML Engineer at Freshworks with 5.2 years experience. Recent role: Applied ML Engineer at Freshworks. Matched JD skills: FAISS, Vector Search, LLM Fine-tuning, NLP. Redrob signals: 52% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0073883</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2151,19 +2151,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.6473</t>
+          <t>0.6649</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Marginal fit: AI Specialist at Krutrim with 5.3 years experience. Recent role: AI Specialist at Krutrim. Matched JD skills: Vector Search, Python, FAISS. Redrob signals: 92% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0065195</t>
+          <t>CAND_0030953</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2173,19 +2173,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.6423</t>
+          <t>0.6613</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Search Engineer with 5.1 years of background, with limited direct exposure to search/ranking but lists MLOps; included as potential pipeline filler.</t>
+          <t>Marginal fit: Search Engineer at Nykaa with 7.8 years experience. Recent role: Search Engineer at Nykaa. Matched JD skills: MLOps, Python, RAG. Redrob signals: 63% recruiter response rate; 45-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0018722</t>
+          <t>CAND_0067866</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2195,19 +2195,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.6418</t>
+          <t>0.6597</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Python, TensorFlow; included as potential pipeline filler.</t>
+          <t>Marginal fit: Senior Software Engineer (ML) at Tech Mahindra with 6.4 years experience. Recent role: Senior Software Engineer (ML) at Tech Mahindra. Matched JD skills: Embeddings. Redrob signals: 79% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
+          <t>CAND_0076163</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2217,19 +2217,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.6404</t>
+          <t>0.6547</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 8.0 years of background, having some background in Vector Search, TensorFlow, Embeddings but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: NLP Engineer at Ola with 6.9 years experience. Recent role: NLP Engineer at Ola. Matched JD skills: PyTorch, Python, MLOps. Redrob signals: 84% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0076163</t>
+          <t>CAND_0006418</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2239,19 +2239,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.6381</t>
+          <t>0.6528</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (6.9 YoE), having some background in PyTorch, Python, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Machine Learning Engineer at Verloop.io with 5.7 years experience. Recent role: Machine Learning Engineer at Verloop.io. Matched JD skills: Embeddings, TensorFlow. Redrob signals: 92% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2261,19 +2261,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.6362</t>
+          <t>0.651</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.0 YoE), mostly showing adjacent skills like Pinecone, Python, RAG; included as potential pipeline filler.</t>
+          <t>Marginal fit: Applied ML Engineer at Freshworks with 8.0 years experience. Recent role: Applied ML Engineer at Freshworks. Matched JD skills: Vector Search, TensorFlow, Embeddings, Pinecone. Redrob signals: 42% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0053591</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2283,19 +2283,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.6354</t>
+          <t>0.6475</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Alternative profile showing 8.0 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like Python; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: AI Engineer at Ola with 5.3 years experience. Recent role: AI Engineer at Ola. Matched JD skills: Embeddings, Milvus, RAG. Redrob signals: 81% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0067866</t>
+          <t>CAND_0074735</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2305,19 +2305,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.6342</t>
+          <t>0.646</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.4 years of background, possessing partial overlap in Embeddings; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Applied ML Engineer at Rephrase.ai with 5.5 years experience. Recent role: Applied ML Engineer at Rephrase.ai. Matched JD skills: RAG, Information Retrieval, Vector Search, TensorFlow. Redrob signals: 77% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2327,19 +2327,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.6339</t>
+          <t>0.6446</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Marginal fit: Recommendation Systems Engineer at CRED with 8.0 years experience. Recent role: Recommendation Systems Engineer at CRED. Matched JD skills: FAISS, Milvus, MLOps, Information Retrieval. Redrob signals: 77% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0049978</t>
+          <t>CAND_0082086</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.6296</t>
+          <t>0.6426</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.6 years of background, with limited direct exposure to search/ranking but lists PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Marginal fit: Senior Software Engineer (ML) at Razorpay with 6.0 years experience. Recent role: Senior Software Engineer (ML) at Razorpay. Matched JD skills: FAISS, Pinecone, PyTorch, Milvus. Redrob signals: 85% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0024466</t>
+          <t>CAND_0049978</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2371,19 +2371,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.6289</t>
+          <t>0.6422</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Marginal fit: Senior Software Engineer (ML) at Sarvam AI with 6.6 years experience. Recent role: Senior Software Engineer (ML) at Sarvam AI. Matched JD skills: PyTorch, Embeddings. Redrob signals: 71% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0074735</t>
+          <t>CAND_0073314</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2393,19 +2393,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.6287</t>
+          <t>0.6415</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 5.5 years of background, with limited direct exposure to search/ranking but lists RAG, Information Retrieval, Vector Search; included as potential pipeline filler.</t>
+          <t>Marginal fit: Senior Software Engineer (ML) at Aganitha with 5.2 years experience. Recent role: Senior Software Engineer (ML) at Aganitha. Matched JD skills: Milvus, PyTorch, MLOps. Redrob signals: 84% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0044883</t>
+          <t>CAND_0024466</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2415,19 +2415,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.626</t>
+          <t>0.641</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
+          <t>Marginal fit: Search Engineer at PharmEasy with 5.2 years experience. Recent role: Search Engineer at PharmEasy. Matched JD skills: MLOps, LLM Fine-tuning, NLP, Pinecone. Redrob signals: 47% recruiter response rate; 120-day notice period; open to work. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0040117</t>
+          <t>CAND_0033842</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2437,19 +2437,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.6231</t>
+          <t>0.641</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Candidate with 6.5 years experience as Recommendation Systems Engineer, with limited direct exposure to search/ranking but lists Embeddings, RAG, FAISS; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: Senior Software Engineer (ML) at Rephrase.ai with 5.8 years experience. Recent role: Senior Software Engineer (ML) at Rephrase.ai. Matched JD skills: MLOps, NLP, Pinecone. Redrob signals: 34% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
+          <t>CAND_0024878</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2459,19 +2459,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.6213</t>
+          <t>0.6409</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 8.0 years of background, with limited direct exposure to search/ranking but lists FAISS, Milvus, MLOps; included as potential pipeline filler.</t>
+          <t>Marginal fit: AI Specialist at HCL with 5.7 years experience. Recent role: AI Specialist at HCL. Matched JD skills: NLP, MLOps, Information Retrieval. Redrob signals: 84% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0049771</t>
+          <t>CAND_0070514</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2481,19 +2481,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.6192</t>
+          <t>0.6399</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), with limited direct exposure to search/ranking but lists Python, PyTorch, MLOps; included as potential pipeline filler.</t>
+          <t>Marginal fit: AI Specialist at Glance with 5.5 years experience. Recent role: AI Specialist at Glance. Matched JD skills: Pinecone, Python, MLOps, FAISS. Redrob signals: 80% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0093331</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2503,19 +2503,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.6147</t>
+          <t>0.639</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (16.1 YoE), having some background in PyTorch, Embeddings, Milvus but less specialized; included as potential pipeline filler.</t>
+          <t>Marginal fit: Senior Data Scientist at Flipkart with 6.5 years experience. Recent role: Senior Data Scientist at Flipkart. Matched JD skills: PyTorch, NLP, RAG, Embeddings. Redrob signals: 67% recruiter response rate; 45-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0082086</t>
+          <t>CAND_0072660</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2525,19 +2525,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.6145</t>
+          <t>0.6384</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.0 years of background, having some background in FAISS, Pinecone, PyTorch but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Machine Learning Engineer at Unacademy with 7.1 years experience. Recent role: Machine Learning Engineer at Unacademy. Matched JD skills: PyTorch, Information Retrieval, FAISS, Python. Redrob signals: 53% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0078508</t>
+          <t>CAND_0016657</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2547,19 +2547,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.6134</t>
+          <t>0.6355</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.2 YoE), with limited direct exposure to search/ranking but lists Embeddings, NLP; included as potential pipeline filler.</t>
+          <t>Marginal fit: AI Research Engineer at PhonePe with 5.3 years experience. Recent role: AI Research Engineer at PhonePe. Matched JD skills: PyTorch, MLOps, TensorFlow, Vector Search. Redrob signals: 52% recruiter response rate; 60-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0072660</t>
+          <t>CAND_0010770</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.6133</t>
+          <t>0.6347</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.1 YoE as Machine Learning Engineer, mostly showing adjacent skills like PyTorch, Information Retrieval, FAISS; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: Recommendation Systems Engineer at Aganitha with 15.2 years experience. Recent role: Recommendation Systems Engineer at Aganitha. Matched JD skills: TensorFlow, MLOps. Redrob signals: 73% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0050707</t>
+          <t>CAND_0044883</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2591,19 +2591,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.6129</t>
+          <t>0.6342</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Specialist (5.3 YoE), having some background in RAG, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Marginal fit: AI Engineer at Mad Street Den with 6.3 years experience. Recent role: AI Engineer at Mad Street Den. Matched JD skills: Embeddings, LLM Fine-tuning, TensorFlow, PyTorch. Redrob signals: 84% recruiter response rate; 90-day notice period. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0093883</t>
+          <t>CAND_0040117</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2613,19 +2613,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.6121</t>
+          <t>0.6335</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), possessing partial overlap in Embeddings, MLOps, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Recommendation Systems Engineer at PhonePe with 6.5 years experience. Recent role: Recommendation Systems Engineer at PhonePe. Matched JD skills: Embeddings, RAG, FAISS. Redrob signals: 66% recruiter response rate; 15-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0007567</t>
+          <t>CAND_0078508</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2635,12 +2635,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.6118</t>
+          <t>0.6334</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.1 YoE as AI Specialist, possessing partial overlap in NLP, MLOps, FAISS; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: AI Research Engineer at Rephrase.ai with 5.2 years experience. Recent role: AI Research Engineer at Rephrase.ai. Matched JD skills: Embeddings, NLP, LLM Fine-tuning. Redrob signals: 34% recruiter response rate; 30-day notice period.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: apply visual display fixes, memory optimizations and update contact number
</commit_message>
<xml_diff>
--- a/outputs/mohd_ibadullah.xlsx
+++ b/outputs/mohd_ibadullah.xlsx
@@ -457,12 +457,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.994</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Outstanding candidate as Senior Machine Learning Engineer showing 8.1 years of experience, shows deep technical expertise in Python, Information Retrieval, Embeddings and search infrastructure. Highly active on Redrob with a 87% recruiter response rate.</t>
+          <t>Strong top-tier match: Senior Machine Learning Engineer at Flipkart with 8.1 years experience. Recent role: Senior Machine Learning Engineer at Flipkart. Matched JD skills: Python, LLM Fine-tuning, Information Retrieval, Embeddings. Redrob signals: 87% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
@@ -479,12 +479,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.9617</t>
+          <t>0.9554</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Top-tier candidate currently working as Senior Applied Scientist (5.3 YoE), demonstrates strong proficiency in Vector Search, Pinecone, Embeddings and alignment with the JD. Available quickly with a short notice period of 0 days.</t>
+          <t>Strong top-tier match: Senior Applied Scientist at Sarvam AI with 5.3 years experience. Recent role: Senior Applied Scientist at Sarvam AI. Matched JD skills: Vector Search, LLM Fine-tuning, Pinecone, Embeddings. Redrob signals: 55% recruiter response rate; 0-day notice period; open to work.</t>
         </is>
       </c>
     </row>
@@ -501,12 +501,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.9568</t>
+          <t>0.9501</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Top-tier candidate currently working as Senior NLP Engineer (5.2 YoE), offers solid expertise in MLOps, Information Retrieval, Python which matches the core ranking mandate. Excellent platform engagement with 86% response rate.</t>
+          <t>Strong top-tier match: Senior NLP Engineer at Netflix with 5.2 years experience. Recent role: Senior NLP Engineer at Netflix. Matched JD skills: MLOps, Information Retrieval, Python, NLP. Redrob signals: 86% recruiter response rate; 60-day notice period.</t>
         </is>
       </c>
     </row>
@@ -523,19 +523,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.9388</t>
+          <t>0.9441</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Highly relevant Senior AI Engineer with 5.9 years of background, offers solid expertise in FAISS, TensorFlow, NLP which matches the core ranking mandate. Excellent platform engagement with 80% response rate.</t>
+          <t>Strong top-tier match: Senior AI Engineer at Apple with 5.9 years experience. Recent role: Senior AI Engineer at Apple. Matched JD skills: FAISS, TensorFlow, NLP, Pinecone. Redrob signals: 80% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0011687</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -545,19 +545,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.9221</t>
+          <t>0.905</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in TensorFlow, FAISS, Embeddings and search infrastructure. Available quickly with a short notice period of 15 days.</t>
+          <t>Strong top-tier match: Senior AI Engineer at Netflix with 7.8 years experience. Recent role: Senior AI Engineer at Netflix. Matched JD skills: Pinecone, Information Retrieval, Embeddings, RAG. Redrob signals: 76% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -567,19 +567,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.9179</t>
+          <t>0.9039</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Highly relevant Lead AI Engineer with 6.7 years of background, demonstrates strong proficiency in Information Retrieval, PyTorch, Vector Search and alignment with the JD. Highly active on Redrob with a 73% recruiter response rate.</t>
+          <t>Strong top-tier match: Senior NLP Engineer at Salesforce with 8.9 years experience. Recent role: Senior NLP Engineer at Salesforce. Matched JD skills: Python, Pinecone. Redrob signals: 78% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0046064</t>
+          <t>CAND_0008425</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -589,19 +589,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.9127</t>
+          <t>0.9018</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Highly relevant Senior NLP Engineer with 8.9 years of background, has successfully deployed systems involving Python, Pinecone at scale. Highly active on Redrob with a 78% recruiter response rate.</t>
+          <t>Strong top-tier match: Senior NLP Engineer at Ola with 7.8 years experience. Recent role: Senior NLP Engineer at Ola. Matched JD skills: NLP, TensorFlow, Python, Information Retrieval. Redrob signals: 66% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0039754</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.9086</t>
+          <t>0.8957</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Exceptional Senior AI Engineer offering 7.8 years of experience, offers solid expertise in Pinecone, Information Retrieval, Embeddings which matches the core ranking mandate. Highly active on Redrob with a 76% recruiter response rate.</t>
+          <t>Strong top-tier match: Senior Applied Scientist at Meta with 16.2 years experience. Recent role: Senior Applied Scientist at Meta. Matched JD skills: LLM Fine-tuning, NLP, Python, TensorFlow. Redrob signals: 81% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0008425</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -633,19 +633,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.9083</t>
+          <t>0.877</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Exceptional Senior NLP Engineer offering 7.8 years of experience, shows deep technical expertise in NLP, TensorFlow, Python and search infrastructure. Highly active on Redrob with a 66% recruiter response rate.</t>
+          <t>Strong top-tier match: Staff Machine Learning Engineer at Paytm with 7.0 years experience. Recent role: Staff Machine Learning Engineer at Paytm. Matched JD skills: Pinecone, Information Retrieval, RAG, Python. Redrob signals: 95% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -655,19 +655,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.8949</t>
+          <t>0.8726</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Exceptional Senior Machine Learning Engineer offering 6.1 years of experience, demonstrates strong proficiency in Information Retrieval, TensorFlow, NLP and alignment with the JD. Highly active on Redrob with a 88% recruiter response rate.</t>
+          <t>Strong top-tier match: Staff Machine Learning Engineer at Yellow.ai with 8.6 years experience. Recent role: Staff Machine Learning Engineer at Yellow.ai. Matched JD skills: Pinecone, RAG, TensorFlow, MLOps. Redrob signals: 83% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0039754</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -677,19 +677,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.8863</t>
+          <t>0.8722</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Exceptional Senior Applied Scientist offering 16.2 years of experience, offers solid expertise in NLP, Python, TensorFlow which matches the core ranking mandate. Highly active on Redrob with a 81% recruiter response rate.</t>
+          <t>Solid fit: Senior AI Engineer at Meta with 7.9 years experience. Recent role: Senior AI Engineer at Meta. Matched JD skills: NLP, Python, Ranking Systems. Redrob signals: 79% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -699,19 +699,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.8734</t>
+          <t>0.8696</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Highly relevant Staff Machine Learning Engineer with 7.0 years of background, demonstrates strong proficiency in Pinecone, Information Retrieval, RAG and alignment with the JD. Highly active on Redrob with a 95% recruiter response rate.</t>
+          <t>Solid fit: Senior Machine Learning Engineer at Genpact AI with 6.1 years experience. Recent role: Senior Machine Learning Engineer at Genpact AI. Matched JD skills: Information Retrieval, TensorFlow, NLP. Redrob signals: 88% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -721,19 +721,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.8682</t>
+          <t>0.868</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Exceptional Staff Machine Learning Engineer offering 8.6 years of experience, shows deep technical expertise in Pinecone, RAG, TensorFlow and search infrastructure. Highly active on Redrob with a 83% recruiter response rate.</t>
+          <t>Solid fit: Lead AI Engineer at Meta with 8.6 years experience. Recent role: Lead AI Engineer at Meta. Matched JD skills: LLM Fine-tuning, Vector Search, NLP, MLOps. Redrob signals: 11% recruiter response rate; 30-day notice period. Concerns: low recruiter engagement.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -743,19 +743,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.867</t>
+          <t>0.8653</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Exceptional Senior Machine Learning Engineer offering 7.2 years of experience, has successfully deployed systems involving Pinecone, Information Retrieval, Milvus at scale. Highly active on Redrob with a 61% recruiter response rate.</t>
+          <t>Solid fit: Lead AI Engineer at Razorpay with 6.7 years experience. Recent role: Lead AI Engineer at Razorpay. Matched JD skills: Information Retrieval, PyTorch, Vector Search, Python. Redrob signals: 73% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -765,19 +765,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.8666</t>
+          <t>0.8615</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Outstanding candidate as Senior AI Engineer showing 7.9 years of experience, shows deep technical expertise in NLP, Python, Ranking Systems and search infrastructure. Highly active on Redrob with a 79% recruiter response rate.</t>
+          <t>Solid fit: Senior NLP Engineer at Niramai with 7.8 years experience. Recent role: Senior NLP Engineer at Niramai. Matched JD skills: TensorFlow, FAISS, Embeddings, MLOps. Redrob signals: 89% recruiter response rate; 15-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0033861</t>
+          <t>CAND_0007411</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -787,19 +787,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.8573</t>
+          <t>0.8536</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior NLP Engineer with 8.0 years in the field, matching key job requirements like TensorFlow, Pinecone, Vector Search, though platform response rate is lower (16%).</t>
+          <t>Solid fit: Senior Machine Learning Engineer at Amazon with 8.0 years experience. Recent role: Senior Machine Learning Engineer at Amazon. Matched JD skills: LLM Fine-tuning, Vector Search, PyTorch, Information Retrieval. Redrob signals: 12% recruiter response rate; 15-day notice period. Concerns: low recruiter engagement.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0095528</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -809,19 +809,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.8355</t>
+          <t>0.847</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Competent Senior Data Scientist (5.3 YoE), matching key job requirements like PyTorch, Vector Search, Python. Good overall behavioral signals.</t>
+          <t>Solid fit: Senior Machine Learning Engineer at Zomato with 7.2 years experience. Recent role: Senior Machine Learning Engineer at Zomato. Matched JD skills: Pinecone, Information Retrieval, Milvus, RAG. Redrob signals: 61% recruiter response rate; 15-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0033861</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -831,19 +831,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.8052</t>
+          <t>0.8334</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Solid candidate working as Lead AI Engineer with 8.6 years in the field, matching key job requirements like Vector Search, NLP, MLOps, though platform response rate is lower (11%).</t>
+          <t>Solid fit: Senior NLP Engineer at Mad Street Den with 8.0 years experience. Recent role: Senior NLP Engineer at Mad Street Den. Matched JD skills: TensorFlow, Pinecone, Vector Search, Milvus. Redrob signals: 16% recruiter response rate; 30-day notice period. Concerns: low recruiter engagement.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0095528</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -853,19 +853,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.7895</t>
+          <t>0.8021</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior AI Engineer with 5.9 years in the field, matching key job requirements like Python, PyTorch, note the longer notice period of 90 days.</t>
+          <t>Solid fit: Senior Data Scientist at Netflix with 5.3 years experience. Recent role: Senior Data Scientist at Netflix. Matched JD skills: PyTorch, Vector Search, LLM Fine-tuning, Python. Redrob signals: 55% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -875,19 +875,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.7865</t>
+          <t>0.7983</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (5.7 YoE), who brings relevant experience in Information Retrieval, PyTorch, Python. Good overall behavioral signals.</t>
+          <t>Solid fit: Senior AI Engineer at Adobe with 5.9 years experience. Recent role: Senior AI Engineer at Adobe. Matched JD skills: Python, PyTorch, Information Retrieval. Redrob signals: 81% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -897,19 +897,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.7793</t>
+          <t>0.7946</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (16.9 YoE), with matching skills in Information Retrieval, FAISS, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Solid fit: Applied ML Engineer at Haptik with 14.1 years experience. Recent role: Applied ML Engineer at Haptik. Matched JD skills: PyTorch, NLP, Embeddings, Pinecone. Redrob signals: 87% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -919,19 +919,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.7786</t>
+          <t>0.7899</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Competent Applied ML Engineer (14.1 YoE), matching key job requirements like PyTorch, NLP, Embeddings, note the longer notice period of 90 days.</t>
+          <t>Solid fit: AI Engineer at CRED with 16.9 years experience. Recent role: AI Engineer at CRED. Matched JD skills: Information Retrieval, FAISS, RAG, Embeddings. Redrob signals: 72% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -941,12 +941,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.7706</t>
+          <t>0.7889</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Strong Lead AI Engineer with 6.4 years of experience, who brings relevant experience in Python, Ranking Systems, NLP. Good overall behavioral signals.</t>
+          <t>Solid fit: AI Engineer at Microsoft with 5.7 years experience. Recent role: AI Engineer at Microsoft. Matched JD skills: Information Retrieval, PyTorch, Python, NLP. Redrob signals: 94% recruiter response rate; 30-day notice period.</t>
         </is>
       </c>
     </row>
@@ -963,19 +963,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.7556</t>
+          <t>0.7724</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 7.8 years in the field, matching key job requirements like RAG, TensorFlow, Vector Search. Good overall behavioral signals.</t>
+          <t>Solid fit: Senior Data Scientist at Niramai with 7.8 years experience. Recent role: Senior Data Scientist at Niramai. Matched JD skills: RAG, TensorFlow, Vector Search, LLM Fine-tuning. Redrob signals: 48% recruiter response rate; 15-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0083307</t>
+          <t>CAND_0030468</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -985,19 +985,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.752</t>
+          <t>0.7653</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 7.8 years in the field, matching key job requirements like Embeddings, Pinecone, Python, note the longer notice period of 120 days.</t>
+          <t>Solid fit: Senior Applied Scientist at Swiggy with 5.4 years experience. Recent role: Senior Applied Scientist at Swiggy. Matched JD skills: Information Retrieval, TensorFlow, Ranking Systems, Milvus. Redrob signals: 78% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0064326</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1007,12 +1007,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.7494</t>
+          <t>0.7618</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Solid candidate working as Search Engineer with 7.6 years in the field, matching key job requirements like PyTorch, Milvus, RAG. Good overall behavioral signals.</t>
+          <t>Solid fit: AI Engineer at Zoho with 5.8 years experience. Recent role: AI Engineer at Zoho. Matched JD skills: MLOps, NLP, FAISS, LLM Fine-tuning. Redrob signals: 57% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
@@ -1029,19 +1029,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.7421</t>
+          <t>0.7597</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 5.3 YoE, who brings relevant experience in Milvus, Embeddings, Vector Search. Good overall behavioral signals.</t>
+          <t>Solid fit: Senior Data Scientist at Razorpay with 5.3 years experience. Recent role: Senior Data Scientist at Razorpay. Matched JD skills: Milvus, Embeddings, Vector Search. Redrob signals: 66% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0083307</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1051,12 +1051,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.7379</t>
+          <t>0.7566</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Well-qualified Senior Data Scientist showing 6.6 YoE, possessing practical experience in Information Retrieval, Pinecone, Vector Search. Good overall behavioral signals.</t>
+          <t>Solid fit: Search Engineer at CRED with 7.8 years experience. Recent role: Search Engineer at CRED. Matched JD skills: Embeddings, Pinecone, Python, Vector Search. Redrob signals: 70% recruiter response rate; 120-day notice period; open to work. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
@@ -1073,19 +1073,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.7328</t>
+          <t>0.7367</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Strong Recommendation Systems Engineer with 6.0 years of experience, matching key job requirements like FAISS, MLOps, Embeddings. Good overall behavioral signals.</t>
+          <t>Solid fit: Recommendation Systems Engineer at CRED with 6.0 years experience. Recent role: Recommendation Systems Engineer at CRED. Matched JD skills: FAISS, MLOps, Embeddings, Vector Search. Redrob signals: 90% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1095,19 +1095,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.7288</t>
+          <t>0.7328</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (7.7 YoE), possessing practical experience in Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Solid fit: Lead AI Engineer at Sarvam AI with 6.4 years experience. Recent role: Lead AI Engineer at Sarvam AI. Matched JD skills: Python, Ranking Systems, Information Retrieval, NLP. Redrob signals: 86% recruiter response rate; 0-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0032515</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1117,19 +1117,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.7286</t>
+          <t>0.732</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 6.7 years in the field, with matching skills in Embeddings, TensorFlow, Information Retrieval and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Machine Learning Engineer at PharmEasy with 5.1 years experience. Recent role: Machine Learning Engineer at PharmEasy. Matched JD skills: Milvus, Vector Search, LLM Fine-tuning, NLP. Redrob signals: 54% recruiter response rate; 45-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0032515</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1139,19 +1139,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.727</t>
+          <t>0.7299</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Strong Machine Learning Engineer with 5.1 years of experience, who brings relevant experience in Milvus, Vector Search, NLP. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Machine Learning Engineer at Genpact AI with 7.2 years experience. Recent role: Machine Learning Engineer at Genpact AI. Matched JD skills: RAG, FAISS, Embeddings, PyTorch. Redrob signals: 60% recruiter response rate; 120-day notice period; open to work. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1161,19 +1161,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.7221</t>
+          <t>0.7281</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Solid candidate working as Machine Learning Engineer with 7.2 years in the field, matching key job requirements like RAG, FAISS, Embeddings, note the longer notice period of 120 days.</t>
+          <t>Qualified but not ideal: AI Engineer at Microsoft with 6.9 years experience. Recent role: AI Engineer at Microsoft. Matched JD skills: Python, Vector Search. Redrob signals: 81% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0049896</t>
+          <t>CAND_0093763</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1183,19 +1183,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.7215</t>
+          <t>0.7275</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (7.3 YoE), with matching skills in PyTorch, Information Retrieval, NLP and solid backend fundamentals, note the longer notice period of 90 days.</t>
+          <t>Qualified but not ideal: Senior Software Engineer (ML) at Swiggy with 5.0 years experience. Recent role: Senior Software Engineer (ML) at Swiggy. Matched JD skills: FAISS, Vector Search, PyTorch, TensorFlow. Redrob signals: 92% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0052682</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.7213</t>
+          <t>0.7249</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 6.9 years in the field, matching key job requirements like Python, Vector Search. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: NLP Engineer at Aganitha with 6.6 years experience. Recent role: NLP Engineer at Aganitha. Matched JD skills: FAISS, PyTorch, Python, Embeddings. Redrob signals: 88% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0024620</t>
+          <t>CAND_0098454</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1227,19 +1227,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.7176</t>
+          <t>0.7245</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (5.9 YoE), possessing practical experience in Information Retrieval, Python. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: AI Specialist at Meesho with 6.6 years experience. Recent role: AI Specialist at Meesho. Matched JD skills: Vector Search, MLOps, NLP, Pinecone. Redrob signals: 87% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0052682</t>
+          <t>CAND_0024620</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.7165</t>
+          <t>0.724</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Strong NLP Engineer with 6.6 years of experience, who brings relevant experience in FAISS, PyTorch, Python. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: AI Engineer at PharmEasy with 5.9 years experience. Recent role: AI Engineer at PharmEasy. Matched JD skills: Information Retrieval, Python. Redrob signals: 41% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0070525</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1271,19 +1271,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.7123</t>
+          <t>0.7208</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Strong Senior Software Engineer (ML) with 5.4 years of experience, who brings relevant experience in Python, Embeddings. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Senior Data Scientist at Google with 6.5 years experience. Recent role: Senior Data Scientist at Google. Matched JD skills: Milvus, TensorFlow, Python. Redrob signals: 72% recruiter response rate; 120-day notice period; open to work. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0010685</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1293,19 +1293,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.7084</t>
+          <t>0.719</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Solid candidate working as NLP Engineer with 6.7 years in the field, with matching skills in PyTorch, Information Retrieval, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: AI Engineer at Google with 7.3 years experience. Recent role: AI Engineer at Google. Matched JD skills: Pinecone, Vector Search, RAG, Information Retrieval. Redrob signals: 78% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
+          <t>CAND_0059795</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1315,19 +1315,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.7071</t>
+          <t>0.7183</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 5.8 years in the field, matching key job requirements like MLOps, NLP, FAISS. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Senior Software Engineer (ML) at Locobuzz with 5.6 years experience. Recent role: Senior Software Engineer (ML) at Locobuzz. Matched JD skills: Python. Redrob signals: 75% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1337,19 +1337,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.7069</t>
+          <t>0.7174</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Solid candidate working as AI Engineer with 7.3 years in the field, matching key job requirements like Pinecone, Vector Search, RAG. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Senior Data Scientist at Flipkart with 6.6 years experience. Recent role: Senior Data Scientist at Flipkart. Matched JD skills: Information Retrieval, Pinecone, Vector Search, NLP. Redrob signals: 56% recruiter response rate; 60-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0030468</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1359,19 +1359,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.7037</t>
+          <t>0.7135</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Applied Scientist with 5.4 years in the field, matching key job requirements like TensorFlow, Ranking Systems, Milvus. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: AI Engineer at PolicyBazaar with 7.7 years experience. Recent role: AI Engineer at PolicyBazaar. Matched JD skills: Vector Search, NLP, LLM Fine-tuning. Redrob signals: 60% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0064326</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1381,19 +1381,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.7003</t>
+          <t>0.7127</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Data Scientist with 6.5 years in the field, matching key job requirements like Milvus, TensorFlow, Python, note the longer notice period of 120 days.</t>
+          <t>Qualified but not ideal: Search Engineer at Sarvam AI with 7.6 years experience. Recent role: Search Engineer at Sarvam AI. Matched JD skills: PyTorch, Milvus, RAG, Python. Redrob signals: 94% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0081686</t>
+          <t>CAND_0010685</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1403,19 +1403,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>0.7112</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Competent Search Engineer (6.0 YoE), matching key job requirements like Embeddings, FAISS, Milvus. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: NLP Engineer at Rephrase.ai with 6.7 years experience. Recent role: NLP Engineer at Rephrase.ai. Matched JD skills: PyTorch, Information Retrieval, RAG. Redrob signals: 83% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0012837</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1425,19 +1425,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.6997</t>
+          <t>0.7101</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Solid candidate working as Staff Machine Learning Engineer with 8.8 years in the field, matching key job requirements like MLOps, Python, Milvus. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Junior ML Engineer at Sarvam AI with 6.4 years experience. Recent role: Junior ML Engineer at Sarvam AI. Matched JD skills: Vector Search, MLOps, NLP. Redrob signals: 81% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0096172</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1447,19 +1447,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.6963</t>
+          <t>0.7085</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Solid candidate working as NLP Engineer with 5.2 years in the field, with matching skills in Python, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: AI Engineer at Rephrase.ai with 6.8 years experience. Recent role: AI Engineer at Rephrase.ai. Matched JD skills: PyTorch, LLM Fine-tuning, FAISS, NLP. Redrob signals: 77% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0058412</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.6949</t>
+          <t>0.7065</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Software Engineer (ML) with 6.6 years in the field, with matching skills in Embeddings, Milvus, RAG and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Senior Machine Learning Engineer at Niramai with 7.9 years experience. Recent role: Senior Machine Learning Engineer at Niramai. Matched JD skills: Ranking Systems, TensorFlow, Information Retrieval. Redrob signals: 61% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0025882</t>
+          <t>CAND_0077285</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1491,19 +1491,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.6942</t>
+          <t>0.7049</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Solid candidate working as Senior Software Engineer (ML) with 5.6 years in the field, with matching skills in FAISS, Vector Search, Milvus and solid backend fundamentals. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Recommendation Systems Engineer at Nykaa with 5.5 years experience. Recent role: Recommendation Systems Engineer at Nykaa. Matched JD skills: Pinecone, Embeddings, Information Retrieval, LLM Fine-tuning. Redrob signals: 56% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.6939</t>
+          <t>0.7031</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Competent AI Engineer (6.8 YoE), matching key job requirements like PyTorch, FAISS, NLP. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Senior Applied Scientist at Niramai with 9.0 years experience. Recent role: Senior Applied Scientist at Niramai. Matched JD skills: PyTorch, NLP, Information Retrieval. Redrob signals: 63% recruiter response rate; 0-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0077285</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1535,19 +1535,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.6911</t>
+          <t>0.7022</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Competent Recommendation Systems Engineer (5.5 YoE), matching key job requirements like Pinecone, Embeddings, Information Retrieval. Good overall behavioral signals.</t>
+          <t>Qualified but not ideal: Applied ML Engineer at Saarthi.ai with 5.8 years experience. Recent role: Applied ML Engineer at Saarthi.ai. Matched JD skills: Vector Search, Milvus, Embeddings, PyTorch. Redrob signals: 72% recruiter response rate; 30-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1557,19 +1557,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.6896</t>
+          <t>0.701</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Applied ML Engineer, mostly showing adjacent skills like Vector Search, Milvus, Embeddings; moderate fit with some technical gaps for this senior role.</t>
+          <t>Qualified but not ideal: Staff Machine Learning Engineer at Salesforce with 8.8 years experience. Recent role: Staff Machine Learning Engineer at Salesforce. Matched JD skills: MLOps, Information Retrieval, Python, Milvus. Redrob signals: 66% recruiter response rate; 0-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0043860</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1579,19 +1579,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.6888</t>
+          <t>0.7002</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.1 YoE as Junior ML Engineer, mostly showing adjacent skills like Information Retrieval, PyTorch, Vector Search; moderate fit with some technical gaps for this senior role.</t>
+          <t>Qualified but not ideal: AI Engineer at Vedantu with 6.7 years experience. Recent role: AI Engineer at Vedantu. Matched JD skills: Embeddings, TensorFlow, Information Retrieval, Milvus. Redrob signals: 74% recruiter response rate; 15-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1601,19 +1601,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.6848</t>
+          <t>0.6942</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Candidate with 7.2 years experience as Search Engineer, mostly showing adjacent skills like Embeddings, Information Retrieval, PyTorch; moderate fit with some technical gaps for this senior role.</t>
+          <t>Qualified but not ideal: Recommendation Systems Engineer at upGrad with 5.8 years experience. Recent role: Recommendation Systems Engineer at upGrad. Matched JD skills: FAISS, Vector Search, Milvus, Pinecone. Redrob signals: 75% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1623,19 +1623,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.6825</t>
+          <t>0.6933</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.2 years of background, with limited direct exposure to search/ranking but lists NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Qualified but not ideal: Search Engineer at Google with 7.2 years experience. Recent role: Search Engineer at Google. Matched JD skills: Embeddings, Information Retrieval, PyTorch, NLP. Redrob signals: 56% recruiter response rate; 120-day notice period; open to work. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0029367</t>
+          <t>CAND_0012632</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1645,19 +1645,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.6815</t>
+          <t>0.6914</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Data Scientist, mostly showing adjacent skills like TensorFlow, FAISS, RAG; included as potential pipeline filler.</t>
+          <t>Qualified but not ideal: AI Specialist at Razorpay with 6.0 years experience. Recent role: AI Specialist at Razorpay. Matched JD skills: MLOps, Python, Pinecone, Vector Search. Redrob signals: 53% recruiter response rate; 120-day notice period. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0098454</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1667,12 +1667,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.681</t>
+          <t>0.6912</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Candidate with 6.6 years experience as AI Specialist, possessing partial overlap in Vector Search, MLOps, NLP; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Qualified but not ideal: Senior Data Scientist at Microsoft with 7.0 years experience. Recent role: Senior Data Scientist at Microsoft. Matched JD skills: MLOps, Milvus, RAG, Information Retrieval. Redrob signals: 49% recruiter response rate; 90-day notice period. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.6807</t>
+          <t>0.6897</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Recommendation Systems Engineer (7.9 YoE), having some background in Python, Embeddings but less specialized; included as potential pipeline filler.</t>
+          <t>Qualified but not ideal: Recommendation Systems Engineer at Wysa with 7.9 years experience. Recent role: Recommendation Systems Engineer at Wysa. Matched JD skills: Python, Embeddings. Redrob signals: 62% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1711,19 +1711,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.6801</t>
+          <t>0.6895</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Candidate with 5.8 years experience as Recommendation Systems Engineer, mostly showing adjacent skills like FAISS, Vector Search, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Qualified but not ideal: Senior Data Scientist at Sarvam AI with 7.4 years experience. Recent role: Senior Data Scientist at Sarvam AI. Matched JD skills: TensorFlow, LLM Fine-tuning, RAG, Information Retrieval. Redrob signals: 56% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0012837</t>
+          <t>CAND_0000031</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1733,19 +1733,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.6793</t>
+          <t>0.6876</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.4 YoE as Junior ML Engineer, mostly showing adjacent skills like Vector Search, MLOps, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Qualified but not ideal: Recommendation Systems Engineer at Swiggy with 6.0 years experience. Recent role: Recommendation Systems Engineer at Swiggy. Matched JD skills: FAISS, Pinecone, MLOps, Embeddings. Redrob signals: 91% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0049896</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1755,19 +1755,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.679</t>
+          <t>0.6858</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.2 YoE), having some background in FAISS, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Qualified but not ideal: Search Engineer at Unacademy with 7.3 years experience. Recent role: Search Engineer at Unacademy. Matched JD skills: PyTorch, Information Retrieval, LLM Fine-tuning, NLP. Redrob signals: 43% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0099401</t>
+          <t>CAND_0007567</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1777,19 +1777,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.6777</t>
+          <t>0.6849</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.7 YoE), having some background in Embeddings, Information Retrieval, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: AI Specialist at Niramai with 6.1 years experience. Recent role: AI Specialist at Niramai. Matched JD skills: LLM Fine-tuning, NLP, MLOps, FAISS. Redrob signals: 80% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0081686</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1799,19 +1799,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.675</t>
+          <t>0.6831</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Alternative profile showing 9.0 YoE as Senior Applied Scientist, mostly showing adjacent skills like PyTorch, NLP; included as potential pipeline filler.</t>
+          <t>Marginal fit: Search Engineer at Netflix with 6.0 years experience. Recent role: Search Engineer at Netflix. Matched JD skills: Embeddings, FAISS, Milvus, Python. Redrob signals: 91% recruiter response rate; 60-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0061265</t>
+          <t>CAND_0041402</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1821,19 +1821,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.6748</t>
+          <t>0.6798</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Vector Search, Embeddings, Milvus; included as potential pipeline filler.</t>
+          <t>Marginal fit: AI Specialist at Ola with 6.3 years experience. Recent role: AI Specialist at Ola. Matched JD skills: Information Retrieval, RAG, Vector Search. Redrob signals: 44% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0006557</t>
+          <t>CAND_0017960</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1843,19 +1843,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.6714</t>
+          <t>0.6794</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (7.9 YoE), having some background in Vector Search, FAISS, Pinecone but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Recommendation Systems Engineer at Nykaa with 7.7 years experience. Recent role: Recommendation Systems Engineer at Nykaa. Matched JD skills: Python, Information Retrieval. Redrob signals: 72% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0027801</t>
+          <t>CAND_0095619</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1865,19 +1865,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.6712</t>
+          <t>0.6792</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Candidate with 7.4 years experience as NLP Engineer, mostly showing adjacent skills like FAISS, Milvus, TensorFlow; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Marginal fit: NLP Engineer at Nykaa with 15.6 years experience. Recent role: NLP Engineer at Nykaa. Matched JD skills: Pinecone, NLP, Information Retrieval, LLM Fine-tuning. Redrob signals: 90% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0000031</t>
+          <t>CAND_0027801</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1887,19 +1887,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.6703</t>
+          <t>0.6788</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 6.0 years of background, possessing partial overlap in FAISS, Pinecone, MLOps; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: NLP Engineer at InMobi with 7.4 years experience. Recent role: NLP Engineer at InMobi. Matched JD skills: FAISS, Milvus, TensorFlow, MLOps. Redrob signals: 65% recruiter response rate; 120-day notice period; open to work. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.6693</t>
+          <t>0.6752</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 7.4 years of background, having some background in TensorFlow, RAG, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Staff Machine Learning Engineer at LinkedIn with 8.0 years experience. Recent role: Staff Machine Learning Engineer at LinkedIn. Matched JD skills: Information Retrieval, Python. Redrob signals: 87% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0041402</t>
+          <t>CAND_0065195</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1931,19 +1931,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.6666</t>
+          <t>0.6748</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Candidate with 6.3 years experience as AI Specialist, mostly showing adjacent skills like Information Retrieval, RAG, Vector Search; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Search Engineer at CRED with 5.1 years experience. Recent role: Search Engineer at CRED. Matched JD skills: MLOps. Redrob signals: 80% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0006557</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1953,19 +1953,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.665</t>
+          <t>0.6738</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.0 YoE as Senior Data Scientist, mostly showing adjacent skills like MLOps, Milvus, RAG; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: NLP Engineer at Paytm with 7.9 years experience. Recent role: NLP Engineer at Paytm. Matched JD skills: Vector Search, FAISS, Pinecone, Information Retrieval. Redrob signals: 63% recruiter response rate; 120-day notice period; open to work. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0017960</t>
+          <t>CAND_0036121</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1975,19 +1975,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.6646</t>
+          <t>0.6728</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Recommendation Systems Engineer (7.7 YoE), having some background in Python, Information Retrieval but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: ML Engineer at Wysa with 5.2 years experience. Recent role: ML Engineer at Wysa. Matched JD skills: Embeddings, Vector Search, Information Retrieval. Redrob signals: 49% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0064256</t>
+          <t>CAND_0070202</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1997,19 +1997,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.6623</t>
+          <t>0.6728</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Junior ML Engineer (6.4 YoE), having some background in PyTorch, MLOps, Python but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Machine Learning Engineer at BYJU'S with 5.1 years experience. Recent role: Machine Learning Engineer at BYJU'S. Matched JD skills: Embeddings, LLM Fine-tuning, PyTorch, RAG. Redrob signals: 60% recruiter response rate; 90-day notice period. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0070202</t>
+          <t>CAND_0064256</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2019,19 +2019,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.6615</t>
+          <t>0.6714</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Candidate with 5.1 years experience as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, PyTorch, RAG; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Junior ML Engineer at BYJU'S with 6.4 years experience. Recent role: Junior ML Engineer at BYJU'S. Matched JD skills: PyTorch, MLOps, Python, Embeddings. Redrob signals: 86% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0015967</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2041,19 +2041,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.6561</t>
+          <t>0.6711</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Candidate with 6.9 years experience as Senior Software Engineer (ML), with limited direct exposure to search/ranking but lists NLP, Embeddings, Milvus; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: Senior Software Engineer (ML) at Razorpay with 5.4 years experience. Recent role: Senior Software Engineer (ML) at Razorpay. Matched JD skills: Pinecone, TensorFlow, Embeddings. Redrob signals: 45% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0051630</t>
+          <t>CAND_0092568</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2063,19 +2063,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.6558</t>
+          <t>0.6702</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.0 YoE as Machine Learning Engineer, mostly showing adjacent skills like Embeddings, Python, NLP; included as potential pipeline filler.</t>
+          <t>Marginal fit: AI Specialist at TCS with 5.7 years experience. Recent role: AI Specialist at TCS. Matched JD skills: Vector Search, Milvus, Python, Pinecone. Redrob signals: 39% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0095619</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2085,19 +2085,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.654</t>
+          <t>0.669</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Candidate with 15.6 years experience as NLP Engineer, possessing partial overlap in Pinecone, NLP, Information Retrieval; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Marginal fit: Senior Data Scientist at Rephrase.ai with 5.7 years experience. Recent role: Senior Data Scientist at Rephrase.ai. Matched JD skills: TensorFlow, FAISS, RAG, NLP. Redrob signals: 77% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0087006</t>
+          <t>CAND_0077498</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.6531</t>
+          <t>0.6688</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Alternative profile showing 5.7 YoE as Senior Software Engineer (ML), mostly showing adjacent skills like Information Retrieval, RAG, NLP; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: Senior Software Engineer (ML) at Niramai with 5.4 years experience. Recent role: Senior Software Engineer (ML) at Niramai. Matched JD skills: Embeddings, Milvus. Redrob signals: 89% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0030953</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.6512</t>
+          <t>0.6669</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.8 YoE as Search Engineer, possessing partial overlap in MLOps, Python, RAG; included as potential pipeline filler.</t>
+          <t>Marginal fit: Applied ML Engineer at Freshworks with 5.2 years experience. Recent role: Applied ML Engineer at Freshworks. Matched JD skills: FAISS, Vector Search, LLM Fine-tuning, NLP. Redrob signals: 52% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0073883</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2151,19 +2151,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.6473</t>
+          <t>0.6649</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.5 YoE as Senior Data Scientist, possessing partial overlap in PyTorch, NLP, RAG; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Marginal fit: AI Specialist at Krutrim with 5.3 years experience. Recent role: AI Specialist at Krutrim. Matched JD skills: Vector Search, Python, FAISS. Redrob signals: 92% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0065195</t>
+          <t>CAND_0030953</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2173,19 +2173,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.6423</t>
+          <t>0.6613</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Search Engineer with 5.1 years of background, with limited direct exposure to search/ranking but lists MLOps; included as potential pipeline filler.</t>
+          <t>Marginal fit: Search Engineer at Nykaa with 7.8 years experience. Recent role: Search Engineer at Nykaa. Matched JD skills: MLOps, Python, RAG. Redrob signals: 63% recruiter response rate; 45-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0018722</t>
+          <t>CAND_0067866</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2195,19 +2195,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.6418</t>
+          <t>0.6597</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.6 YoE as Recommendation Systems Engineer, possessing partial overlap in Python, TensorFlow; included as potential pipeline filler.</t>
+          <t>Marginal fit: Senior Software Engineer (ML) at Tech Mahindra with 6.4 years experience. Recent role: Senior Software Engineer (ML) at Tech Mahindra. Matched JD skills: Embeddings. Redrob signals: 79% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
+          <t>CAND_0076163</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2217,19 +2217,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.6404</t>
+          <t>0.6547</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 8.0 years of background, having some background in Vector Search, TensorFlow, Embeddings but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: NLP Engineer at Ola with 6.9 years experience. Recent role: NLP Engineer at Ola. Matched JD skills: PyTorch, Python, MLOps. Redrob signals: 84% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0076163</t>
+          <t>CAND_0006418</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2239,19 +2239,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.6381</t>
+          <t>0.6528</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (6.9 YoE), having some background in PyTorch, Python, MLOps but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Machine Learning Engineer at Verloop.io with 5.7 years experience. Recent role: Machine Learning Engineer at Verloop.io. Matched JD skills: Embeddings, TensorFlow. Redrob signals: 92% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2261,19 +2261,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.6362</t>
+          <t>0.651</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (5.0 YoE), mostly showing adjacent skills like Pinecone, Python, RAG; included as potential pipeline filler.</t>
+          <t>Marginal fit: Applied ML Engineer at Freshworks with 8.0 years experience. Recent role: Applied ML Engineer at Freshworks. Matched JD skills: Vector Search, TensorFlow, Embeddings, Pinecone. Redrob signals: 42% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0053591</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2283,19 +2283,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.6354</t>
+          <t>0.6475</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Alternative profile showing 8.0 YoE as Staff Machine Learning Engineer, mostly showing adjacent skills like Python; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: AI Engineer at Ola with 5.3 years experience. Recent role: AI Engineer at Ola. Matched JD skills: Embeddings, Milvus, RAG. Redrob signals: 81% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0067866</t>
+          <t>CAND_0074735</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2305,19 +2305,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.6342</t>
+          <t>0.646</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.4 years of background, possessing partial overlap in Embeddings; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Applied ML Engineer at Rephrase.ai with 5.5 years experience. Recent role: Applied ML Engineer at Rephrase.ai. Matched JD skills: RAG, Information Retrieval, Vector Search, TensorFlow. Redrob signals: 77% recruiter response rate; 90-day notice period; open to work. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2327,19 +2327,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.6339</t>
+          <t>0.6446</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Applied ML Engineer (6.6 YoE), having some background in Milvus, Embeddings, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Marginal fit: Recommendation Systems Engineer at CRED with 8.0 years experience. Recent role: Recommendation Systems Engineer at CRED. Matched JD skills: FAISS, Milvus, MLOps, Information Retrieval. Redrob signals: 77% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0049978</t>
+          <t>CAND_0082086</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.6296</t>
+          <t>0.6426</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.6 years of background, with limited direct exposure to search/ranking but lists PyTorch, Embeddings; would require substantial ramp-up time for retrieval systems.</t>
+          <t>Marginal fit: Senior Software Engineer (ML) at Razorpay with 6.0 years experience. Recent role: Senior Software Engineer (ML) at Razorpay. Matched JD skills: FAISS, Pinecone, PyTorch, Milvus. Redrob signals: 85% recruiter response rate; 45-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0024466</t>
+          <t>CAND_0049978</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2371,19 +2371,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.6289</t>
+          <t>0.6422</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as Search Engineer (5.2 YoE), mostly showing adjacent skills like MLOps, NLP, Pinecone; included as potential pipeline filler.</t>
+          <t>Marginal fit: Senior Software Engineer (ML) at Sarvam AI with 6.6 years experience. Recent role: Senior Software Engineer (ML) at Sarvam AI. Matched JD skills: PyTorch, Embeddings. Redrob signals: 71% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0074735</t>
+          <t>CAND_0073314</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2393,19 +2393,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.6287</t>
+          <t>0.6415</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 5.5 years of background, with limited direct exposure to search/ranking but lists RAG, Information Retrieval, Vector Search; included as potential pipeline filler.</t>
+          <t>Marginal fit: Senior Software Engineer (ML) at Aganitha with 5.2 years experience. Recent role: Senior Software Engineer (ML) at Aganitha. Matched JD skills: Milvus, PyTorch, MLOps. Redrob signals: 84% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0044883</t>
+          <t>CAND_0024466</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2415,19 +2415,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.626</t>
+          <t>0.641</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.3 YoE as AI Engineer, mostly showing adjacent skills like Embeddings, TensorFlow, PyTorch; included as potential pipeline filler.</t>
+          <t>Marginal fit: Search Engineer at PharmEasy with 5.2 years experience. Recent role: Search Engineer at PharmEasy. Matched JD skills: MLOps, LLM Fine-tuning, NLP, Pinecone. Redrob signals: 47% recruiter response rate; 120-day notice period; open to work. Concerns: long notice (120 days).</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0040117</t>
+          <t>CAND_0033842</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2437,19 +2437,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.6231</t>
+          <t>0.641</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Candidate with 6.5 years experience as Recommendation Systems Engineer, with limited direct exposure to search/ranking but lists Embeddings, RAG, FAISS; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: Senior Software Engineer (ML) at Rephrase.ai with 5.8 years experience. Recent role: Senior Software Engineer (ML) at Rephrase.ai. Matched JD skills: MLOps, NLP, Pinecone. Redrob signals: 34% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
+          <t>CAND_0024878</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2459,19 +2459,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.6213</t>
+          <t>0.6409</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 8.0 years of background, with limited direct exposure to search/ranking but lists FAISS, Milvus, MLOps; included as potential pipeline filler.</t>
+          <t>Marginal fit: AI Specialist at HCL with 5.7 years experience. Recent role: AI Specialist at HCL. Matched JD skills: NLP, MLOps, Information Retrieval. Redrob signals: 84% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0049771</t>
+          <t>CAND_0070514</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2481,19 +2481,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.6192</t>
+          <t>0.6399</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), with limited direct exposure to search/ranking but lists Python, PyTorch, MLOps; included as potential pipeline filler.</t>
+          <t>Marginal fit: AI Specialist at Glance with 5.5 years experience. Recent role: AI Specialist at Glance. Matched JD skills: Pinecone, Python, MLOps, FAISS. Redrob signals: 80% recruiter response rate; 60-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0093331</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2503,19 +2503,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.6147</t>
+          <t>0.639</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as NLP Engineer (16.1 YoE), having some background in PyTorch, Embeddings, Milvus but less specialized; included as potential pipeline filler.</t>
+          <t>Marginal fit: Senior Data Scientist at Flipkart with 6.5 years experience. Recent role: Senior Data Scientist at Flipkart. Matched JD skills: PyTorch, NLP, RAG, Embeddings. Redrob signals: 67% recruiter response rate; 45-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0082086</t>
+          <t>CAND_0072660</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2525,19 +2525,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.6145</t>
+          <t>0.6384</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.0 years of background, having some background in FAISS, Pinecone, PyTorch but less specialized; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Machine Learning Engineer at Unacademy with 7.1 years experience. Recent role: Machine Learning Engineer at Unacademy. Matched JD skills: PyTorch, Information Retrieval, FAISS, Python. Redrob signals: 53% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0078508</t>
+          <t>CAND_0016657</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2547,19 +2547,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.6134</t>
+          <t>0.6355</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.2 YoE), with limited direct exposure to search/ranking but lists Embeddings, NLP; included as potential pipeline filler.</t>
+          <t>Marginal fit: AI Research Engineer at PhonePe with 5.3 years experience. Recent role: AI Research Engineer at PhonePe. Matched JD skills: PyTorch, MLOps, TensorFlow, Vector Search. Redrob signals: 52% recruiter response rate; 60-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0072660</t>
+          <t>CAND_0010770</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.6133</t>
+          <t>0.6347</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Alternative profile showing 7.1 YoE as Machine Learning Engineer, mostly showing adjacent skills like PyTorch, Information Retrieval, FAISS; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: Recommendation Systems Engineer at Aganitha with 15.2 years experience. Recent role: Recommendation Systems Engineer at Aganitha. Matched JD skills: TensorFlow, MLOps. Redrob signals: 73% recruiter response rate; 30-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0050707</t>
+          <t>CAND_0044883</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2591,19 +2591,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.6129</t>
+          <t>0.6342</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Specialist (5.3 YoE), having some background in RAG, Vector Search, NLP but less specialized; included as potential pipeline filler.</t>
+          <t>Marginal fit: AI Engineer at Mad Street Den with 6.3 years experience. Recent role: AI Engineer at Mad Street Den. Matched JD skills: Embeddings, LLM Fine-tuning, TensorFlow, PyTorch. Redrob signals: 84% recruiter response rate; 90-day notice period. Concerns: long notice (90 days).</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0093883</t>
+          <t>CAND_0040117</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2613,19 +2613,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.6121</t>
+          <t>0.6335</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Adjacent candidate working as AI Research Engineer (5.0 YoE), possessing partial overlap in Embeddings, MLOps, Milvus; lower title relevance to the specific AI/ML requirements.</t>
+          <t>Marginal fit: Recommendation Systems Engineer at PhonePe with 6.5 years experience. Recent role: Recommendation Systems Engineer at PhonePe. Matched JD skills: Embeddings, RAG, FAISS. Redrob signals: 66% recruiter response rate; 15-day notice period; open to work.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0007567</t>
+          <t>CAND_0078508</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2635,12 +2635,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.6118</t>
+          <t>0.6334</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Alternative profile showing 6.1 YoE as AI Specialist, possessing partial overlap in NLP, MLOps, FAISS; moderate fit with some technical gaps for this senior role.</t>
+          <t>Marginal fit: AI Research Engineer at Rephrase.ai with 5.2 years experience. Recent role: AI Research Engineer at Rephrase.ai. Matched JD skills: Embeddings, NLP, LLM Fine-tuning. Redrob signals: 34% recruiter response rate; 30-day notice period.</t>
         </is>
       </c>
     </row>

</xml_diff>